<commit_message>
Data integrity audit + parser bug fix for split career records in PDFs
Co-authored-by: danieljohnconstantine-a11y <229551202+danieljohnconstantine-a11y@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/track_ensemble_predictions.xlsx
+++ b/outputs/track_ensemble_predictions.xlsx
@@ -69,14 +69,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1260,7 +1259,7 @@
         <v>0.1260721347299472</v>
       </c>
       <c r="CV2" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3">
@@ -1576,7 +1575,7 @@
         <v>0.1625306628053156</v>
       </c>
       <c r="CV3" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -1896,7 +1895,7 @@
         <v>0.1286591613929863</v>
       </c>
       <c r="CV4" s="3" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
@@ -2216,7 +2215,7 @@
         <v>0.1132561476213603</v>
       </c>
       <c r="CV5" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6">
@@ -2536,7 +2535,7 @@
         <v>0.1051605783613476</v>
       </c>
       <c r="CV6" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7">
@@ -2858,7 +2857,7 @@
         <v>0.1652897957764627</v>
       </c>
       <c r="CV7" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -3180,7 +3179,7 @@
         <v>0.09140855787291713</v>
       </c>
       <c r="CV8" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9">
@@ -3502,7 +3501,7 @@
         <v>0.1344385171561472</v>
       </c>
       <c r="CV9" s="3" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10">
@@ -3824,7 +3823,7 @@
         <v>0.07976905941388192</v>
       </c>
       <c r="CV10" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11">
@@ -4146,7 +4145,7 @@
         <v>0.1145875844408943</v>
       </c>
       <c r="CV11" s="1" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12">
@@ -4468,7 +4467,7 @@
         <v>0.09845369382088337</v>
       </c>
       <c r="CV12" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13">
@@ -4489,16 +4488,16 @@
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>14.6</v>
+        <v>14.2</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>10.8</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>13.3</v>
+        <v>14.1</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>14.39999961853027</v>
+        <v>14.69999980926514</v>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
@@ -4613,7 +4612,7 @@
         <v>0.7</v>
       </c>
       <c r="AQ13" s="5" t="n">
-        <v>0.3612167300380228</v>
+        <v>0.2464985994397759</v>
       </c>
       <c r="AR13" s="5" t="n">
         <v>0</v>
@@ -4716,7 +4715,7 @@
         <v>0.95</v>
       </c>
       <c r="BX13" s="5" t="n">
-        <v>1.15</v>
+        <v>1.08</v>
       </c>
       <c r="BY13" s="5" t="n">
         <v>1</v>
@@ -4784,13 +4783,13 @@
         <v>1.12</v>
       </c>
       <c r="CT13" s="5" t="n">
-        <v>131.1227611937934</v>
+        <v>114.750434382638</v>
       </c>
       <c r="CU13" s="5" t="n">
-        <v>0.1418977944854592</v>
+        <v>0.1423060978684225</v>
       </c>
       <c r="CV13" s="5" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
@@ -4811,13 +4810,13 @@
         </is>
       </c>
       <c r="E14" s="1" t="n">
-        <v>12.6</v>
+        <v>14.1</v>
       </c>
       <c r="F14" s="1" t="n">
         <v>9.5</v>
       </c>
       <c r="G14" s="1" t="n">
-        <v>11.4</v>
+        <v>13.3</v>
       </c>
       <c r="H14" s="1" t="n">
         <v>15</v>
@@ -5112,7 +5111,7 @@
         <v>0.1411613306056487</v>
       </c>
       <c r="CV14" s="1" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15">
@@ -5434,7 +5433,7 @@
         <v>0.1652652043871021</v>
       </c>
       <c r="CV15" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
@@ -5455,16 +5454,16 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>10.7</v>
+        <v>8.9</v>
       </c>
       <c r="F16" t="n">
-        <v>6.4</v>
+        <v>5.3</v>
       </c>
       <c r="G16" t="n">
-        <v>7.7</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H16" t="n">
-        <v>8.699999809265137</v>
+        <v>9.899999618530273</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5579,7 +5578,7 @@
         <v>0.7</v>
       </c>
       <c r="AQ16" t="n">
-        <v>1.684210526315789</v>
+        <v>0.2625698324022346</v>
       </c>
       <c r="AR16" t="n">
         <v>0</v>
@@ -5747,16 +5746,16 @@
         <v>1</v>
       </c>
       <c r="CS16" t="n">
-        <v>1.02</v>
+        <v>1.06</v>
       </c>
       <c r="CT16" t="n">
-        <v>64.95807094718577</v>
+        <v>60.91633194905642</v>
       </c>
       <c r="CU16" t="n">
-        <v>0.08247134240859975</v>
+        <v>0.088619378737623</v>
       </c>
       <c r="CV16" t="n">
-        <v>28</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17">
@@ -6078,7 +6077,7 @@
         <v>0.06830316292322795</v>
       </c>
       <c r="CV17" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18">
@@ -6099,13 +6098,13 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>8.699999999999999</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F18" t="n">
         <v>5.5</v>
       </c>
       <c r="G18" t="n">
-        <v>9.6</v>
+        <v>7.7</v>
       </c>
       <c r="H18" t="n">
         <v>8.899999618530273</v>
@@ -6400,7 +6399,7 @@
         <v>0.08191991195115091</v>
       </c>
       <c r="CV18" t="n">
-        <v>39</v>
+        <v>44</v>
       </c>
     </row>
     <row r="19">
@@ -7044,7 +7043,7 @@
         <v>0.1608540970046943</v>
       </c>
       <c r="CV20" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21">
@@ -7368,7 +7367,7 @@
         <v>0.09666427075736089</v>
       </c>
       <c r="CV21" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22">
@@ -7692,7 +7691,7 @@
         <v>0.09706834479120105</v>
       </c>
       <c r="CV22" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23">
@@ -8014,7 +8013,7 @@
         <v>0.1008147403809615</v>
       </c>
       <c r="CV23" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="24">
@@ -8980,7 +8979,7 @@
         <v>0.1135893631962572</v>
       </c>
       <c r="CV26" s="1" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="27">
@@ -9302,7 +9301,7 @@
         <v>0.09825313227729313</v>
       </c>
       <c r="CV27" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="28">
@@ -9624,7 +9623,7 @@
         <v>0.08676000130870118</v>
       </c>
       <c r="CV28" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="29">
@@ -9946,7 +9945,7 @@
         <v>0.109178442445187</v>
       </c>
       <c r="CV29" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="30">
@@ -10268,7 +10267,7 @@
         <v>0.1604039401570834</v>
       </c>
       <c r="CV30" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="31">
@@ -10590,7 +10589,7 @@
         <v>0.1069220686246048</v>
       </c>
       <c r="CV31" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="32">
@@ -10910,7 +10909,7 @@
         <v>0.08241970311172873</v>
       </c>
       <c r="CV32" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="33">
@@ -11232,7 +11231,7 @@
         <v>0.09417600485572684</v>
       </c>
       <c r="CV33" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="34">
@@ -11554,7 +11553,7 @@
         <v>0.1040625603537052</v>
       </c>
       <c r="CV34" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="35">
@@ -11876,7 +11875,7 @@
         <v>0.08603241629849213</v>
       </c>
       <c r="CV35" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="36">
@@ -12198,7 +12197,7 @@
         <v>0.1356388948087271</v>
       </c>
       <c r="CV36" s="3" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="37">
@@ -12520,7 +12519,7 @@
         <v>0.1147786069773509</v>
       </c>
       <c r="CV37" s="1" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="38">
@@ -12842,7 +12841,7 @@
         <v>0.02</v>
       </c>
       <c r="CV38" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="39">
@@ -13166,7 +13165,7 @@
         <v>0.1660563254512836</v>
       </c>
       <c r="CV39" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40">
@@ -13490,7 +13489,7 @@
         <v>0.1322455171729895</v>
       </c>
       <c r="CV40" s="3" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="41">
@@ -13814,7 +13813,7 @@
         <v>0.1076272725488008</v>
       </c>
       <c r="CV41" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="42">
@@ -14138,7 +14137,7 @@
         <v>0.1296742341846661</v>
       </c>
       <c r="CV42" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="43">
@@ -14462,7 +14461,7 @@
         <v>0.07347743790301546</v>
       </c>
       <c r="CV43" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="44">
@@ -14786,7 +14785,7 @@
         <v>0.09639037166595606</v>
       </c>
       <c r="CV44" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="45">
@@ -15110,327 +15109,329 @@
         <v>0.07583603002769503</v>
       </c>
       <c r="CV45" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="inlineStr">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t>Angle Park</t>
         </is>
       </c>
-      <c r="B46" s="6" t="n">
+      <c r="B46" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="C46" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D46" s="6" t="inlineStr">
+      <c r="C46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
         <is>
           <t>Kisauni</t>
         </is>
       </c>
-      <c r="E46" s="6" t="n">
-        <v>10.3</v>
-      </c>
-      <c r="F46" s="6" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="G46" s="6" t="n">
-        <v>10.2</v>
-      </c>
-      <c r="H46" s="6" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="I46" s="6" t="inlineStr">
+      <c r="E46" s="4" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="F46" s="4" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="G46" s="4" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="H46" s="4" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="I46" s="4" t="inlineStr">
         <is>
           <t>13112</t>
         </is>
       </c>
-      <c r="J46" s="6" t="inlineStr">
+      <c r="J46" s="4" t="inlineStr">
         <is>
           <t>Ryan Tugwell</t>
         </is>
       </c>
-      <c r="K46" s="6" t="inlineStr">
+      <c r="K46" s="4" t="inlineStr">
         <is>
           <t>3d</t>
         </is>
       </c>
-      <c r="L46" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M46" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="N46" s="6" t="n">
+      <c r="L46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N46" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="O46" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="P46" s="4" t="n">
+        <v>117</v>
+      </c>
+      <c r="Q46" s="4" t="n">
+        <v>160880</v>
+      </c>
+      <c r="R46" s="4" t="n">
         <v>118</v>
       </c>
-      <c r="O46" s="6" t="n">
+      <c r="S46" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="P46" s="6" t="n">
+      <c r="T46" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="Q46" s="6" t="n">
-        <v>160880</v>
-      </c>
-      <c r="R46" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S46" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T46" s="6" t="inlineStr"/>
-      <c r="U46" s="6" t="inlineStr"/>
-      <c r="V46" s="6" t="inlineStr">
+      <c r="U46" s="4" t="inlineStr"/>
+      <c r="V46" s="4" t="inlineStr">
         <is>
           <t>08:58PM</t>
         </is>
       </c>
-      <c r="W46" s="6" t="n">
+      <c r="W46" s="4" t="n">
         <v>530</v>
       </c>
-      <c r="X46" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y46" s="6" t="n">
+      <c r="X46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y46" s="4" t="n">
         <v>30.24</v>
       </c>
-      <c r="Z46" s="6" t="inlineStr"/>
-      <c r="AA46" s="6" t="n">
+      <c r="Z46" s="4" t="inlineStr"/>
+      <c r="AA46" s="4" t="n">
         <v>5.14</v>
       </c>
-      <c r="AB46" s="6" t="inlineStr">
+      <c r="AB46" s="4" t="inlineStr">
         <is>
           <t>[30.56, 30.24, 30.36]</t>
         </is>
       </c>
-      <c r="AC46" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="AD46" s="6" t="n">
+      <c r="AC46" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD46" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="AE46" s="6" t="inlineStr">
+      <c r="AE46" s="4" t="inlineStr">
         <is>
           <t>Dog</t>
         </is>
       </c>
-      <c r="AF46" s="6" t="inlineStr">
+      <c r="AF46" s="4" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="AG46" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH46" s="6" t="n">
+      <c r="AG46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI46" s="4" t="n">
+        <v>63.0952380952381</v>
+      </c>
+      <c r="AJ46" s="4" t="n">
+        <v>103.1128404669261</v>
+      </c>
+      <c r="AK46" s="4" t="n">
+        <v>0.1319932658214889</v>
+      </c>
+      <c r="AL46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN46" s="4" t="n">
+        <v>0.3162393162393162</v>
+      </c>
+      <c r="AO46" s="4" t="n">
         <v>0.5</v>
       </c>
-      <c r="AI46" s="6" t="n">
-        <v>63.0952380952381</v>
-      </c>
-      <c r="AJ46" s="6" t="n">
-        <v>103.1128404669261</v>
-      </c>
-      <c r="AK46" s="6" t="n">
-        <v>0.1319932658214889</v>
-      </c>
-      <c r="AL46" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM46" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN46" s="6" t="n">
-        <v>8.428571428571429</v>
-      </c>
-      <c r="AO46" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP46" s="6" t="n">
+      <c r="AP46" s="4" t="n">
         <v>0.7</v>
       </c>
-      <c r="AQ46" s="6" t="n">
-        <v>1.684210526315789</v>
-      </c>
-      <c r="AR46" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS46" s="6" t="n">
+      <c r="AQ46" s="4" t="n">
+        <v>0.2625698324022346</v>
+      </c>
+      <c r="AR46" s="4" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="AS46" s="4" t="n">
+        <v>0.3675213675213675</v>
+      </c>
+      <c r="AT46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW46" s="4" t="n">
         <v>0.5</v>
       </c>
-      <c r="AT46" s="6" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="AU46" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AV46" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AW46" s="6" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AX46" s="6" t="n">
+      <c r="AX46" s="4" t="n">
         <v>0.6</v>
       </c>
-      <c r="AY46" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ46" s="6" t="n">
+      <c r="AY46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ46" s="4" t="n">
         <v>0.15</v>
       </c>
-      <c r="BA46" s="6" t="n">
+      <c r="BA46" s="4" t="n">
         <v>0.01699999999999999</v>
       </c>
-      <c r="BB46" s="6" t="n">
+      <c r="BB46" s="4" t="n">
         <v>0.04066666666666666</v>
       </c>
-      <c r="BC46" s="6" t="n">
+      <c r="BC46" s="4" t="n">
         <v>0.08</v>
       </c>
-      <c r="BD46" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE46" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF46" s="6" t="inlineStr">
+      <c r="BD46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF46" s="4" t="inlineStr">
         <is>
           <t>BOX1_SPEED</t>
         </is>
       </c>
-      <c r="BG46" s="6" t="n">
+      <c r="BG46" s="4" t="n">
         <v>36</v>
       </c>
-      <c r="BH46" s="6" t="n">
+      <c r="BH46" s="4" t="n">
         <v>1.05</v>
       </c>
-      <c r="BI46" s="6" t="n">
+      <c r="BI46" s="4" t="n">
         <v>0.02</v>
       </c>
-      <c r="BJ46" s="6" t="n">
+      <c r="BJ46" s="4" t="n">
         <v>1.05</v>
       </c>
-      <c r="BK46" s="6" t="n">
+      <c r="BK46" s="4" t="n">
         <v>17.52645502645503</v>
       </c>
-      <c r="BL46" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="BM46" s="6" t="n">
+      <c r="BL46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM46" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="BN46" s="4" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="BO46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP46" s="4" t="n">
+        <v>0.7906661778027998</v>
+      </c>
+      <c r="BQ46" s="4" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="BR46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BT46" s="4" t="inlineStr">
+        <is>
+          <t>MIDDLE</t>
+        </is>
+      </c>
+      <c r="BU46" s="4" t="n">
         <v>0.85</v>
       </c>
-      <c r="BN46" s="6" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="BO46" s="6" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="BP46" s="6" t="n">
-        <v>0.7906661778027998</v>
-      </c>
-      <c r="BQ46" s="6" t="n">
+      <c r="BV46" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BW46" s="4" t="n">
         <v>0.95</v>
       </c>
-      <c r="BR46" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BS46" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT46" s="6" t="inlineStr">
-        <is>
-          <t>MIDDLE</t>
-        </is>
-      </c>
-      <c r="BU46" s="6" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="BV46" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="BW46" s="6" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="BX46" s="6" t="n">
+      <c r="BX46" s="4" t="n">
         <v>1.15</v>
       </c>
-      <c r="BY46" s="6" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="BZ46" s="6" t="n">
+      <c r="BY46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BZ46" s="4" t="n">
         <v>1.05</v>
       </c>
-      <c r="CA46" s="6" t="inlineStr">
+      <c r="CA46" s="4" t="inlineStr">
         <is>
           <t>SAND</t>
         </is>
       </c>
-      <c r="CB46" s="6" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="CC46" s="6" t="n">
-        <v>8.928571428571429</v>
-      </c>
-      <c r="CD46" s="6" t="n">
+      <c r="CB46" s="4" t="n">
+        <v>0.9898</v>
+      </c>
+      <c r="CC46" s="4" t="n">
+        <v>0.6837606837606838</v>
+      </c>
+      <c r="CD46" s="4" t="n">
         <v>0.5625</v>
       </c>
-      <c r="CE46" s="6" t="n">
+      <c r="CE46" s="4" t="n">
         <v>0.8125</v>
       </c>
-      <c r="CF46" s="6" t="n">
+      <c r="CF46" s="4" t="n">
         <v>32.23672383382358</v>
       </c>
-      <c r="CG46" s="6" t="n">
+      <c r="CG46" s="4" t="n">
         <v>0.160334471830431</v>
       </c>
-      <c r="CH46" s="6" t="n">
+      <c r="CH46" s="4" t="n">
         <v>-0.374518208497209</v>
       </c>
-      <c r="CI46" s="6" t="n">
+      <c r="CI46" s="4" t="n">
         <v>-0.7135928774974345</v>
       </c>
-      <c r="CJ46" s="6" t="n">
+      <c r="CJ46" s="4" t="n">
         <v>0.8</v>
       </c>
-      <c r="CK46" s="6" t="n">
+      <c r="CK46" s="4" t="n">
         <v>0.8</v>
       </c>
-      <c r="CL46" s="6" t="n">
+      <c r="CL46" s="4" t="n">
         <v>0.375</v>
       </c>
-      <c r="CM46" s="6" t="n">
+      <c r="CM46" s="4" t="n">
         <v>1.1</v>
       </c>
-      <c r="CN46" s="6" t="n">
+      <c r="CN46" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="CO46" s="6" t="n">
+      <c r="CO46" s="4" t="n">
         <v>0.005</v>
       </c>
-      <c r="CP46" s="6" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="CQ46" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="CR46" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="CS46" s="6" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="CT46" s="6" t="n">
-        <v>126.0522304592091</v>
-      </c>
-      <c r="CU46" s="6" t="n">
-        <v>0.1028815779114074</v>
-      </c>
-      <c r="CV46" s="6" t="n">
-        <v>31</v>
+      <c r="CP46" s="4" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="CQ46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="CR46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="CS46" s="4" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="CT46" s="4" t="n">
+        <v>65.99763046312871</v>
+      </c>
+      <c r="CU46" s="4" t="n">
+        <v>0.166779231915248</v>
+      </c>
+      <c r="CV46" s="4" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="47">
@@ -15460,7 +15461,7 @@
         <v>7.4</v>
       </c>
       <c r="H47" t="n">
-        <v>8.699999999999999</v>
+        <v>8.9</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
@@ -15752,329 +15753,329 @@
         <v>0.09633270820640256</v>
       </c>
       <c r="CV47" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="inlineStr">
+      <c r="A48" t="inlineStr">
         <is>
           <t>Angle Park</t>
         </is>
       </c>
-      <c r="B48" s="1" t="n">
+      <c r="B48" t="n">
         <v>8</v>
       </c>
-      <c r="C48" s="1" t="n">
+      <c r="C48" t="n">
         <v>3</v>
       </c>
-      <c r="D48" s="1" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>Manifesto</t>
         </is>
       </c>
-      <c r="E48" s="1" t="n">
+      <c r="E48" t="n">
         <v>11</v>
       </c>
-      <c r="F48" s="1" t="n">
+      <c r="F48" t="n">
         <v>8.1</v>
       </c>
-      <c r="G48" s="1" t="n">
+      <c r="G48" t="n">
         <v>10.4</v>
       </c>
-      <c r="H48" s="1" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="I48" s="1" t="inlineStr">
+      <c r="H48" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="I48" t="inlineStr">
         <is>
           <t>36x11</t>
         </is>
       </c>
-      <c r="J48" s="1" t="inlineStr">
+      <c r="J48" t="inlineStr">
         <is>
           <t>Colin Swain</t>
         </is>
       </c>
-      <c r="K48" s="1" t="inlineStr">
+      <c r="K48" t="inlineStr">
         <is>
           <t>2b</t>
         </is>
       </c>
-      <c r="L48" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M48" s="1" t="n">
+      <c r="L48" t="n">
+        <v>0</v>
+      </c>
+      <c r="M48" t="n">
         <v>3</v>
       </c>
-      <c r="N48" s="1" t="n">
+      <c r="N48" t="n">
         <v>13</v>
       </c>
-      <c r="O48" s="1" t="n">
+      <c r="O48" t="n">
         <v>13</v>
       </c>
-      <c r="P48" s="1" t="n">
+      <c r="P48" t="n">
         <v>38</v>
       </c>
-      <c r="Q48" s="1" t="n">
+      <c r="Q48" t="n">
         <v>27585</v>
       </c>
-      <c r="R48" s="1" t="n">
+      <c r="R48" t="n">
         <v>3</v>
       </c>
-      <c r="S48" s="1" t="n">
+      <c r="S48" t="n">
         <v>11</v>
       </c>
-      <c r="T48" s="1" t="n">
+      <c r="T48" t="n">
         <v>11</v>
       </c>
-      <c r="U48" s="1" t="inlineStr"/>
-      <c r="V48" s="1" t="inlineStr">
+      <c r="U48" t="inlineStr"/>
+      <c r="V48" t="inlineStr">
         <is>
           <t>08:58PM</t>
         </is>
       </c>
-      <c r="W48" s="1" t="n">
+      <c r="W48" t="n">
         <v>530</v>
       </c>
-      <c r="X48" s="1" t="n">
+      <c r="X48" t="n">
         <v>-0.5</v>
       </c>
-      <c r="Y48" s="1" t="n">
+      <c r="Y48" t="n">
         <v>30.57</v>
       </c>
-      <c r="Z48" s="1" t="inlineStr"/>
-      <c r="AA48" s="1" t="n">
+      <c r="Z48" t="inlineStr"/>
+      <c r="AA48" t="n">
         <v>3.2</v>
       </c>
-      <c r="AB48" s="1" t="inlineStr">
+      <c r="AB48" t="inlineStr">
         <is>
           <t>[30.57, 30.63]</t>
         </is>
       </c>
-      <c r="AC48" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="AD48" s="1" t="n">
+      <c r="AC48" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD48" t="n">
         <v>2</v>
       </c>
-      <c r="AE48" s="1" t="inlineStr">
+      <c r="AE48" t="inlineStr">
         <is>
           <t>Bitch</t>
         </is>
       </c>
-      <c r="AF48" s="1" t="inlineStr">
+      <c r="AF48" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="AG48" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH48" s="1" t="n">
+      <c r="AG48" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH48" t="n">
         <v>0.9</v>
       </c>
-      <c r="AI48" s="1" t="n">
+      <c r="AI48" t="n">
         <v>62.41413150147203</v>
       </c>
-      <c r="AJ48" s="1" t="n">
+      <c r="AJ48" t="n">
         <v>165.625</v>
       </c>
-      <c r="AK48" s="1" t="n">
+      <c r="AK48" t="n">
         <v>0.02999999999999936</v>
       </c>
-      <c r="AL48" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM48" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN48" s="1" t="n">
+      <c r="AL48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN48" t="n">
         <v>0.3421052631578947</v>
       </c>
-      <c r="AO48" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP48" s="1" t="n">
+      <c r="AO48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP48" t="n">
         <v>0.7</v>
       </c>
-      <c r="AQ48" s="1" t="n">
+      <c r="AQ48" t="n">
         <v>0.1891891891891892</v>
       </c>
-      <c r="AR48" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS48" s="1" t="n">
+      <c r="AR48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS48" t="n">
         <v>0.3421052631578947</v>
       </c>
-      <c r="AT48" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AU48" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AV48" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AW48" s="1" t="n">
+      <c r="AT48" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU48" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV48" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW48" t="n">
         <v>0.5</v>
       </c>
-      <c r="AX48" s="1" t="n">
+      <c r="AX48" t="n">
         <v>0.6</v>
       </c>
-      <c r="AY48" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ48" s="1" t="n">
+      <c r="AY48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ48" t="n">
         <v>-0.03800000000000001</v>
       </c>
-      <c r="BA48" s="1" t="n">
+      <c r="BA48" t="n">
         <v>-0.042</v>
       </c>
-      <c r="BB48" s="1" t="n">
+      <c r="BB48" t="n">
         <v>-0.03966666666666666</v>
       </c>
-      <c r="BC48" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD48" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE48" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF48" s="1" t="inlineStr">
+      <c r="BC48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF48" t="inlineStr">
         <is>
           <t>BOX1_SPEED</t>
         </is>
       </c>
-      <c r="BG48" s="1" t="n">
+      <c r="BG48" t="n">
         <v>24</v>
       </c>
-      <c r="BH48" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI48" s="1" t="n">
+      <c r="BH48" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI48" t="n">
         <v>-0.01</v>
       </c>
-      <c r="BJ48" s="1" t="n">
+      <c r="BJ48" t="n">
         <v>0.8</v>
       </c>
-      <c r="BK48" s="1" t="n">
+      <c r="BK48" t="n">
         <v>17.3372587504089</v>
       </c>
-      <c r="BL48" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="BM48" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN48" s="1" t="n">
+      <c r="BL48" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM48" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN48" t="n">
         <v>1.32</v>
       </c>
-      <c r="BO48" s="1" t="n">
+      <c r="BO48" t="n">
         <v>0.97</v>
       </c>
-      <c r="BP48" s="1" t="n">
+      <c r="BP48" t="n">
         <v>0.3273999636091727</v>
       </c>
-      <c r="BQ48" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="BR48" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="BS48" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT48" s="1" t="inlineStr">
+      <c r="BQ48" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS48" t="n">
+        <v>1</v>
+      </c>
+      <c r="BT48" t="inlineStr">
         <is>
           <t>MIDDLE</t>
         </is>
       </c>
-      <c r="BU48" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="BV48" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="BW48" s="1" t="n">
+      <c r="BU48" t="n">
+        <v>1</v>
+      </c>
+      <c r="BV48" t="b">
+        <v>1</v>
+      </c>
+      <c r="BW48" t="n">
         <v>1.02</v>
       </c>
-      <c r="BX48" s="1" t="n">
+      <c r="BX48" t="n">
         <v>1.03</v>
       </c>
-      <c r="BY48" s="1" t="n">
+      <c r="BY48" t="n">
         <v>0.97</v>
       </c>
-      <c r="BZ48" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="CA48" s="1" t="inlineStr">
+      <c r="BZ48" t="n">
+        <v>1</v>
+      </c>
+      <c r="CA48" t="inlineStr">
         <is>
           <t>SAND</t>
         </is>
       </c>
-      <c r="CB48" s="1" t="n">
+      <c r="CB48" t="n">
         <v>1.0302</v>
       </c>
-      <c r="CC48" s="1" t="n">
+      <c r="CC48" t="n">
         <v>0.6842105263157895</v>
       </c>
-      <c r="CD48" s="1" t="n">
+      <c r="CD48" t="n">
         <v>0.9375</v>
       </c>
-      <c r="CE48" s="1" t="n">
+      <c r="CE48" t="n">
         <v>0.125</v>
       </c>
-      <c r="CF48" s="1" t="n">
+      <c r="CF48" t="n">
         <v>32.23672383382358</v>
       </c>
-      <c r="CG48" s="1" t="n">
+      <c r="CG48" t="n">
         <v>0.160334471830431</v>
       </c>
-      <c r="CH48" s="1" t="n">
+      <c r="CH48" t="n">
         <v>0.8930818818010421</v>
       </c>
-      <c r="CI48" s="1" t="n">
+      <c r="CI48" t="n">
         <v>1.21957016815679</v>
       </c>
-      <c r="CJ48" s="1" t="n">
+      <c r="CJ48" t="n">
         <v>0.8</v>
       </c>
-      <c r="CK48" s="1" t="n">
+      <c r="CK48" t="n">
         <v>0.8</v>
       </c>
-      <c r="CL48" s="1" t="n">
+      <c r="CL48" t="n">
         <v>0.375</v>
       </c>
-      <c r="CM48" s="1" t="n">
+      <c r="CM48" t="n">
         <v>1.1</v>
       </c>
-      <c r="CN48" s="1" t="n">
+      <c r="CN48" t="n">
         <v>8</v>
       </c>
-      <c r="CO48" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="CP48" s="1" t="n">
+      <c r="CO48" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP48" t="n">
         <v>1.32</v>
       </c>
-      <c r="CQ48" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="CR48" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="CS48" s="1" t="n">
+      <c r="CQ48" t="n">
+        <v>1</v>
+      </c>
+      <c r="CR48" t="n">
+        <v>1</v>
+      </c>
+      <c r="CS48" t="n">
         <v>1.06</v>
       </c>
-      <c r="CT48" s="1" t="n">
+      <c r="CT48" t="n">
         <v>66.6130438920828</v>
       </c>
-      <c r="CU48" s="1" t="n">
+      <c r="CU48" t="n">
         <v>0.1103239108481305</v>
       </c>
-      <c r="CV48" s="1" t="n">
-        <v>25</v>
+      <c r="CV48" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="49">
@@ -16104,7 +16105,7 @@
         <v>9.199999999999999</v>
       </c>
       <c r="H49" t="n">
-        <v>13.3</v>
+        <v>12.6</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
@@ -16396,7 +16397,7 @@
         <v>0.1037764009220073</v>
       </c>
       <c r="CV49" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="50">
@@ -16426,7 +16427,7 @@
         <v>8.6</v>
       </c>
       <c r="H50" t="n">
-        <v>12.4</v>
+        <v>11.7</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
@@ -16718,7 +16719,7 @@
         <v>0.1014313255415832</v>
       </c>
       <c r="CV50" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="51">
@@ -16739,16 +16740,16 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>7.2</v>
+        <v>7.8</v>
       </c>
       <c r="F51" t="n">
-        <v>6</v>
+        <v>6.3</v>
       </c>
       <c r="G51" t="n">
-        <v>5.7</v>
+        <v>7.1</v>
       </c>
       <c r="H51" t="n">
-        <v>7.8</v>
+        <v>8</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
@@ -16772,24 +16773,26 @@
         <v>6</v>
       </c>
       <c r="N51" t="n">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="O51" t="n">
-        <v>7</v>
+        <v>41</v>
       </c>
       <c r="P51" t="n">
-        <v>7</v>
+        <v>101</v>
       </c>
       <c r="Q51" t="n">
         <v>48095</v>
       </c>
       <c r="R51" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="S51" t="n">
-        <v>0</v>
-      </c>
-      <c r="T51" t="inlineStr"/>
+        <v>7</v>
+      </c>
+      <c r="T51" t="n">
+        <v>7</v>
+      </c>
       <c r="U51" t="inlineStr"/>
       <c r="V51" t="inlineStr">
         <is>
@@ -16834,7 +16837,7 @@
         <v>1</v>
       </c>
       <c r="AH51" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="AI51" t="n">
         <v>62.99108616705183</v>
@@ -16852,25 +16855,25 @@
         <v>0</v>
       </c>
       <c r="AN51" t="n">
-        <v>4</v>
+        <v>0.2079207920792079</v>
       </c>
       <c r="AO51" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="AP51" t="n">
         <v>0.7</v>
       </c>
       <c r="AQ51" t="n">
-        <v>0.3612167300380228</v>
+        <v>0.2464985994397759</v>
       </c>
       <c r="AR51" t="n">
-        <v>0</v>
+        <v>-0.1</v>
       </c>
       <c r="AS51" t="n">
-        <v>1</v>
+        <v>0.405940594059406</v>
       </c>
       <c r="AT51" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="AU51" t="n">
         <v>1</v>
@@ -16929,19 +16932,19 @@
         <v>1</v>
       </c>
       <c r="BM51" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="BN51" t="n">
-        <v>0.75</v>
+        <v>1.5</v>
       </c>
       <c r="BO51" t="n">
-        <v>0.85</v>
+        <v>1</v>
       </c>
       <c r="BP51" t="n">
         <v>0.4323068302005309</v>
       </c>
       <c r="BQ51" t="n">
-        <v>0.88</v>
+        <v>0.95</v>
       </c>
       <c r="BR51" t="n">
         <v>0</v>
@@ -16955,7 +16958,7 @@
         </is>
       </c>
       <c r="BU51" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="BV51" t="b">
         <v>0</v>
@@ -16964,10 +16967,10 @@
         <v>1</v>
       </c>
       <c r="BX51" t="n">
-        <v>1.15</v>
+        <v>1.08</v>
       </c>
       <c r="BY51" t="n">
-        <v>0.85</v>
+        <v>1</v>
       </c>
       <c r="BZ51" t="n">
         <v>1.05</v>
@@ -16978,10 +16981,10 @@
         </is>
       </c>
       <c r="CB51" t="n">
-        <v>1.01</v>
+        <v>0.9898</v>
       </c>
       <c r="CC51" t="n">
-        <v>5</v>
+        <v>0.6138613861386139</v>
       </c>
       <c r="CD51" t="n">
         <v>0.25</v>
@@ -17020,7 +17023,7 @@
         <v>0</v>
       </c>
       <c r="CP51" t="n">
-        <v>0.75</v>
+        <v>1.5</v>
       </c>
       <c r="CQ51" t="n">
         <v>1</v>
@@ -17032,657 +17035,657 @@
         <v>1.12</v>
       </c>
       <c r="CT51" t="n">
-        <v>74.45335202631934</v>
+        <v>61.35885913685802</v>
       </c>
       <c r="CU51" t="n">
-        <v>0.07230316483482319</v>
+        <v>0.07783416366858009</v>
       </c>
       <c r="CV51" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="A52" s="3" t="inlineStr">
         <is>
           <t>Angle Park</t>
         </is>
       </c>
-      <c r="B52" s="2" t="n">
+      <c r="B52" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="C52" s="2" t="n">
+      <c r="C52" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="D52" s="3" t="inlineStr">
         <is>
           <t>Mallee Beauty</t>
         </is>
       </c>
-      <c r="E52" s="2" t="n">
+      <c r="E52" s="3" t="n">
         <v>13.7</v>
       </c>
-      <c r="F52" s="2" t="n">
+      <c r="F52" s="3" t="n">
         <v>14.6</v>
       </c>
-      <c r="G52" s="2" t="n">
+      <c r="G52" s="3" t="n">
         <v>13.8</v>
       </c>
-      <c r="H52" s="2" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="I52" s="2" t="inlineStr">
+      <c r="H52" s="3" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="I52" s="3" t="inlineStr">
         <is>
           <t>11142</t>
         </is>
       </c>
-      <c r="J52" s="2" t="inlineStr">
+      <c r="J52" s="3" t="inlineStr">
         <is>
           <t>Cameron Butcher</t>
         </is>
       </c>
-      <c r="K52" s="2" t="inlineStr">
+      <c r="K52" s="3" t="inlineStr">
         <is>
           <t>3b</t>
         </is>
       </c>
-      <c r="L52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M52" s="2" t="n">
+      <c r="L52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M52" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="N52" s="2" t="n">
+      <c r="N52" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="O52" s="2" t="n">
+      <c r="O52" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="P52" s="2" t="n">
+      <c r="P52" s="3" t="n">
         <v>47</v>
       </c>
-      <c r="Q52" s="2" t="n">
+      <c r="Q52" s="3" t="n">
         <v>257345</v>
       </c>
-      <c r="R52" s="2" t="n">
+      <c r="R52" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="S52" s="2" t="n">
+      <c r="S52" s="3" t="n">
         <v>42</v>
       </c>
-      <c r="T52" s="2" t="n">
+      <c r="T52" s="3" t="n">
         <v>55</v>
       </c>
-      <c r="U52" s="2" t="inlineStr"/>
-      <c r="V52" s="2" t="inlineStr">
+      <c r="U52" s="3" t="inlineStr"/>
+      <c r="V52" s="3" t="inlineStr">
         <is>
           <t>08:58PM</t>
         </is>
       </c>
-      <c r="W52" s="2" t="n">
+      <c r="W52" s="3" t="n">
         <v>530</v>
       </c>
-      <c r="X52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y52" s="2" t="n">
+      <c r="X52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y52" s="3" t="n">
         <v>30.1</v>
       </c>
-      <c r="Z52" s="2" t="inlineStr"/>
-      <c r="AA52" s="2" t="n">
+      <c r="Z52" s="3" t="inlineStr"/>
+      <c r="AA52" s="3" t="n">
         <v>5.18</v>
       </c>
-      <c r="AB52" s="2" t="inlineStr">
+      <c r="AB52" s="3" t="inlineStr">
         <is>
           <t>[30.39, 30.1, 30.24]</t>
         </is>
       </c>
-      <c r="AC52" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AD52" s="2" t="n">
+      <c r="AC52" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD52" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="AE52" s="2" t="inlineStr">
+      <c r="AE52" s="3" t="inlineStr">
         <is>
           <t>Bitch</t>
         </is>
       </c>
-      <c r="AF52" s="2" t="inlineStr">
+      <c r="AF52" s="3" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="AG52" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH52" s="2" t="n">
+      <c r="AG52" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH52" s="3" t="n">
         <v>0.5</v>
       </c>
-      <c r="AI52" s="2" t="n">
+      <c r="AI52" s="3" t="n">
         <v>63.38870431893688</v>
       </c>
-      <c r="AJ52" s="2" t="n">
+      <c r="AJ52" s="3" t="n">
         <v>102.3166023166023</v>
       </c>
-      <c r="AK52" s="2" t="n">
+      <c r="AK52" s="3" t="n">
         <v>0.1184154644555437</v>
       </c>
-      <c r="AL52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN52" s="2" t="n">
+      <c r="AL52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN52" s="3" t="n">
         <v>0.7021276595744681</v>
       </c>
-      <c r="AO52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP52" s="2" t="n">
+      <c r="AO52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP52" s="3" t="n">
         <v>0.7</v>
       </c>
-      <c r="AQ52" s="2" t="n">
+      <c r="AQ52" s="3" t="n">
         <v>0.3894230769230769</v>
       </c>
-      <c r="AR52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS52" s="2" t="n">
+      <c r="AR52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS52" s="3" t="n">
         <v>0.1276595744680851</v>
       </c>
-      <c r="AT52" s="2" t="n">
+      <c r="AT52" s="3" t="n">
         <v>0.4</v>
       </c>
-      <c r="AU52" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AV52" s="2" t="n">
+      <c r="AU52" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV52" s="3" t="n">
         <v>0.7</v>
       </c>
-      <c r="AW52" s="2" t="n">
+      <c r="AW52" s="3" t="n">
         <v>0.5</v>
       </c>
-      <c r="AX52" s="2" t="n">
+      <c r="AX52" s="3" t="n">
         <v>0.6</v>
       </c>
-      <c r="AY52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ52" s="2" t="n">
+      <c r="AY52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ52" s="3" t="n">
         <v>-0.08400000000000001</v>
       </c>
-      <c r="BA52" s="2" t="n">
+      <c r="BA52" s="3" t="n">
         <v>-0.007999999999999993</v>
       </c>
-      <c r="BB52" s="2" t="n">
+      <c r="BB52" s="3" t="n">
         <v>-0.01366666666666666</v>
       </c>
-      <c r="BC52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE52" s="2" t="n">
+      <c r="BC52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE52" s="3" t="n">
         <v>-0.05</v>
       </c>
-      <c r="BF52" s="2" t="inlineStr">
+      <c r="BF52" s="3" t="inlineStr">
         <is>
           <t>BOX1_SPEED</t>
         </is>
       </c>
-      <c r="BG52" s="2" t="n">
+      <c r="BG52" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="BH52" s="2" t="n">
+      <c r="BH52" s="3" t="n">
         <v>1.05</v>
       </c>
-      <c r="BI52" s="2" t="n">
+      <c r="BI52" s="3" t="n">
         <v>-0.01</v>
       </c>
-      <c r="BJ52" s="2" t="n">
+      <c r="BJ52" s="3" t="n">
         <v>0.85</v>
       </c>
-      <c r="BK52" s="2" t="n">
+      <c r="BK52" s="3" t="n">
         <v>17.60797342192691</v>
       </c>
-      <c r="BL52" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="BM52" s="2" t="n">
+      <c r="BL52" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM52" s="3" t="n">
         <v>0.95</v>
       </c>
-      <c r="BN52" s="2" t="n">
+      <c r="BN52" s="3" t="n">
         <v>0.9</v>
       </c>
-      <c r="BO52" s="2" t="n">
+      <c r="BO52" s="3" t="n">
         <v>0.8</v>
       </c>
-      <c r="BP52" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ52" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="BR52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BS52" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT52" s="2" t="inlineStr">
+      <c r="BP52" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ52" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS52" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BT52" s="3" t="inlineStr">
         <is>
           <t>MIDDLE</t>
         </is>
       </c>
-      <c r="BU52" s="2" t="n">
+      <c r="BU52" s="3" t="n">
         <v>0.92</v>
       </c>
-      <c r="BV52" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BW52" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="BX52" s="2" t="n">
+      <c r="BV52" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="BW52" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BX52" s="3" t="n">
         <v>1.15</v>
       </c>
-      <c r="BY52" s="2" t="n">
+      <c r="BY52" s="3" t="n">
         <v>0.8</v>
       </c>
-      <c r="BZ52" s="2" t="n">
+      <c r="BZ52" s="3" t="n">
         <v>1.05</v>
       </c>
-      <c r="CA52" s="2" t="inlineStr">
+      <c r="CA52" s="3" t="inlineStr">
         <is>
           <t>SAND</t>
         </is>
       </c>
-      <c r="CB52" s="2" t="n">
+      <c r="CB52" s="3" t="n">
         <v>1.01</v>
       </c>
-      <c r="CC52" s="2" t="n">
+      <c r="CC52" s="3" t="n">
         <v>0.8297872340425532</v>
       </c>
-      <c r="CD52" s="2" t="n">
+      <c r="CD52" s="3" t="n">
         <v>0.125</v>
       </c>
-      <c r="CE52" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="CF52" s="2" t="n">
+      <c r="CE52" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="CF52" s="3" t="n">
         <v>32.23672383382358</v>
       </c>
-      <c r="CG52" s="2" t="n">
+      <c r="CG52" s="3" t="n">
         <v>0.160334471830431</v>
       </c>
-      <c r="CH52" s="2" t="n">
+      <c r="CH52" s="3" t="n">
         <v>-0.9122879437752404</v>
       </c>
-      <c r="CI52" s="2" t="n">
+      <c r="CI52" s="3" t="n">
         <v>-0.7382162176482663</v>
       </c>
-      <c r="CJ52" s="2" t="n">
+      <c r="CJ52" s="3" t="n">
         <v>0.8</v>
       </c>
-      <c r="CK52" s="2" t="n">
+      <c r="CK52" s="3" t="n">
         <v>0.8</v>
       </c>
-      <c r="CL52" s="2" t="n">
+      <c r="CL52" s="3" t="n">
         <v>0.375</v>
       </c>
-      <c r="CM52" s="2" t="n">
+      <c r="CM52" s="3" t="n">
         <v>1.1</v>
       </c>
-      <c r="CN52" s="2" t="n">
+      <c r="CN52" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="CO52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="CP52" s="2" t="n">
+      <c r="CO52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP52" s="3" t="n">
         <v>0.9</v>
       </c>
-      <c r="CQ52" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="CR52" s="2" t="n">
+      <c r="CQ52" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="CR52" s="3" t="n">
         <v>1.08</v>
       </c>
-      <c r="CS52" s="2" t="n">
+      <c r="CS52" s="3" t="n">
         <v>1.12</v>
       </c>
-      <c r="CT52" s="2" t="n">
+      <c r="CT52" s="3" t="n">
         <v>52.90070798634049</v>
       </c>
-      <c r="CU52" s="2" t="n">
+      <c r="CU52" s="3" t="n">
         <v>0.136574744971208</v>
       </c>
-      <c r="CV52" s="2" t="n">
-        <v>12</v>
+      <c r="CV52" s="3" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="3" t="inlineStr">
+      <c r="A53" s="1" t="inlineStr">
         <is>
           <t>Angle Park</t>
         </is>
       </c>
-      <c r="B53" s="3" t="n">
+      <c r="B53" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="C53" s="3" t="n">
+      <c r="C53" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="D53" s="3" t="inlineStr">
+      <c r="D53" s="1" t="inlineStr">
         <is>
           <t>Flying Artie</t>
         </is>
       </c>
-      <c r="E53" s="3" t="n">
-        <v>13</v>
-      </c>
-      <c r="F53" s="3" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="G53" s="3" t="n">
-        <v>10.7</v>
-      </c>
-      <c r="H53" s="3" t="n">
-        <v>14.2</v>
-      </c>
-      <c r="I53" s="3" t="inlineStr">
+      <c r="E53" s="1" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="F53" s="1" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="G53" s="1" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="H53" s="1" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="I53" s="1" t="inlineStr">
         <is>
           <t>11241</t>
         </is>
       </c>
-      <c r="J53" s="3" t="inlineStr">
+      <c r="J53" s="1" t="inlineStr">
         <is>
           <t>Robin Harnas</t>
         </is>
       </c>
-      <c r="K53" s="3" t="inlineStr">
+      <c r="K53" s="1" t="inlineStr">
         <is>
           <t>2d</t>
         </is>
       </c>
-      <c r="L53" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M53" s="3" t="n">
+      <c r="L53" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M53" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="N53" s="3" t="n">
+      <c r="N53" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="O53" s="3" t="n">
+      <c r="O53" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="P53" s="3" t="n">
+      <c r="P53" s="1" t="n">
         <v>34</v>
       </c>
-      <c r="Q53" s="3" t="n">
+      <c r="Q53" s="1" t="n">
         <v>56480</v>
       </c>
-      <c r="R53" s="3" t="n">
+      <c r="R53" s="1" t="n">
         <v>19</v>
       </c>
-      <c r="S53" s="3" t="n">
+      <c r="S53" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="T53" s="3" t="n">
+      <c r="T53" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="U53" s="3" t="inlineStr"/>
-      <c r="V53" s="3" t="inlineStr">
+      <c r="U53" s="1" t="inlineStr"/>
+      <c r="V53" s="1" t="inlineStr">
         <is>
           <t>08:58PM</t>
         </is>
       </c>
-      <c r="W53" s="3" t="n">
+      <c r="W53" s="1" t="n">
         <v>530</v>
       </c>
-      <c r="X53" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y53" s="3" t="n">
+      <c r="X53" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y53" s="1" t="n">
         <v>30.24</v>
       </c>
-      <c r="Z53" s="3" t="inlineStr"/>
-      <c r="AA53" s="3" t="n">
+      <c r="Z53" s="1" t="inlineStr"/>
+      <c r="AA53" s="1" t="n">
         <v>5.14</v>
       </c>
-      <c r="AB53" s="3" t="inlineStr">
+      <c r="AB53" s="1" t="inlineStr">
         <is>
           <t>[30.24, 30.52, 30.46]</t>
         </is>
       </c>
-      <c r="AC53" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AD53" s="3" t="n">
+      <c r="AC53" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD53" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="AE53" s="3" t="inlineStr">
+      <c r="AE53" s="1" t="inlineStr">
         <is>
           <t>Dog</t>
         </is>
       </c>
-      <c r="AF53" s="3" t="inlineStr">
+      <c r="AF53" s="1" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="AG53" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH53" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI53" s="3" t="n">
+      <c r="AG53" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH53" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI53" s="1" t="n">
         <v>63.0952380952381</v>
       </c>
-      <c r="AJ53" s="3" t="n">
+      <c r="AJ53" s="1" t="n">
         <v>103.1128404669261</v>
       </c>
-      <c r="AK53" s="3" t="n">
+      <c r="AK53" s="1" t="n">
         <v>0.1203698005684526</v>
       </c>
-      <c r="AL53" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM53" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN53" s="3" t="n">
+      <c r="AL53" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM53" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN53" s="1" t="n">
         <v>0.5882352941176471</v>
       </c>
-      <c r="AO53" s="3" t="n">
+      <c r="AO53" s="1" t="n">
         <v>0.5</v>
       </c>
-      <c r="AP53" s="3" t="n">
+      <c r="AP53" s="1" t="n">
         <v>0.7</v>
       </c>
-      <c r="AQ53" s="3" t="n">
-        <v>0.3612167300380228</v>
-      </c>
-      <c r="AR53" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS53" s="3" t="n">
+      <c r="AQ53" s="1" t="n">
+        <v>0.2464985994397759</v>
+      </c>
+      <c r="AR53" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS53" s="1" t="n">
         <v>0.3529411764705883</v>
       </c>
-      <c r="AT53" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AU53" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AV53" s="3" t="n">
+      <c r="AT53" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU53" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV53" s="1" t="n">
         <v>0.7</v>
       </c>
-      <c r="AW53" s="3" t="n">
+      <c r="AW53" s="1" t="n">
         <v>0.5</v>
       </c>
-      <c r="AX53" s="3" t="n">
+      <c r="AX53" s="1" t="n">
         <v>0.6</v>
       </c>
-      <c r="AY53" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ53" s="3" t="n">
+      <c r="AY53" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ53" s="1" t="n">
         <v>-0.02500000000000001</v>
       </c>
-      <c r="BA53" s="3" t="n">
+      <c r="BA53" s="1" t="n">
         <v>0.01699999999999999</v>
       </c>
-      <c r="BB53" s="3" t="n">
+      <c r="BB53" s="1" t="n">
         <v>0.02366666666666667</v>
       </c>
-      <c r="BC53" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD53" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE53" s="3" t="n">
+      <c r="BC53" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD53" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE53" s="1" t="n">
         <v>-0.05</v>
       </c>
-      <c r="BF53" s="3" t="inlineStr">
+      <c r="BF53" s="1" t="inlineStr">
         <is>
           <t>BOX1_SPEED</t>
         </is>
       </c>
-      <c r="BG53" s="3" t="n">
+      <c r="BG53" s="1" t="n">
         <v>24</v>
       </c>
-      <c r="BH53" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI53" s="3" t="n">
+      <c r="BH53" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI53" s="1" t="n">
         <v>0.01</v>
       </c>
-      <c r="BJ53" s="3" t="n">
+      <c r="BJ53" s="1" t="n">
         <v>1.08</v>
       </c>
-      <c r="BK53" s="3" t="n">
+      <c r="BK53" s="1" t="n">
         <v>17.52645502645503</v>
       </c>
-      <c r="BL53" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="BM53" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN53" s="3" t="n">
+      <c r="BL53" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM53" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN53" s="1" t="n">
         <v>1.5</v>
       </c>
-      <c r="BO53" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="BP53" s="3" t="n">
+      <c r="BO53" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP53" s="1" t="n">
         <v>0.4684782973984828</v>
       </c>
-      <c r="BQ53" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="BR53" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BS53" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT53" s="3" t="inlineStr">
+      <c r="BQ53" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR53" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS53" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BT53" s="1" t="inlineStr">
         <is>
           <t>MIDDLE</t>
         </is>
       </c>
-      <c r="BU53" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="BV53" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="BW53" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="BX53" s="3" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="BY53" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="BZ53" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="CA53" s="3" t="inlineStr">
+      <c r="BU53" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BV53" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="BW53" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BX53" s="1" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="BY53" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BZ53" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="CA53" s="1" t="inlineStr">
         <is>
           <t>SAND</t>
         </is>
       </c>
-      <c r="CB53" s="3" t="n">
+      <c r="CB53" s="1" t="n">
         <v>1.0302</v>
       </c>
-      <c r="CC53" s="3" t="n">
+      <c r="CC53" s="1" t="n">
         <v>0.9411764705882353</v>
       </c>
-      <c r="CD53" s="3" t="n">
+      <c r="CD53" s="1" t="n">
         <v>0.5625</v>
       </c>
-      <c r="CE53" s="3" t="n">
+      <c r="CE53" s="1" t="n">
         <v>0.8125</v>
       </c>
-      <c r="CF53" s="3" t="n">
+      <c r="CF53" s="1" t="n">
         <v>32.23672383382358</v>
       </c>
-      <c r="CG53" s="3" t="n">
+      <c r="CG53" s="1" t="n">
         <v>0.160334471830431</v>
       </c>
-      <c r="CH53" s="3" t="n">
+      <c r="CH53" s="1" t="n">
         <v>-0.374518208497209</v>
       </c>
-      <c r="CI53" s="3" t="n">
+      <c r="CI53" s="1" t="n">
         <v>-0.7135928774974345</v>
       </c>
-      <c r="CJ53" s="3" t="n">
+      <c r="CJ53" s="1" t="n">
         <v>0.8</v>
       </c>
-      <c r="CK53" s="3" t="n">
+      <c r="CK53" s="1" t="n">
         <v>0.8</v>
       </c>
-      <c r="CL53" s="3" t="n">
+      <c r="CL53" s="1" t="n">
         <v>0.375</v>
       </c>
-      <c r="CM53" s="3" t="n">
+      <c r="CM53" s="1" t="n">
         <v>1.1</v>
       </c>
-      <c r="CN53" s="3" t="n">
+      <c r="CN53" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="CO53" s="3" t="n">
+      <c r="CO53" s="1" t="n">
         <v>0.01</v>
       </c>
-      <c r="CP53" s="3" t="n">
+      <c r="CP53" s="1" t="n">
         <v>1.5</v>
       </c>
-      <c r="CQ53" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="CR53" s="3" t="n">
+      <c r="CQ53" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="CR53" s="1" t="n">
         <v>1.08</v>
       </c>
-      <c r="CS53" s="3" t="n">
+      <c r="CS53" s="1" t="n">
         <v>1.12</v>
       </c>
-      <c r="CT53" s="3" t="n">
-        <v>165.3011823480963</v>
-      </c>
-      <c r="CU53" s="3" t="n">
-        <v>0.1300554250792006</v>
-      </c>
-      <c r="CV53" s="3" t="n">
-        <v>18</v>
+      <c r="CT53" s="1" t="n">
+        <v>144.6879256484342</v>
+      </c>
+      <c r="CU53" s="1" t="n">
+        <v>0.1267187448826116</v>
+      </c>
+      <c r="CV53" s="1" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="54">
@@ -18004,7 +18007,7 @@
         <v>0.1393027472124736</v>
       </c>
       <c r="CV54" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="55">
@@ -18326,7 +18329,7 @@
         <v>0.1394559435269302</v>
       </c>
       <c r="CV55" s="3" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="56">
@@ -18648,7 +18651,7 @@
         <v>0.1238933353620053</v>
       </c>
       <c r="CV56" s="1" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="57">
@@ -18675,7 +18678,7 @@
         <v>6.4</v>
       </c>
       <c r="G57" t="n">
-        <v>6</v>
+        <v>5.9</v>
       </c>
       <c r="H57" t="n">
         <v>6.400000095367432</v>
@@ -18793,7 +18796,7 @@
         <v>0.7</v>
       </c>
       <c r="AQ57" t="n">
-        <v>0.3612167300380228</v>
+        <v>0.2464985994397759</v>
       </c>
       <c r="AR57" t="n">
         <v>-0.1</v>
@@ -18896,7 +18899,7 @@
         <v>1</v>
       </c>
       <c r="BX57" t="n">
-        <v>1.15</v>
+        <v>1.08</v>
       </c>
       <c r="BY57" t="n">
         <v>1</v>
@@ -18964,13 +18967,13 @@
         <v>1.12</v>
       </c>
       <c r="CT57" t="n">
-        <v>24.15899382400527</v>
+        <v>22.35830026557508</v>
       </c>
       <c r="CU57" t="n">
-        <v>0.0663479652756825</v>
+        <v>0.06607022728298181</v>
       </c>
       <c r="CV57" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="58">
@@ -18994,13 +18997,13 @@
         <v>8.1</v>
       </c>
       <c r="F58" t="n">
-        <v>7.2</v>
+        <v>6.1</v>
       </c>
       <c r="G58" t="n">
         <v>6.8</v>
       </c>
       <c r="H58" t="n">
-        <v>8.100000381469727</v>
+        <v>7.900000095367432</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
@@ -19115,7 +19118,7 @@
         <v>0.7</v>
       </c>
       <c r="AQ58" t="n">
-        <v>0.3612167300380228</v>
+        <v>0.2464985994397759</v>
       </c>
       <c r="AR58" t="n">
         <v>0</v>
@@ -19218,7 +19221,7 @@
         <v>1.02</v>
       </c>
       <c r="BX58" t="n">
-        <v>1.15</v>
+        <v>1.08</v>
       </c>
       <c r="BY58" t="n">
         <v>1</v>
@@ -19286,13 +19289,13 @@
         <v>1.12</v>
       </c>
       <c r="CT58" t="n">
-        <v>36.28600227228602</v>
+        <v>33.726031598427</v>
       </c>
       <c r="CU58" t="n">
-        <v>0.08013403303370537</v>
+        <v>0.07636074508537904</v>
       </c>
       <c r="CV58" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="59">
@@ -19611,10 +19614,10 @@
         <v>42.04620567322814</v>
       </c>
       <c r="CU59" t="n">
-        <v>0.0869083253214753</v>
+        <v>0.08690832532147527</v>
       </c>
       <c r="CV59" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="60">
@@ -19938,7 +19941,7 @@
         <v>0.1659305258964381</v>
       </c>
       <c r="CV60" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="61">
@@ -19968,7 +19971,7 @@
         <v>13</v>
       </c>
       <c r="H61" s="1" t="n">
-        <v>14.9</v>
+        <v>15.1</v>
       </c>
       <c r="I61" s="1" t="inlineStr">
         <is>
@@ -20262,7 +20265,7 @@
         <v>0.1349597594223109</v>
       </c>
       <c r="CV61" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="62">
@@ -20292,7 +20295,7 @@
         <v>12.8</v>
       </c>
       <c r="H62" t="n">
-        <v>12.4</v>
+        <v>13.1</v>
       </c>
       <c r="I62" t="inlineStr">
         <is>
@@ -20584,7 +20587,7 @@
         <v>0.1328299897872628</v>
       </c>
       <c r="CV62" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="63">
@@ -20605,16 +20608,16 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>11</v>
+        <v>12.1</v>
       </c>
       <c r="F63" t="n">
-        <v>9.199999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G63" t="n">
-        <v>9.800000000000001</v>
+        <v>11.4</v>
       </c>
       <c r="H63" t="n">
-        <v>11.2</v>
+        <v>12.1</v>
       </c>
       <c r="I63" t="inlineStr">
         <is>
@@ -20729,7 +20732,7 @@
         <v>0.7</v>
       </c>
       <c r="AQ63" t="n">
-        <v>0.3612167300380228</v>
+        <v>0.2464985994397759</v>
       </c>
       <c r="AR63" t="n">
         <v>0</v>
@@ -20832,7 +20835,7 @@
         <v>1.02</v>
       </c>
       <c r="BX63" t="n">
-        <v>1.15</v>
+        <v>1.08</v>
       </c>
       <c r="BY63" t="n">
         <v>1</v>
@@ -20900,13 +20903,13 @@
         <v>1.12</v>
       </c>
       <c r="CT63" t="n">
-        <v>43.19735811163048</v>
+        <v>40.14407598592515</v>
       </c>
       <c r="CU63" t="n">
-        <v>0.1104419274167062</v>
+        <v>0.1212132419814804</v>
       </c>
       <c r="CV63" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="64">
@@ -20936,7 +20939,7 @@
         <v>13.2</v>
       </c>
       <c r="H64" s="3" t="n">
-        <v>13.7</v>
+        <v>14.1</v>
       </c>
       <c r="I64" s="3" t="inlineStr">
         <is>
@@ -21228,7 +21231,7 @@
         <v>0.1405261090109344</v>
       </c>
       <c r="CV64" s="3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Full pipeline test: RF/GB/XGB verified, Race 8 100% individual scoring confirmed, audit report generated
Co-authored-by: danieljohnconstantine-a11y <229551202+danieljohnconstantine-a11y@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/track_ensemble_predictions.xlsx
+++ b/outputs/track_ensemble_predictions.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CV64"/>
+  <dimension ref="A1:CW64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -942,6 +942,11 @@
       </c>
       <c r="CV1" t="inlineStr">
         <is>
+          <t>Low_Confidence</t>
+        </is>
+      </c>
+      <c r="CW1" t="inlineStr">
+        <is>
           <t>ML_Rank</t>
         </is>
       </c>
@@ -1258,7 +1263,10 @@
       <c r="CU2" s="1" t="n">
         <v>0.1260721347299472</v>
       </c>
-      <c r="CV2" s="1" t="n">
+      <c r="CV2" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW2" s="1" t="n">
         <v>22</v>
       </c>
     </row>
@@ -1574,7 +1582,10 @@
       <c r="CU3" s="2" t="n">
         <v>0.1625306628053156</v>
       </c>
-      <c r="CV3" s="2" t="n">
+      <c r="CV3" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW3" s="2" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1894,7 +1905,10 @@
       <c r="CU4" s="3" t="n">
         <v>0.1286591613929863</v>
       </c>
-      <c r="CV4" s="3" t="n">
+      <c r="CV4" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW4" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2214,7 +2228,10 @@
       <c r="CU5" t="n">
         <v>0.1132561476213603</v>
       </c>
-      <c r="CV5" t="n">
+      <c r="CV5" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW5" t="n">
         <v>27</v>
       </c>
     </row>
@@ -2534,7 +2551,10 @@
       <c r="CU6" t="n">
         <v>0.1051605783613476</v>
       </c>
-      <c r="CV6" t="n">
+      <c r="CV6" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW6" t="n">
         <v>32</v>
       </c>
     </row>
@@ -2856,7 +2876,10 @@
       <c r="CU7" s="4" t="n">
         <v>0.1652897957764627</v>
       </c>
-      <c r="CV7" s="4" t="n">
+      <c r="CV7" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW7" s="4" t="n">
         <v>4</v>
       </c>
     </row>
@@ -3178,7 +3201,10 @@
       <c r="CU8" t="n">
         <v>0.09140855787291713</v>
       </c>
-      <c r="CV8" t="n">
+      <c r="CV8" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW8" t="n">
         <v>40</v>
       </c>
     </row>
@@ -3498,9 +3524,12 @@
         <v>102.1548547727191</v>
       </c>
       <c r="CU9" s="3" t="n">
-        <v>0.1344385171561472</v>
-      </c>
-      <c r="CV9" s="3" t="n">
+        <v>0.1344385171561473</v>
+      </c>
+      <c r="CV9" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW9" s="3" t="n">
         <v>16</v>
       </c>
     </row>
@@ -3822,7 +3851,10 @@
       <c r="CU10" t="n">
         <v>0.07976905941388192</v>
       </c>
-      <c r="CV10" t="n">
+      <c r="CV10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW10" t="n">
         <v>46</v>
       </c>
     </row>
@@ -4144,7 +4176,10 @@
       <c r="CU11" s="1" t="n">
         <v>0.1145875844408943</v>
       </c>
-      <c r="CV11" s="1" t="n">
+      <c r="CV11" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW11" s="1" t="n">
         <v>25</v>
       </c>
     </row>
@@ -4466,7 +4501,10 @@
       <c r="CU12" t="n">
         <v>0.09845369382088337</v>
       </c>
-      <c r="CV12" t="n">
+      <c r="CV12" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW12" t="n">
         <v>35</v>
       </c>
     </row>
@@ -4788,7 +4826,10 @@
       <c r="CU13" s="5" t="n">
         <v>0.1423060978684225</v>
       </c>
-      <c r="CV13" s="5" t="n">
+      <c r="CV13" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW13" s="5" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5110,7 +5151,10 @@
       <c r="CU14" s="1" t="n">
         <v>0.1411613306056487</v>
       </c>
-      <c r="CV14" s="1" t="n">
+      <c r="CV14" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW14" s="1" t="n">
         <v>11</v>
       </c>
     </row>
@@ -5432,7 +5476,10 @@
       <c r="CU15" s="2" t="n">
         <v>0.1652652043871021</v>
       </c>
-      <c r="CV15" s="2" t="n">
+      <c r="CV15" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW15" s="2" t="n">
         <v>4</v>
       </c>
     </row>
@@ -5754,7 +5801,10 @@
       <c r="CU16" t="n">
         <v>0.088619378737623</v>
       </c>
-      <c r="CV16" t="n">
+      <c r="CV16" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW16" t="n">
         <v>41</v>
       </c>
     </row>
@@ -6076,7 +6126,10 @@
       <c r="CU17" t="n">
         <v>0.06830316292322795</v>
       </c>
-      <c r="CV17" t="n">
+      <c r="CV17" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW17" t="n">
         <v>50</v>
       </c>
     </row>
@@ -6398,7 +6451,10 @@
       <c r="CU18" t="n">
         <v>0.08191991195115091</v>
       </c>
-      <c r="CV18" t="n">
+      <c r="CV18" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW18" t="n">
         <v>44</v>
       </c>
     </row>
@@ -6720,7 +6776,10 @@
       <c r="CU19" s="5" t="n">
         <v>0.1194168146714083</v>
       </c>
-      <c r="CV19" s="5" t="n">
+      <c r="CV19" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW19" s="5" t="n">
         <v>8</v>
       </c>
     </row>
@@ -7042,7 +7101,10 @@
       <c r="CU20" s="2" t="n">
         <v>0.1608540970046943</v>
       </c>
-      <c r="CV20" s="2" t="n">
+      <c r="CV20" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW20" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -7366,7 +7428,10 @@
       <c r="CU21" t="n">
         <v>0.09666427075736089</v>
       </c>
-      <c r="CV21" t="n">
+      <c r="CV21" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW21" t="n">
         <v>27</v>
       </c>
     </row>
@@ -7690,7 +7755,10 @@
       <c r="CU22" t="n">
         <v>0.09706834479120105</v>
       </c>
-      <c r="CV22" t="n">
+      <c r="CV22" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW22" t="n">
         <v>36</v>
       </c>
     </row>
@@ -8012,7 +8080,10 @@
       <c r="CU23" s="1" t="n">
         <v>0.1008147403809615</v>
       </c>
-      <c r="CV23" s="1" t="n">
+      <c r="CV23" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW23" s="1" t="n">
         <v>20</v>
       </c>
     </row>
@@ -8334,7 +8405,10 @@
       <c r="CU24" s="5" t="n">
         <v>0.1430787140775155</v>
       </c>
-      <c r="CV24" s="5" t="n">
+      <c r="CV24" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW24" s="5" t="n">
         <v>9</v>
       </c>
     </row>
@@ -8656,7 +8730,10 @@
       <c r="CU25" s="2" t="n">
         <v>0.18</v>
       </c>
-      <c r="CV25" s="2" t="n">
+      <c r="CV25" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW25" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8978,7 +9055,10 @@
       <c r="CU26" s="1" t="n">
         <v>0.1135893631962572</v>
       </c>
-      <c r="CV26" s="1" t="n">
+      <c r="CV26" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW26" s="1" t="n">
         <v>26</v>
       </c>
     </row>
@@ -9300,7 +9380,10 @@
       <c r="CU27" t="n">
         <v>0.09825313227729313</v>
       </c>
-      <c r="CV27" t="n">
+      <c r="CV27" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW27" t="n">
         <v>35</v>
       </c>
     </row>
@@ -9622,7 +9705,10 @@
       <c r="CU28" t="n">
         <v>0.08676000130870118</v>
       </c>
-      <c r="CV28" t="n">
+      <c r="CV28" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW28" t="n">
         <v>42</v>
       </c>
     </row>
@@ -9944,7 +10030,10 @@
       <c r="CU29" t="n">
         <v>0.109178442445187</v>
       </c>
-      <c r="CV29" t="n">
+      <c r="CV29" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW29" t="n">
         <v>29</v>
       </c>
     </row>
@@ -10266,7 +10355,10 @@
       <c r="CU30" s="4" t="n">
         <v>0.1604039401570834</v>
       </c>
-      <c r="CV30" s="4" t="n">
+      <c r="CV30" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW30" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -10588,7 +10680,10 @@
       <c r="CU31" t="n">
         <v>0.1069220686246048</v>
       </c>
-      <c r="CV31" t="n">
+      <c r="CV31" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW31" t="n">
         <v>31</v>
       </c>
     </row>
@@ -10908,7 +11003,10 @@
       <c r="CU32" t="n">
         <v>0.08241970311172873</v>
       </c>
-      <c r="CV32" t="n">
+      <c r="CV32" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW32" t="n">
         <v>44</v>
       </c>
     </row>
@@ -11230,7 +11328,10 @@
       <c r="CU33" t="n">
         <v>0.09417600485572684</v>
       </c>
-      <c r="CV33" t="n">
+      <c r="CV33" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW33" t="n">
         <v>39</v>
       </c>
     </row>
@@ -11552,7 +11653,10 @@
       <c r="CU34" t="n">
         <v>0.1040625603537052</v>
       </c>
-      <c r="CV34" t="n">
+      <c r="CV34" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW34" t="n">
         <v>33</v>
       </c>
     </row>
@@ -11874,7 +11978,10 @@
       <c r="CU35" t="n">
         <v>0.08603241629849213</v>
       </c>
-      <c r="CV35" t="n">
+      <c r="CV35" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW35" t="n">
         <v>43</v>
       </c>
     </row>
@@ -12196,7 +12303,10 @@
       <c r="CU36" s="3" t="n">
         <v>0.1356388948087271</v>
       </c>
-      <c r="CV36" s="3" t="n">
+      <c r="CV36" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW36" s="3" t="n">
         <v>14</v>
       </c>
     </row>
@@ -12518,7 +12628,10 @@
       <c r="CU37" s="1" t="n">
         <v>0.1147786069773509</v>
       </c>
-      <c r="CV37" s="1" t="n">
+      <c r="CV37" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW37" s="1" t="n">
         <v>25</v>
       </c>
     </row>
@@ -12840,7 +12953,10 @@
       <c r="CU38" t="n">
         <v>0.02</v>
       </c>
-      <c r="CV38" t="n">
+      <c r="CV38" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW38" t="n">
         <v>52</v>
       </c>
     </row>
@@ -13164,7 +13280,10 @@
       <c r="CU39" s="4" t="n">
         <v>0.1660563254512836</v>
       </c>
-      <c r="CV39" s="4" t="n">
+      <c r="CV39" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW39" s="4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -13488,7 +13607,10 @@
       <c r="CU40" s="3" t="n">
         <v>0.1322455171729895</v>
       </c>
-      <c r="CV40" s="3" t="n">
+      <c r="CV40" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW40" s="3" t="n">
         <v>18</v>
       </c>
     </row>
@@ -13812,7 +13934,10 @@
       <c r="CU41" t="n">
         <v>0.1076272725488008</v>
       </c>
-      <c r="CV41" t="n">
+      <c r="CV41" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW41" t="n">
         <v>30</v>
       </c>
     </row>
@@ -14136,7 +14261,10 @@
       <c r="CU42" s="1" t="n">
         <v>0.1296742341846661</v>
       </c>
-      <c r="CV42" s="1" t="n">
+      <c r="CV42" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW42" s="1" t="n">
         <v>19</v>
       </c>
     </row>
@@ -14460,7 +14588,10 @@
       <c r="CU43" t="n">
         <v>0.07347743790301546</v>
       </c>
-      <c r="CV43" t="n">
+      <c r="CV43" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW43" t="n">
         <v>49</v>
       </c>
     </row>
@@ -14782,9 +14913,12 @@
         <v>85.19101234137541</v>
       </c>
       <c r="CU44" t="n">
-        <v>0.09639037166595606</v>
-      </c>
-      <c r="CV44" t="n">
+        <v>0.09639037166595604</v>
+      </c>
+      <c r="CV44" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW44" t="n">
         <v>37</v>
       </c>
     </row>
@@ -15108,7 +15242,10 @@
       <c r="CU45" t="n">
         <v>0.07583603002769503</v>
       </c>
-      <c r="CV45" t="n">
+      <c r="CV45" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW45" t="n">
         <v>48</v>
       </c>
     </row>
@@ -15430,7 +15567,10 @@
       <c r="CU46" s="4" t="n">
         <v>0.166779231915248</v>
       </c>
-      <c r="CV46" s="4" t="n">
+      <c r="CV46" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW46" s="4" t="n">
         <v>2</v>
       </c>
     </row>
@@ -15752,7 +15892,10 @@
       <c r="CU47" t="n">
         <v>0.09633270820640256</v>
       </c>
-      <c r="CV47" t="n">
+      <c r="CV47" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW47" t="n">
         <v>37</v>
       </c>
     </row>
@@ -16074,7 +16217,10 @@
       <c r="CU48" t="n">
         <v>0.1103239108481305</v>
       </c>
-      <c r="CV48" t="n">
+      <c r="CV48" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW48" t="n">
         <v>28</v>
       </c>
     </row>
@@ -16396,7 +16542,10 @@
       <c r="CU49" t="n">
         <v>0.1037764009220073</v>
       </c>
-      <c r="CV49" t="n">
+      <c r="CV49" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW49" t="n">
         <v>33</v>
       </c>
     </row>
@@ -16718,7 +16867,10 @@
       <c r="CU50" t="n">
         <v>0.1014313255415832</v>
       </c>
-      <c r="CV50" t="n">
+      <c r="CV50" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW50" t="n">
         <v>34</v>
       </c>
     </row>
@@ -17040,7 +17192,10 @@
       <c r="CU51" t="n">
         <v>0.07783416366858009</v>
       </c>
-      <c r="CV51" t="n">
+      <c r="CV51" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW51" t="n">
         <v>47</v>
       </c>
     </row>
@@ -17362,7 +17517,10 @@
       <c r="CU52" s="3" t="n">
         <v>0.136574744971208</v>
       </c>
-      <c r="CV52" s="3" t="n">
+      <c r="CV52" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW52" s="3" t="n">
         <v>13</v>
       </c>
     </row>
@@ -17684,7 +17842,10 @@
       <c r="CU53" s="1" t="n">
         <v>0.1267187448826116</v>
       </c>
-      <c r="CV53" s="1" t="n">
+      <c r="CV53" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW53" s="1" t="n">
         <v>21</v>
       </c>
     </row>
@@ -18006,7 +18167,10 @@
       <c r="CU54" s="4" t="n">
         <v>0.1393027472124736</v>
       </c>
-      <c r="CV54" s="4" t="n">
+      <c r="CV54" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW54" s="4" t="n">
         <v>12</v>
       </c>
     </row>
@@ -18328,7 +18492,10 @@
       <c r="CU55" s="3" t="n">
         <v>0.1394559435269302</v>
       </c>
-      <c r="CV55" s="3" t="n">
+      <c r="CV55" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW55" s="3" t="n">
         <v>23</v>
       </c>
     </row>
@@ -18650,7 +18817,10 @@
       <c r="CU56" s="1" t="n">
         <v>0.1238933353620053</v>
       </c>
-      <c r="CV56" s="1" t="n">
+      <c r="CV56" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW56" s="1" t="n">
         <v>28</v>
       </c>
     </row>
@@ -18972,7 +19142,10 @@
       <c r="CU57" t="n">
         <v>0.06607022728298181</v>
       </c>
-      <c r="CV57" t="n">
+      <c r="CV57" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW57" t="n">
         <v>51</v>
       </c>
     </row>
@@ -19294,7 +19467,10 @@
       <c r="CU58" t="n">
         <v>0.07636074508537904</v>
       </c>
-      <c r="CV58" t="n">
+      <c r="CV58" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW58" t="n">
         <v>45</v>
       </c>
     </row>
@@ -19614,9 +19790,12 @@
         <v>42.04620567322814</v>
       </c>
       <c r="CU59" t="n">
-        <v>0.08690832532147527</v>
-      </c>
-      <c r="CV59" t="n">
+        <v>0.0869083253214753</v>
+      </c>
+      <c r="CV59" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW59" t="n">
         <v>38</v>
       </c>
     </row>
@@ -19940,7 +20119,10 @@
       <c r="CU60" s="4" t="n">
         <v>0.1659305258964381</v>
       </c>
-      <c r="CV60" s="4" t="n">
+      <c r="CV60" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW60" s="4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -20264,7 +20446,10 @@
       <c r="CU61" s="1" t="n">
         <v>0.1349597594223109</v>
       </c>
-      <c r="CV61" s="1" t="n">
+      <c r="CV61" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW61" s="1" t="n">
         <v>15</v>
       </c>
     </row>
@@ -20586,7 +20771,10 @@
       <c r="CU62" t="n">
         <v>0.1328299897872628</v>
       </c>
-      <c r="CV62" t="n">
+      <c r="CV62" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW62" t="n">
         <v>17</v>
       </c>
     </row>
@@ -20908,7 +21096,10 @@
       <c r="CU63" t="n">
         <v>0.1212132419814804</v>
       </c>
-      <c r="CV63" t="n">
+      <c r="CV63" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW63" t="n">
         <v>24</v>
       </c>
     </row>
@@ -21230,7 +21421,10 @@
       <c r="CU64" s="3" t="n">
         <v>0.1405261090109344</v>
       </c>
-      <c r="CV64" s="3" t="n">
+      <c r="CV64" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW64" s="3" t="n">
         <v>11</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix varied scores: cross-card normalization replaces rank-based; fix .bat for local PC
Co-authored-by: danieljohnconstantine-a11y <229551202+danieljohnconstantine-a11y@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/track_ensemble_predictions.xlsx
+++ b/outputs/track_ensemble_predictions.xlsx
@@ -971,19 +971,19 @@
         </is>
       </c>
       <c r="E2" s="1" t="n">
-        <v>14</v>
+        <v>13.61</v>
       </c>
       <c r="F2" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>14</v>
+        <v>13.07</v>
       </c>
       <c r="H2" s="1" t="n">
-        <v>18</v>
+        <v>12.92</v>
       </c>
       <c r="I2" s="1" t="n">
-        <v>18</v>
+        <v>10.64</v>
       </c>
       <c r="J2" s="1" t="inlineStr">
         <is>
@@ -1272,7 +1272,7 @@
         <v>34.72964079687296</v>
       </c>
       <c r="CV2" s="1" t="n">
-        <v>0.14</v>
+        <v>0.1361329569776661</v>
       </c>
       <c r="CW2" s="1" t="n">
         <v>2</v>
@@ -1296,19 +1296,19 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>18</v>
+        <v>13.92</v>
       </c>
       <c r="F3" s="2" t="b">
         <v>0</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>14</v>
+        <v>12.92</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>14</v>
+        <v>10.64</v>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
@@ -1595,7 +1595,7 @@
         <v>32.03800807223286</v>
       </c>
       <c r="CV3" s="2" t="n">
-        <v>0.18</v>
+        <v>0.1391732451813974</v>
       </c>
       <c r="CW3" s="2" t="n">
         <v>1</v>
@@ -1619,19 +1619,19 @@
         </is>
       </c>
       <c r="E4" s="3" t="n">
-        <v>10</v>
+        <v>12.82</v>
       </c>
       <c r="F4" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>10</v>
+        <v>10.64</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>10</v>
+        <v>12.92</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>10</v>
+        <v>10.64</v>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
@@ -1920,7 +1920,7 @@
         <v>25.61890479836698</v>
       </c>
       <c r="CV4" s="3" t="n">
-        <v>0.09999999999999999</v>
+        <v>0.1281986298224856</v>
       </c>
       <c r="CW4" s="3" t="n">
         <v>3</v>
@@ -1944,19 +1944,19 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>6</v>
+        <v>12.41</v>
       </c>
       <c r="F5" t="b">
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>6</v>
+        <v>10.28</v>
       </c>
       <c r="H5" t="n">
-        <v>6</v>
+        <v>11.79</v>
       </c>
       <c r="I5" t="n">
-        <v>6</v>
+        <v>10.64</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -2243,7 +2243,7 @@
         <v>22.50741453971432</v>
       </c>
       <c r="CV5" t="n">
-        <v>0.06</v>
+        <v>0.1240807669875728</v>
       </c>
       <c r="CW5" t="n">
         <v>4</v>
@@ -2267,19 +2267,19 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>10.15</v>
       </c>
       <c r="F6" t="b">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>2</v>
+        <v>8.42</v>
       </c>
       <c r="H6" t="n">
-        <v>2</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="I6" t="n">
-        <v>2</v>
+        <v>8.99</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
         <v>21.29686553522198</v>
       </c>
       <c r="CV6" t="n">
-        <v>0.01999999999999999</v>
+        <v>0.1014557131860618</v>
       </c>
       <c r="CW6" t="n">
         <v>5</v>
@@ -2592,19 +2592,19 @@
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>14</v>
+        <v>13.82</v>
       </c>
       <c r="F7" s="4" t="b">
         <v>0</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>14</v>
+        <v>13.7</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>18</v>
+        <v>12.92</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>18</v>
+        <v>10.64</v>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
@@ -2893,7 +2893,7 @@
         <v>69.41178693631963</v>
       </c>
       <c r="CV7" s="4" t="n">
-        <v>0.14</v>
+        <v>0.1381879754279961</v>
       </c>
       <c r="CW7" s="4" t="n">
         <v>2</v>
@@ -2917,19 +2917,19 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>2</v>
+        <v>11.1</v>
       </c>
       <c r="F8" t="b">
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>6</v>
+        <v>7.38</v>
       </c>
       <c r="H8" t="n">
-        <v>2</v>
+        <v>11.65</v>
       </c>
       <c r="I8" t="n">
-        <v>6</v>
+        <v>10.09</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -3218,7 +3218,7 @@
         <v>39.65910723315122</v>
       </c>
       <c r="CV8" t="n">
-        <v>0.01999999999999999</v>
+        <v>0.1109838248173262</v>
       </c>
       <c r="CW8" t="n">
         <v>5</v>
@@ -3242,19 +3242,19 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>6</v>
+        <v>11.42</v>
       </c>
       <c r="F9" t="b">
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>2</v>
+        <v>6.35</v>
       </c>
       <c r="H9" t="n">
-        <v>14</v>
+        <v>12.92</v>
       </c>
       <c r="I9" t="n">
-        <v>14</v>
+        <v>10.64</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -3543,7 +3543,7 @@
         <v>68.98348778379983</v>
       </c>
       <c r="CV9" t="n">
-        <v>0.06</v>
+        <v>0.1141765297258671</v>
       </c>
       <c r="CW9" t="n">
         <v>4</v>
@@ -3567,19 +3567,19 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>18</v>
+        <v>13.91</v>
       </c>
       <c r="F10" s="2" t="b">
         <v>0</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>18</v>
+        <v>13.97</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>10</v>
+        <v>12.92</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>10</v>
+        <v>10.64</v>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
@@ -3868,7 +3868,7 @@
         <v>33.89278521174827</v>
       </c>
       <c r="CV10" s="2" t="n">
-        <v>0.18</v>
+        <v>0.1390661913302826</v>
       </c>
       <c r="CW10" s="2" t="n">
         <v>1</v>
@@ -3892,19 +3892,19 @@
         </is>
       </c>
       <c r="E11" s="3" t="n">
-        <v>10</v>
+        <v>11.56</v>
       </c>
       <c r="F11" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>10</v>
+        <v>7.78</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>6</v>
+        <v>12.92</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>2</v>
+        <v>10.09</v>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
@@ -4191,7 +4191,7 @@
         <v>40.68215311712356</v>
       </c>
       <c r="CV11" s="3" t="n">
-        <v>0.09999999999999999</v>
+        <v>0.1155618596551397</v>
       </c>
       <c r="CW11" s="3" t="n">
         <v>3</v>
@@ -4215,19 +4215,19 @@
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>18</v>
+        <v>12.54</v>
       </c>
       <c r="F12" s="5" t="b">
         <v>0</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>18</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>18</v>
+        <v>12.92</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>18</v>
+        <v>10.64</v>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
@@ -4516,7 +4516,7 @@
         <v>38.13157336798139</v>
       </c>
       <c r="CV12" s="5" t="n">
-        <v>0.18</v>
+        <v>0.1254361572797913</v>
       </c>
       <c r="CW12" s="5" t="n">
         <v>1</v>
@@ -4540,19 +4540,19 @@
         </is>
       </c>
       <c r="E13" s="1" t="n">
-        <v>14</v>
+        <v>12.5</v>
       </c>
       <c r="F13" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G13" s="1" t="n">
-        <v>14</v>
+        <v>9.68</v>
       </c>
       <c r="H13" s="1" t="n">
-        <v>14</v>
+        <v>12.92</v>
       </c>
       <c r="I13" s="1" t="n">
-        <v>14</v>
+        <v>10.64</v>
       </c>
       <c r="J13" s="1" t="inlineStr">
         <is>
@@ -4839,7 +4839,7 @@
         <v>30.45699061463905</v>
       </c>
       <c r="CV13" s="1" t="n">
-        <v>0.14</v>
+        <v>0.1250480299948628</v>
       </c>
       <c r="CW13" s="1" t="n">
         <v>2</v>
@@ -4863,19 +4863,19 @@
         </is>
       </c>
       <c r="E14" s="3" t="n">
-        <v>10</v>
+        <v>10.71</v>
       </c>
       <c r="F14" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>2</v>
+        <v>4.62</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>6</v>
+        <v>12.37</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>10</v>
+        <v>10.64</v>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
@@ -5164,7 +5164,7 @@
         <v>35.49477212531589</v>
       </c>
       <c r="CV14" s="3" t="n">
-        <v>0.09999999999999999</v>
+        <v>0.1071021012249545</v>
       </c>
       <c r="CW14" s="3" t="n">
         <v>3</v>
@@ -5188,19 +5188,19 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>6</v>
+        <v>10.1</v>
       </c>
       <c r="F15" t="b">
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>6</v>
+        <v>5.36</v>
       </c>
       <c r="H15" t="n">
-        <v>10</v>
+        <v>12.92</v>
       </c>
       <c r="I15" t="n">
-        <v>6</v>
+        <v>8.99</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -5489,7 +5489,7 @@
         <v>30.47009428669543</v>
       </c>
       <c r="CV15" t="n">
-        <v>0.06</v>
+        <v>0.1010347407347857</v>
       </c>
       <c r="CW15" t="n">
         <v>4</v>
@@ -5513,19 +5513,19 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>8.960000000000001</v>
       </c>
       <c r="F16" t="b">
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>10</v>
+        <v>6.14</v>
       </c>
       <c r="H16" t="n">
-        <v>2</v>
+        <v>9.09</v>
       </c>
       <c r="I16" t="n">
-        <v>2</v>
+        <v>8.31</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -5814,7 +5814,7 @@
         <v>16.45773528369265</v>
       </c>
       <c r="CV16" t="n">
-        <v>0.01999999999999999</v>
+        <v>0.08960406842680481</v>
       </c>
       <c r="CW16" t="n">
         <v>5</v>
@@ -5838,19 +5838,19 @@
         </is>
       </c>
       <c r="E17" s="6" t="n">
-        <v>5.2</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="F17" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>8.4</v>
+        <v>7.29</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>5.2</v>
+        <v>6.91</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>5.2</v>
+        <v>7.26</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
@@ -6139,7 +6139,7 @@
         <v>46.31123877395689</v>
       </c>
       <c r="CV17" s="6" t="n">
-        <v>0.05199999999999999</v>
+        <v>0.0814378297606214</v>
       </c>
       <c r="CW17" s="6" t="n">
         <v>5</v>
@@ -6163,19 +6163,19 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>18</v>
+        <v>15.87</v>
       </c>
       <c r="F18" s="2" t="b">
         <v>0</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>11.6</v>
+        <v>11.1</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>14.8</v>
+        <v>14.13</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>18</v>
+        <v>14.96</v>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
@@ -6464,7 +6464,7 @@
         <v>64.29480699112658</v>
       </c>
       <c r="CV18" s="2" t="n">
-        <v>0.18</v>
+        <v>0.1586738445185035</v>
       </c>
       <c r="CW18" s="2" t="n">
         <v>1</v>
@@ -6488,19 +6488,19 @@
         </is>
       </c>
       <c r="E19" s="1" t="n">
-        <v>14.8</v>
+        <v>15.32</v>
       </c>
       <c r="F19" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G19" s="1" t="n">
-        <v>18</v>
+        <v>16.12</v>
       </c>
       <c r="H19" s="1" t="n">
-        <v>18</v>
+        <v>15.04</v>
       </c>
       <c r="I19" s="1" t="n">
-        <v>14.8</v>
+        <v>10.92</v>
       </c>
       <c r="J19" s="1" t="inlineStr">
         <is>
@@ -6789,7 +6789,7 @@
         <v>87.27525463894267</v>
       </c>
       <c r="CV19" s="1" t="n">
-        <v>0.148</v>
+        <v>0.1532454146467241</v>
       </c>
       <c r="CW19" s="1" t="n">
         <v>2</v>
@@ -6813,19 +6813,19 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>4.79</v>
       </c>
       <c r="F20" t="b">
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>5.2</v>
+        <v>7.28</v>
       </c>
       <c r="H20" t="n">
-        <v>2</v>
+        <v>4.41</v>
       </c>
       <c r="I20" t="n">
-        <v>2</v>
+        <v>2.75</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -7114,7 +7114,7 @@
         <v>54.01328993905518</v>
       </c>
       <c r="CV20" t="n">
-        <v>0.01999999999999999</v>
+        <v>0.04793159979826155</v>
       </c>
       <c r="CW20" t="n">
         <v>6</v>
@@ -7138,19 +7138,19 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>8.4</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="F21" t="b">
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>2</v>
+        <v>3.48</v>
       </c>
       <c r="H21" t="n">
-        <v>8.4</v>
+        <v>8.69</v>
       </c>
       <c r="I21" t="n">
-        <v>8.4</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -7439,7 +7439,7 @@
         <v>26.46479136458998</v>
       </c>
       <c r="CV21" t="n">
-        <v>0.08399999999999999</v>
+        <v>0.08618933392862109</v>
       </c>
       <c r="CW21" t="n">
         <v>4</v>
@@ -7463,19 +7463,19 @@
         </is>
       </c>
       <c r="E22" s="3" t="n">
-        <v>11.6</v>
+        <v>13.36</v>
       </c>
       <c r="F22" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>14.8</v>
+        <v>13.53</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>11.6</v>
+        <v>13.44</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>11.6</v>
+        <v>9.74</v>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
@@ -7764,7 +7764,7 @@
         <v>53.79607804334986</v>
       </c>
       <c r="CV22" s="3" t="n">
-        <v>0.116</v>
+        <v>0.1335725473012733</v>
       </c>
       <c r="CW22" s="3" t="n">
         <v>3</v>
@@ -7788,19 +7788,19 @@
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>10</v>
+        <v>12.43</v>
       </c>
       <c r="F23" s="7" t="b">
         <v>0</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>10</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>14</v>
+        <v>12.37</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>18</v>
+        <v>10.64</v>
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
@@ -8091,7 +8091,7 @@
         <v>86.57372316731569</v>
       </c>
       <c r="CV23" s="7" t="n">
-        <v>0.09999999999999999</v>
+        <v>0.1242577627519266</v>
       </c>
       <c r="CW23" s="7" t="n">
         <v>3</v>
@@ -8115,19 +8115,19 @@
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>18</v>
+        <v>14.87</v>
       </c>
       <c r="F24" s="2" t="b">
         <v>0</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>14</v>
+        <v>12.92</v>
       </c>
       <c r="H24" s="2" t="n">
         <v>18</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>14</v>
+        <v>10.64</v>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
@@ -8416,7 +8416,7 @@
         <v>71.83467085044155</v>
       </c>
       <c r="CV24" s="2" t="n">
-        <v>0.18</v>
+        <v>0.1487126426164271</v>
       </c>
       <c r="CW24" s="2" t="n">
         <v>1</v>
@@ -8440,19 +8440,19 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>9.33</v>
       </c>
       <c r="F25" t="b">
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>2</v>
+        <v>6.07</v>
       </c>
       <c r="H25" t="n">
-        <v>2</v>
+        <v>5.19</v>
       </c>
       <c r="I25" t="n">
-        <v>10</v>
+        <v>10.64</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
@@ -8741,7 +8741,7 @@
         <v>25.95960081773428</v>
       </c>
       <c r="CV25" t="n">
-        <v>0.01999999999999999</v>
+        <v>0.09333374851245842</v>
       </c>
       <c r="CW25" t="n">
         <v>5</v>
@@ -8765,19 +8765,19 @@
         </is>
       </c>
       <c r="E26" s="1" t="n">
-        <v>14</v>
+        <v>12.96</v>
       </c>
       <c r="F26" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G26" s="1" t="n">
-        <v>18</v>
+        <v>13.85</v>
       </c>
       <c r="H26" s="1" t="n">
-        <v>10</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="I26" s="1" t="n">
-        <v>6</v>
+        <v>10.64</v>
       </c>
       <c r="J26" s="1" t="inlineStr">
         <is>
@@ -9066,7 +9066,7 @@
         <v>34.36805861712836</v>
       </c>
       <c r="CV26" s="1" t="n">
-        <v>0.14</v>
+        <v>0.1295676381994014</v>
       </c>
       <c r="CW26" s="1" t="n">
         <v>2</v>
@@ -9090,19 +9090,19 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>6</v>
+        <v>9.68</v>
       </c>
       <c r="F27" t="b">
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>6</v>
+        <v>6.36</v>
       </c>
       <c r="H27" t="n">
-        <v>6</v>
+        <v>8.73</v>
       </c>
       <c r="I27" t="n">
-        <v>2</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -9391,7 +9391,7 @@
         <v>35.31530196492779</v>
       </c>
       <c r="CV27" t="n">
-        <v>0.06</v>
+        <v>0.0967909051470203</v>
       </c>
       <c r="CW27" t="n">
         <v>4</v>
@@ -9415,19 +9415,19 @@
         </is>
       </c>
       <c r="E28" s="4" t="n">
-        <v>14</v>
+        <v>13.52</v>
       </c>
       <c r="F28" s="4" t="b">
         <v>0</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>14</v>
+        <v>12.8</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>18</v>
+        <v>12.92</v>
       </c>
       <c r="I28" s="4" t="n">
-        <v>18</v>
+        <v>10.64</v>
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
@@ -9716,7 +9716,7 @@
         <v>63.538250004872</v>
       </c>
       <c r="CV28" s="4" t="n">
-        <v>0.14</v>
+        <v>0.1352398210726929</v>
       </c>
       <c r="CW28" s="4" t="n">
         <v>2</v>
@@ -9740,19 +9740,19 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>10.1</v>
       </c>
       <c r="F29" t="b">
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>10</v>
+        <v>12.66</v>
       </c>
       <c r="H29" t="n">
-        <v>2</v>
+        <v>6.86</v>
       </c>
       <c r="I29" t="n">
-        <v>2</v>
+        <v>7.61</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -10041,7 +10041,7 @@
         <v>86.10919368570299</v>
       </c>
       <c r="CV29" t="n">
-        <v>0.01999999999999999</v>
+        <v>0.100978002338154</v>
       </c>
       <c r="CW29" t="n">
         <v>5</v>
@@ -10065,7 +10065,7 @@
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>18</v>
+        <v>15.22</v>
       </c>
       <c r="F30" s="2" t="b">
         <v>0</v>
@@ -10074,10 +10074,10 @@
         <v>18</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>14</v>
+        <v>12.92</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>14</v>
+        <v>10.64</v>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
@@ -10366,7 +10366,7 @@
         <v>45.21805941646117</v>
       </c>
       <c r="CV30" s="2" t="n">
-        <v>0.18</v>
+        <v>0.1522363831589941</v>
       </c>
       <c r="CW30" s="2" t="n">
         <v>1</v>
@@ -10390,19 +10390,19 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>6</v>
+        <v>11.29</v>
       </c>
       <c r="F31" t="b">
         <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>2</v>
+        <v>5.96</v>
       </c>
       <c r="H31" t="n">
-        <v>10</v>
+        <v>12.92</v>
       </c>
       <c r="I31" t="n">
-        <v>10</v>
+        <v>10.64</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
@@ -10691,7 +10691,7 @@
         <v>62.56137227099106</v>
       </c>
       <c r="CV31" t="n">
-        <v>0.06</v>
+        <v>0.1128942503575277</v>
       </c>
       <c r="CW31" t="n">
         <v>4</v>
@@ -10715,19 +10715,19 @@
         </is>
       </c>
       <c r="E32" s="3" t="n">
-        <v>10</v>
+        <v>11.58</v>
       </c>
       <c r="F32" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>6</v>
+        <v>6.84</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>6</v>
+        <v>12.92</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>6</v>
+        <v>10.64</v>
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
@@ -11016,7 +11016,7 @@
         <v>65.68001746010384</v>
       </c>
       <c r="CV32" s="3" t="n">
-        <v>0.09999999999999999</v>
+        <v>0.1157743554894085</v>
       </c>
       <c r="CW32" s="3" t="n">
         <v>3</v>
@@ -11040,19 +11040,19 @@
         </is>
       </c>
       <c r="E33" s="6" t="n">
-        <v>5.2</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="F33" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G33" s="6" t="n">
-        <v>8.4</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>5.2</v>
+        <v>11.65</v>
       </c>
       <c r="I33" s="6" t="n">
-        <v>5.2</v>
+        <v>6.32</v>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
@@ -11343,7 +11343,7 @@
         <v>75.88267668374074</v>
       </c>
       <c r="CV33" s="6" t="n">
-        <v>0.05199999999999999</v>
+        <v>0.09213420295376999</v>
       </c>
       <c r="CW33" s="6" t="n">
         <v>5</v>
@@ -11367,19 +11367,19 @@
         </is>
       </c>
       <c r="E34" s="3" t="n">
-        <v>11.6</v>
+        <v>16.21</v>
       </c>
       <c r="F34" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>14.8</v>
+        <v>13.27</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>18</v>
+        <v>12.92</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>11.6</v>
+        <v>14.87</v>
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
@@ -11668,7 +11668,7 @@
         <v>27.32606853835148</v>
       </c>
       <c r="CV34" s="3" t="n">
-        <v>0.116</v>
+        <v>0.1621073102994076</v>
       </c>
       <c r="CW34" s="3" t="n">
         <v>3</v>
@@ -11692,19 +11692,19 @@
         </is>
       </c>
       <c r="E35" s="1" t="n">
-        <v>14.8</v>
+        <v>17.4</v>
       </c>
       <c r="F35" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G35" s="1" t="n">
-        <v>18</v>
+        <v>13.27</v>
       </c>
       <c r="H35" s="1" t="n">
-        <v>14.8</v>
+        <v>12.92</v>
       </c>
       <c r="I35" s="1" t="n">
-        <v>14.8</v>
+        <v>16.86</v>
       </c>
       <c r="J35" s="1" t="inlineStr">
         <is>
@@ -11993,7 +11993,7 @@
         <v>50.37077242720862</v>
       </c>
       <c r="CV35" s="1" t="n">
-        <v>0.148</v>
+        <v>0.1740401909671463</v>
       </c>
       <c r="CW35" s="1" t="n">
         <v>2</v>
@@ -12017,19 +12017,19 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>8.4</v>
+        <v>9.34</v>
       </c>
       <c r="F36" t="b">
         <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>5.2</v>
+        <v>7.23</v>
       </c>
       <c r="H36" t="n">
-        <v>11.6</v>
+        <v>12.92</v>
       </c>
       <c r="I36" t="n">
-        <v>8.4</v>
+        <v>6.69</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
@@ -12318,7 +12318,7 @@
         <v>29.81788831280647</v>
       </c>
       <c r="CV36" t="n">
-        <v>0.08399999999999999</v>
+        <v>0.09336010903885103</v>
       </c>
       <c r="CW36" t="n">
         <v>4</v>
@@ -12342,19 +12342,19 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F37" t="b">
         <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>2</v>
+        <v>4.22</v>
       </c>
       <c r="H37" t="n">
-        <v>2</v>
+        <v>6.86</v>
       </c>
       <c r="I37" t="n">
-        <v>2</v>
+        <v>2.03</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
@@ -12643,7 +12643,7 @@
         <v>34.74305624093601</v>
       </c>
       <c r="CV37" t="n">
-        <v>0.01999999999999999</v>
+        <v>0.03997400859598693</v>
       </c>
       <c r="CW37" t="n">
         <v>6</v>
@@ -12673,10 +12673,10 @@
         <v>0</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>11.6</v>
+        <v>13</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>8.4</v>
+        <v>12.92</v>
       </c>
       <c r="I38" s="2" t="n">
         <v>18</v>
@@ -12992,19 +12992,19 @@
         </is>
       </c>
       <c r="E39" s="5" t="n">
-        <v>18</v>
+        <v>14.26</v>
       </c>
       <c r="F39" s="5" t="b">
         <v>0</v>
       </c>
       <c r="G39" s="5" t="n">
-        <v>18</v>
+        <v>10.1</v>
       </c>
       <c r="H39" s="5" t="n">
-        <v>11.6</v>
+        <v>12.95</v>
       </c>
       <c r="I39" s="5" t="n">
-        <v>18</v>
+        <v>13.33</v>
       </c>
       <c r="J39" s="5" t="inlineStr">
         <is>
@@ -13293,7 +13293,7 @@
         <v>80.3037485203028</v>
       </c>
       <c r="CV39" s="5" t="n">
-        <v>0.18</v>
+        <v>0.1426139155211921</v>
       </c>
       <c r="CW39" s="5" t="n">
         <v>1</v>
@@ -13317,19 +13317,19 @@
         </is>
       </c>
       <c r="E40" s="3" t="n">
-        <v>11.6</v>
+        <v>12.14</v>
       </c>
       <c r="F40" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>8.4</v>
+        <v>8.51</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>14.8</v>
+        <v>13.79</v>
       </c>
       <c r="I40" s="3" t="n">
-        <v>11.6</v>
+        <v>10.29</v>
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
@@ -13618,7 +13618,7 @@
         <v>56.9581760286313</v>
       </c>
       <c r="CV40" s="3" t="n">
-        <v>0.116</v>
+        <v>0.121358727757675</v>
       </c>
       <c r="CW40" s="3" t="n">
         <v>3</v>
@@ -13642,19 +13642,19 @@
         </is>
       </c>
       <c r="E41" s="1" t="n">
-        <v>14.8</v>
+        <v>12.64</v>
       </c>
       <c r="F41" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G41" s="1" t="n">
-        <v>11.6</v>
+        <v>8.81</v>
       </c>
       <c r="H41" s="1" t="n">
-        <v>18</v>
+        <v>15.78</v>
       </c>
       <c r="I41" s="1" t="n">
-        <v>8.4</v>
+        <v>10.11</v>
       </c>
       <c r="J41" s="1" t="inlineStr">
         <is>
@@ -13943,7 +13943,7 @@
         <v>23.26155299711137</v>
       </c>
       <c r="CV41" s="1" t="n">
-        <v>0.148</v>
+        <v>0.1263513647643288</v>
       </c>
       <c r="CW41" s="1" t="n">
         <v>2</v>
@@ -13967,19 +13967,19 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>2</v>
+        <v>7.13</v>
       </c>
       <c r="F42" t="b">
         <v>0</v>
       </c>
       <c r="G42" t="n">
-        <v>2</v>
+        <v>6.21</v>
       </c>
       <c r="H42" t="n">
-        <v>2</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="I42" t="n">
-        <v>2</v>
+        <v>5.37</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
@@ -14268,7 +14268,7 @@
         <v>38.12510585823195</v>
       </c>
       <c r="CV42" t="n">
-        <v>0.01999999999999999</v>
+        <v>0.07128783173964839</v>
       </c>
       <c r="CW42" t="n">
         <v>6</v>
@@ -14292,19 +14292,19 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>5.2</v>
+        <v>10.88</v>
       </c>
       <c r="F43" t="b">
         <v>0</v>
       </c>
       <c r="G43" t="n">
-        <v>14.8</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="H43" t="n">
-        <v>5.2</v>
+        <v>11.82</v>
       </c>
       <c r="I43" t="n">
-        <v>5.2</v>
+        <v>8.65</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
@@ -14593,7 +14593,7 @@
         <v>82.18611361379365</v>
       </c>
       <c r="CV43" t="n">
-        <v>0.05199999999999999</v>
+        <v>0.1087905199298234</v>
       </c>
       <c r="CW43" t="n">
         <v>5</v>
@@ -14617,19 +14617,19 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>8.4</v>
+        <v>11.42</v>
       </c>
       <c r="F44" t="b">
         <v>0</v>
       </c>
       <c r="G44" t="n">
-        <v>5.2</v>
+        <v>6.21</v>
       </c>
       <c r="H44" t="n">
-        <v>8.4</v>
+        <v>12.68</v>
       </c>
       <c r="I44" t="n">
-        <v>14.8</v>
+        <v>10.82</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
@@ -14918,7 +14918,7 @@
         <v>22.48239439190696</v>
       </c>
       <c r="CV44" t="n">
-        <v>0.08399999999999999</v>
+        <v>0.1141555604731149</v>
       </c>
       <c r="CW44" t="n">
         <v>4</v>
@@ -14942,19 +14942,19 @@
         </is>
       </c>
       <c r="E45" s="5" t="n">
-        <v>18</v>
+        <v>8.98</v>
       </c>
       <c r="F45" s="5" t="b">
         <v>0</v>
       </c>
       <c r="G45" s="5" t="n">
-        <v>18</v>
+        <v>8.77</v>
       </c>
       <c r="H45" s="5" t="n">
-        <v>18</v>
+        <v>8.130000000000001</v>
       </c>
       <c r="I45" s="5" t="n">
-        <v>18</v>
+        <v>7.31</v>
       </c>
       <c r="J45" s="5" t="inlineStr">
         <is>
@@ -15243,7 +15243,7 @@
         <v>30.07851398853546</v>
       </c>
       <c r="CV45" s="5" t="n">
-        <v>0.18</v>
+        <v>0.08977856872212464</v>
       </c>
       <c r="CW45" s="5" t="n">
         <v>1</v>
@@ -15267,19 +15267,19 @@
         </is>
       </c>
       <c r="E46" s="1" t="n">
-        <v>14.8</v>
+        <v>5.53</v>
       </c>
       <c r="F46" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G46" s="1" t="n">
-        <v>11.6</v>
+        <v>3.89</v>
       </c>
       <c r="H46" s="1" t="n">
-        <v>5.2</v>
+        <v>5.55</v>
       </c>
       <c r="I46" s="1" t="n">
-        <v>14.8</v>
+        <v>5.33</v>
       </c>
       <c r="J46" s="1" t="inlineStr">
         <is>
@@ -15568,7 +15568,7 @@
         <v>45.6350105748115</v>
       </c>
       <c r="CV46" s="1" t="n">
-        <v>0.148</v>
+        <v>0.05526448237032087</v>
       </c>
       <c r="CW46" s="1" t="n">
         <v>2</v>
@@ -15592,19 +15592,19 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>5.2</v>
+        <v>3.95</v>
       </c>
       <c r="F47" t="b">
         <v>0</v>
       </c>
       <c r="G47" t="n">
-        <v>8.4</v>
+        <v>3.06</v>
       </c>
       <c r="H47" t="n">
-        <v>8.4</v>
+        <v>5.92</v>
       </c>
       <c r="I47" t="n">
-        <v>8.4</v>
+        <v>2.99</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
@@ -15893,7 +15893,7 @@
         <v>36.82384198012345</v>
       </c>
       <c r="CV47" t="n">
-        <v>0.05199999999999999</v>
+        <v>0.03951758648531395</v>
       </c>
       <c r="CW47" t="n">
         <v>5</v>
@@ -16218,7 +16218,7 @@
         <v>20.29090792882856</v>
       </c>
       <c r="CV48" t="n">
-        <v>0.01999999999999999</v>
+        <v>0.02</v>
       </c>
       <c r="CW48" t="n">
         <v>6</v>
@@ -16242,19 +16242,19 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>8.4</v>
+        <v>5.01</v>
       </c>
       <c r="F49" t="b">
         <v>0</v>
       </c>
       <c r="G49" t="n">
-        <v>5.2</v>
+        <v>3.06</v>
       </c>
       <c r="H49" t="n">
-        <v>14.8</v>
+        <v>7.65</v>
       </c>
       <c r="I49" t="n">
-        <v>11.6</v>
+        <v>4.01</v>
       </c>
       <c r="J49" t="inlineStr">
         <is>
@@ -16543,7 +16543,7 @@
         <v>22.87258425791754</v>
       </c>
       <c r="CV49" t="n">
-        <v>0.08399999999999999</v>
+        <v>0.05006908360414854</v>
       </c>
       <c r="CW49" t="n">
         <v>4</v>
@@ -16567,19 +16567,19 @@
         </is>
       </c>
       <c r="E50" s="3" t="n">
-        <v>11.6</v>
+        <v>5.27</v>
       </c>
       <c r="F50" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G50" s="3" t="n">
-        <v>14.8</v>
+        <v>6.88</v>
       </c>
       <c r="H50" s="3" t="n">
-        <v>11.6</v>
+        <v>6.56</v>
       </c>
       <c r="I50" s="3" t="n">
-        <v>5.2</v>
+        <v>2.84</v>
       </c>
       <c r="J50" s="3" t="inlineStr">
         <is>
@@ -16868,7 +16868,7 @@
         <v>43.52254753168122</v>
       </c>
       <c r="CV50" s="3" t="n">
-        <v>0.116</v>
+        <v>0.05274071192659846</v>
       </c>
       <c r="CW50" s="3" t="n">
         <v>3</v>
@@ -16892,19 +16892,19 @@
         </is>
       </c>
       <c r="E51" s="5" t="n">
-        <v>18</v>
+        <v>16.07</v>
       </c>
       <c r="F51" s="5" t="b">
         <v>0</v>
       </c>
       <c r="G51" s="5" t="n">
-        <v>18</v>
+        <v>15.92</v>
       </c>
       <c r="H51" s="5" t="n">
         <v>18</v>
       </c>
       <c r="I51" s="5" t="n">
-        <v>18</v>
+        <v>11.62</v>
       </c>
       <c r="J51" s="5" t="inlineStr">
         <is>
@@ -17191,7 +17191,7 @@
         <v>35.53697669699019</v>
       </c>
       <c r="CV51" s="5" t="n">
-        <v>0.18</v>
+        <v>0.1606895627533124</v>
       </c>
       <c r="CW51" s="5" t="n">
         <v>1</v>
@@ -17215,19 +17215,19 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>8.4</v>
+        <v>11.19</v>
       </c>
       <c r="F52" t="b">
         <v>0</v>
       </c>
       <c r="G52" t="n">
-        <v>8.4</v>
+        <v>9.18</v>
       </c>
       <c r="H52" t="n">
-        <v>11.6</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="I52" t="n">
-        <v>8.4</v>
+        <v>11.29</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
@@ -17514,7 +17514,7 @@
         <v>20.37634261311368</v>
       </c>
       <c r="CV52" t="n">
-        <v>0.08399999999999999</v>
+        <v>0.111875130074499</v>
       </c>
       <c r="CW52" t="n">
         <v>4</v>
@@ -17538,19 +17538,19 @@
         </is>
       </c>
       <c r="E53" s="1" t="n">
-        <v>14.8</v>
+        <v>12.49</v>
       </c>
       <c r="F53" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G53" s="1" t="n">
-        <v>11.6</v>
+        <v>10.28</v>
       </c>
       <c r="H53" s="1" t="n">
-        <v>14.8</v>
+        <v>11.25</v>
       </c>
       <c r="I53" s="1" t="n">
-        <v>14.8</v>
+        <v>11.62</v>
       </c>
       <c r="J53" s="1" t="inlineStr">
         <is>
@@ -17837,7 +17837,7 @@
         <v>26.95190587771532</v>
       </c>
       <c r="CV53" s="1" t="n">
-        <v>0.148</v>
+        <v>0.1249477469668958</v>
       </c>
       <c r="CW53" s="1" t="n">
         <v>2</v>
@@ -17861,19 +17861,19 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>5.2</v>
+        <v>9.51</v>
       </c>
       <c r="F54" t="b">
         <v>0</v>
       </c>
       <c r="G54" t="n">
-        <v>5.2</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="H54" t="n">
-        <v>8.4</v>
+        <v>7.04</v>
       </c>
       <c r="I54" t="n">
-        <v>2</v>
+        <v>9.34</v>
       </c>
       <c r="J54" t="inlineStr">
         <is>
@@ -18160,7 +18160,7 @@
         <v>20.19450366483454</v>
       </c>
       <c r="CV54" t="n">
-        <v>0.05199999999999999</v>
+        <v>0.09512944135130319</v>
       </c>
       <c r="CW54" t="n">
         <v>5</v>
@@ -18184,19 +18184,19 @@
         </is>
       </c>
       <c r="E55" s="3" t="n">
-        <v>11.6</v>
+        <v>11.39</v>
       </c>
       <c r="F55" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G55" s="3" t="n">
-        <v>14.8</v>
+        <v>10.75</v>
       </c>
       <c r="H55" s="3" t="n">
-        <v>5.2</v>
+        <v>6.98</v>
       </c>
       <c r="I55" s="3" t="n">
-        <v>11.6</v>
+        <v>11.43</v>
       </c>
       <c r="J55" s="3" t="inlineStr"/>
       <c r="K55" s="3" t="inlineStr">
@@ -18479,7 +18479,7 @@
         <v>13.2500871363948</v>
       </c>
       <c r="CV55" s="3" t="n">
-        <v>0.116</v>
+        <v>0.1138909381637958</v>
       </c>
       <c r="CW55" s="3" t="n">
         <v>3</v>
@@ -18503,19 +18503,19 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>2</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="F56" t="b">
         <v>0</v>
       </c>
       <c r="G56" t="n">
-        <v>2</v>
+        <v>7.46</v>
       </c>
       <c r="H56" t="n">
-        <v>2</v>
+        <v>3.98</v>
       </c>
       <c r="I56" t="n">
-        <v>5.2</v>
+        <v>11.1</v>
       </c>
       <c r="J56" t="inlineStr">
         <is>
@@ -18802,7 +18802,7 @@
         <v>13.85840582616767</v>
       </c>
       <c r="CV56" t="n">
-        <v>0.01999999999999999</v>
+        <v>0.09366166091721105</v>
       </c>
       <c r="CW56" t="n">
         <v>6</v>
@@ -18826,19 +18826,19 @@
         </is>
       </c>
       <c r="E57" s="6" t="n">
-        <v>4</v>
+        <v>6.57</v>
       </c>
       <c r="F57" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G57" s="6" t="n">
-        <v>4</v>
+        <v>4.56</v>
       </c>
       <c r="H57" s="6" t="n">
-        <v>4</v>
+        <v>4.96</v>
       </c>
       <c r="I57" s="6" t="n">
-        <v>4</v>
+        <v>7.36</v>
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
@@ -19127,7 +19127,7 @@
         <v>26.92168578402094</v>
       </c>
       <c r="CV57" s="6" t="n">
-        <v>0.03999999999999998</v>
+        <v>0.0657328280659851</v>
       </c>
       <c r="CW57" s="6" t="n">
         <v>8</v>
@@ -19151,19 +19151,19 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>12</v>
+        <v>11.31</v>
       </c>
       <c r="F58" t="b">
         <v>0</v>
       </c>
       <c r="G58" t="n">
-        <v>12</v>
+        <v>8.94</v>
       </c>
       <c r="H58" t="n">
-        <v>6</v>
+        <v>9.08</v>
       </c>
       <c r="I58" t="n">
-        <v>8</v>
+        <v>11.29</v>
       </c>
       <c r="J58" t="inlineStr">
         <is>
@@ -19452,7 +19452,7 @@
         <v>22.20750461827885</v>
       </c>
       <c r="CV58" t="n">
-        <v>0.12</v>
+        <v>0.1130515633081382</v>
       </c>
       <c r="CW58" t="n">
         <v>4</v>
@@ -19476,19 +19476,19 @@
         </is>
       </c>
       <c r="E59" s="1" t="n">
-        <v>16</v>
+        <v>13.09</v>
       </c>
       <c r="F59" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G59" s="1" t="n">
-        <v>16</v>
+        <v>13.03</v>
       </c>
       <c r="H59" s="1" t="n">
-        <v>18</v>
+        <v>10.24</v>
       </c>
       <c r="I59" s="1" t="n">
-        <v>18</v>
+        <v>11.62</v>
       </c>
       <c r="J59" s="1" t="inlineStr">
         <is>
@@ -19777,7 +19777,7 @@
         <v>40.76865561318051</v>
       </c>
       <c r="CV59" s="1" t="n">
-        <v>0.16</v>
+        <v>0.130855498145536</v>
       </c>
       <c r="CW59" s="1" t="n">
         <v>2</v>
@@ -19801,19 +19801,19 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>8</v>
+        <v>10.76</v>
       </c>
       <c r="F60" t="b">
         <v>0</v>
       </c>
       <c r="G60" t="n">
-        <v>8</v>
+        <v>5.7</v>
       </c>
       <c r="H60" t="n">
-        <v>16</v>
+        <v>10.24</v>
       </c>
       <c r="I60" t="n">
-        <v>12</v>
+        <v>11.58</v>
       </c>
       <c r="J60" t="inlineStr">
         <is>
@@ -20102,7 +20102,7 @@
         <v>28.48222792320604</v>
       </c>
       <c r="CV60" t="n">
-        <v>0.07999999999999999</v>
+        <v>0.1076366007302374</v>
       </c>
       <c r="CW60" t="n">
         <v>6</v>
@@ -20126,19 +20126,19 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>6</v>
+        <v>10.45</v>
       </c>
       <c r="F61" t="b">
         <v>0</v>
       </c>
       <c r="G61" t="n">
-        <v>6</v>
+        <v>5.22</v>
       </c>
       <c r="H61" t="n">
-        <v>14</v>
+        <v>10.24</v>
       </c>
       <c r="I61" t="n">
-        <v>6</v>
+        <v>11.29</v>
       </c>
       <c r="J61" t="inlineStr">
         <is>
@@ -20427,7 +20427,7 @@
         <v>59.33229979952294</v>
       </c>
       <c r="CV61" t="n">
-        <v>0.06</v>
+        <v>0.104486963036356</v>
       </c>
       <c r="CW61" t="n">
         <v>7</v>
@@ -20451,19 +20451,19 @@
         </is>
       </c>
       <c r="E62" s="3" t="n">
-        <v>14</v>
+        <v>12.4</v>
       </c>
       <c r="F62" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G62" s="3" t="n">
-        <v>14</v>
+        <v>10.84</v>
       </c>
       <c r="H62" s="3" t="n">
-        <v>12</v>
+        <v>10.24</v>
       </c>
       <c r="I62" s="3" t="n">
-        <v>16</v>
+        <v>11.62</v>
       </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
@@ -20752,7 +20752,7 @@
         <v>28.33671922732409</v>
       </c>
       <c r="CV62" s="3" t="n">
-        <v>0.14</v>
+        <v>0.1239950530017397</v>
       </c>
       <c r="CW62" s="3" t="n">
         <v>3</v>
@@ -20776,7 +20776,7 @@
         </is>
       </c>
       <c r="E63" s="2" t="n">
-        <v>18</v>
+        <v>14.64</v>
       </c>
       <c r="F63" s="2" t="b">
         <v>0</v>
@@ -20785,10 +20785,10 @@
         <v>18</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>10</v>
+        <v>10.24</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>14</v>
+        <v>11.62</v>
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
@@ -21077,7 +21077,7 @@
         <v>51.77891737471481</v>
       </c>
       <c r="CV63" s="2" t="n">
-        <v>0.18</v>
+        <v>0.1464450538998176</v>
       </c>
       <c r="CW63" s="2" t="n">
         <v>1</v>
@@ -21101,19 +21101,19 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>10</v>
+        <v>11.07</v>
       </c>
       <c r="F64" t="b">
         <v>0</v>
       </c>
       <c r="G64" t="n">
-        <v>10</v>
+        <v>6.69</v>
       </c>
       <c r="H64" t="n">
-        <v>8</v>
+        <v>10.24</v>
       </c>
       <c r="I64" t="n">
-        <v>10</v>
+        <v>11.58</v>
       </c>
       <c r="J64" t="inlineStr">
         <is>
@@ -21402,7 +21402,7 @@
         <v>27.90654415353914</v>
       </c>
       <c r="CV64" t="n">
-        <v>0.09999999999999999</v>
+        <v>0.110723842664261</v>
       </c>
       <c r="CW64" t="n">
         <v>5</v>
@@ -21432,7 +21432,7 @@
         <v>0</v>
       </c>
       <c r="G65" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="H65" t="n">
         <v>2</v>
@@ -21727,7 +21727,7 @@
         <v>34.47356959119575</v>
       </c>
       <c r="CV65" t="n">
-        <v>0.01999999999999999</v>
+        <v>0.02</v>
       </c>
       <c r="CW65" t="n">
         <v>9</v>
@@ -21751,19 +21751,19 @@
         </is>
       </c>
       <c r="E66" s="6" t="n">
-        <v>2</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="F66" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G66" s="6" t="n">
-        <v>15.71</v>
+        <v>11.16</v>
       </c>
       <c r="H66" s="6" t="n">
-        <v>2</v>
+        <v>5.57</v>
       </c>
       <c r="I66" s="6" t="n">
-        <v>2</v>
+        <v>6.6</v>
       </c>
       <c r="J66" s="6" t="inlineStr">
         <is>
@@ -22052,7 +22052,7 @@
         <v>44.15057677199813</v>
       </c>
       <c r="CV66" s="6" t="n">
-        <v>0.01999999999999999</v>
+        <v>0.08369938500866404</v>
       </c>
       <c r="CW66" s="6" t="n">
         <v>8</v>
@@ -22076,19 +22076,19 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>8.859999999999999</v>
+        <v>11.72</v>
       </c>
       <c r="F67" t="b">
         <v>0</v>
       </c>
       <c r="G67" t="n">
-        <v>6.57</v>
+        <v>8.68</v>
       </c>
       <c r="H67" t="n">
-        <v>18</v>
+        <v>10.24</v>
       </c>
       <c r="I67" t="n">
-        <v>18</v>
+        <v>11.62</v>
       </c>
       <c r="J67" t="inlineStr">
         <is>
@@ -22377,7 +22377,7 @@
         <v>32.98110470944309</v>
       </c>
       <c r="CV67" t="n">
-        <v>0.08857142857142856</v>
+        <v>0.1172208394992819</v>
       </c>
       <c r="CW67" t="n">
         <v>5</v>
@@ -22401,19 +22401,19 @@
         </is>
       </c>
       <c r="E68" s="3" t="n">
-        <v>13.43</v>
+        <v>12.32</v>
       </c>
       <c r="F68" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G68" s="3" t="n">
-        <v>11.14</v>
+        <v>10.58</v>
       </c>
       <c r="H68" s="3" t="n">
-        <v>15.71</v>
+        <v>10.24</v>
       </c>
       <c r="I68" s="3" t="n">
-        <v>15.71</v>
+        <v>11.62</v>
       </c>
       <c r="J68" s="3" t="inlineStr">
         <is>
@@ -22702,7 +22702,7 @@
         <v>21.18032588064538</v>
       </c>
       <c r="CV68" s="3" t="n">
-        <v>0.1342857142857143</v>
+        <v>0.1231718024636708</v>
       </c>
       <c r="CW68" s="3" t="n">
         <v>3</v>
@@ -22726,19 +22726,19 @@
         </is>
       </c>
       <c r="E69" s="1" t="n">
-        <v>15.71</v>
+        <v>12.42</v>
       </c>
       <c r="F69" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G69" s="1" t="n">
-        <v>13.43</v>
+        <v>10.92</v>
       </c>
       <c r="H69" s="1" t="n">
-        <v>13.43</v>
+        <v>10.24</v>
       </c>
       <c r="I69" s="1" t="n">
-        <v>13.43</v>
+        <v>11.62</v>
       </c>
       <c r="J69" s="1" t="inlineStr">
         <is>
@@ -23027,7 +23027,7 @@
         <v>63.12166763346953</v>
       </c>
       <c r="CV69" s="1" t="n">
-        <v>0.1571428571428571</v>
+        <v>0.1242430460983302</v>
       </c>
       <c r="CW69" s="1" t="n">
         <v>2</v>
@@ -23051,19 +23051,19 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>11.14</v>
+        <v>12.21</v>
       </c>
       <c r="F70" t="b">
         <v>0</v>
       </c>
       <c r="G70" t="n">
-        <v>8.859999999999999</v>
+        <v>10.32</v>
       </c>
       <c r="H70" t="n">
-        <v>11.14</v>
+        <v>10.24</v>
       </c>
       <c r="I70" t="n">
-        <v>11.14</v>
+        <v>11.58</v>
       </c>
       <c r="J70" t="inlineStr">
         <is>
@@ -23352,7 +23352,7 @@
         <v>38.80055686046524</v>
       </c>
       <c r="CV70" t="n">
-        <v>0.1114285714285714</v>
+        <v>0.1221047926044134</v>
       </c>
       <c r="CW70" t="n">
         <v>4</v>
@@ -23376,19 +23376,19 @@
         </is>
       </c>
       <c r="E71" s="2" t="n">
-        <v>18</v>
+        <v>12.43</v>
       </c>
       <c r="F71" s="2" t="b">
         <v>0</v>
       </c>
       <c r="G71" s="2" t="n">
-        <v>18</v>
+        <v>12.52</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>4.29</v>
+        <v>8.460000000000001</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>8.859999999999999</v>
+        <v>11.58</v>
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
@@ -23677,7 +23677,7 @@
         <v>31.60264059661428</v>
       </c>
       <c r="CV71" s="2" t="n">
-        <v>0.18</v>
+        <v>0.1242600734309794</v>
       </c>
       <c r="CW71" s="2" t="n">
         <v>1</v>
@@ -23701,19 +23701,19 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>6.57</v>
+        <v>11.1</v>
       </c>
       <c r="F72" t="b">
         <v>0</v>
       </c>
       <c r="G72" t="n">
-        <v>4.29</v>
+        <v>6.78</v>
       </c>
       <c r="H72" t="n">
-        <v>8.859999999999999</v>
+        <v>10.24</v>
       </c>
       <c r="I72" t="n">
-        <v>6.57</v>
+        <v>11.58</v>
       </c>
       <c r="J72" t="inlineStr">
         <is>
@@ -24002,7 +24002,7 @@
         <v>53.70946451048647</v>
       </c>
       <c r="CV72" t="n">
-        <v>0.0657142857142857</v>
+        <v>0.1109997146973182</v>
       </c>
       <c r="CW72" t="n">
         <v>6</v>
@@ -24026,19 +24026,19 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>4.29</v>
+        <v>9.01</v>
       </c>
       <c r="F73" t="b">
         <v>0</v>
       </c>
       <c r="G73" t="n">
-        <v>2</v>
+        <v>4.46</v>
       </c>
       <c r="H73" t="n">
-        <v>6.57</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="I73" t="n">
-        <v>4.29</v>
+        <v>9.6</v>
       </c>
       <c r="J73" t="inlineStr">
         <is>
@@ -24327,7 +24327,7 @@
         <v>29.06154264337536</v>
       </c>
       <c r="CV73" t="n">
-        <v>0.04285714285714284</v>
+        <v>0.09008876386284712</v>
       </c>
       <c r="CW73" t="n">
         <v>7</v>
@@ -24351,19 +24351,19 @@
         </is>
       </c>
       <c r="E74" s="5" t="n">
-        <v>18</v>
+        <v>14.62</v>
       </c>
       <c r="F74" s="5" t="b">
         <v>0</v>
       </c>
       <c r="G74" s="5" t="n">
-        <v>18</v>
+        <v>17.91</v>
       </c>
       <c r="H74" s="5" t="n">
-        <v>18</v>
+        <v>10.24</v>
       </c>
       <c r="I74" s="5" t="n">
-        <v>18</v>
+        <v>11.62</v>
       </c>
       <c r="J74" s="5" t="inlineStr">
         <is>
@@ -24652,7 +24652,7 @@
         <v>85.8015852009059</v>
       </c>
       <c r="CV74" s="5" t="n">
-        <v>0.18</v>
+        <v>0.1461562568166435</v>
       </c>
       <c r="CW74" s="5" t="n">
         <v>1</v>
@@ -24676,19 +24676,19 @@
         </is>
       </c>
       <c r="E75" s="3" t="n">
-        <v>13.43</v>
+        <v>12.6</v>
       </c>
       <c r="F75" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G75" s="3" t="n">
-        <v>13.43</v>
+        <v>11.55</v>
       </c>
       <c r="H75" s="3" t="n">
-        <v>15.71</v>
+        <v>10.24</v>
       </c>
       <c r="I75" s="3" t="n">
-        <v>13.43</v>
+        <v>11.58</v>
       </c>
       <c r="J75" s="3" t="inlineStr">
         <is>
@@ -24975,7 +24975,7 @@
         <v>25.47754324226814</v>
       </c>
       <c r="CV75" s="3" t="n">
-        <v>0.1342857142857143</v>
+        <v>0.12597087874892</v>
       </c>
       <c r="CW75" s="3" t="n">
         <v>3</v>
@@ -24999,19 +24999,19 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>6.57</v>
+        <v>7.23</v>
       </c>
       <c r="F76" t="b">
         <v>0</v>
       </c>
       <c r="G76" t="n">
-        <v>6.57</v>
+        <v>5.37</v>
       </c>
       <c r="H76" t="n">
-        <v>4.29</v>
+        <v>6.46</v>
       </c>
       <c r="I76" t="n">
-        <v>4.29</v>
+        <v>7.36</v>
       </c>
       <c r="J76" t="inlineStr">
         <is>
@@ -25300,7 +25300,7 @@
         <v>38.43614274873409</v>
       </c>
       <c r="CV76" t="n">
-        <v>0.0657142857142857</v>
+        <v>0.07230010924647921</v>
       </c>
       <c r="CW76" t="n">
         <v>6</v>
@@ -25324,19 +25324,19 @@
         </is>
       </c>
       <c r="E77" s="1" t="n">
-        <v>15.71</v>
+        <v>13.38</v>
       </c>
       <c r="F77" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G77" s="1" t="n">
-        <v>15.71</v>
+        <v>14.07</v>
       </c>
       <c r="H77" s="1" t="n">
-        <v>13.43</v>
+        <v>10.24</v>
       </c>
       <c r="I77" s="1" t="n">
-        <v>11.14</v>
+        <v>11.58</v>
       </c>
       <c r="J77" s="1" t="inlineStr">
         <is>
@@ -25623,7 +25623,7 @@
         <v>36.03382967907977</v>
       </c>
       <c r="CV77" s="1" t="n">
-        <v>0.1571428571428571</v>
+        <v>0.1338490735697367</v>
       </c>
       <c r="CW77" s="1" t="n">
         <v>2</v>
@@ -25647,19 +25647,19 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>2</v>
+        <v>4.28</v>
       </c>
       <c r="F78" t="b">
         <v>0</v>
       </c>
       <c r="G78" t="n">
-        <v>4.29</v>
+        <v>2.7</v>
       </c>
       <c r="H78" t="n">
-        <v>2</v>
+        <v>3.63</v>
       </c>
       <c r="I78" t="n">
-        <v>2</v>
+        <v>4.99</v>
       </c>
       <c r="J78" t="inlineStr">
         <is>
@@ -25948,7 +25948,7 @@
         <v>24.81903031572897</v>
       </c>
       <c r="CV78" t="n">
-        <v>0.01999999999999999</v>
+        <v>0.04277681384407453</v>
       </c>
       <c r="CW78" t="n">
         <v>8</v>
@@ -25972,19 +25972,19 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>4.29</v>
+        <v>6.65</v>
       </c>
       <c r="F79" t="b">
         <v>0</v>
       </c>
       <c r="G79" t="n">
-        <v>2</v>
+        <v>2.28</v>
       </c>
       <c r="H79" t="n">
-        <v>6.57</v>
+        <v>7.34</v>
       </c>
       <c r="I79" t="n">
-        <v>6.57</v>
+        <v>7.64</v>
       </c>
       <c r="J79" t="inlineStr">
         <is>
@@ -26273,7 +26273,7 @@
         <v>22.87088606731296</v>
       </c>
       <c r="CV79" t="n">
-        <v>0.04285714285714284</v>
+        <v>0.06654146272515976</v>
       </c>
       <c r="CW79" t="n">
         <v>7</v>
@@ -26297,19 +26297,19 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>11.14</v>
+        <v>12.1</v>
       </c>
       <c r="F80" t="b">
         <v>0</v>
       </c>
       <c r="G80" t="n">
-        <v>11.14</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="H80" t="n">
-        <v>11.14</v>
+        <v>10.24</v>
       </c>
       <c r="I80" t="n">
-        <v>15.71</v>
+        <v>11.62</v>
       </c>
       <c r="J80" t="inlineStr">
         <is>
@@ -26598,7 +26598,7 @@
         <v>22.22177619022168</v>
       </c>
       <c r="CV80" t="n">
-        <v>0.1114285714285714</v>
+        <v>0.1209556339874651</v>
       </c>
       <c r="CW80" t="n">
         <v>4</v>
@@ -26622,19 +26622,19 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>8.859999999999999</v>
+        <v>11</v>
       </c>
       <c r="F81" t="b">
         <v>0</v>
       </c>
       <c r="G81" t="n">
-        <v>8.859999999999999</v>
+        <v>6.46</v>
       </c>
       <c r="H81" t="n">
-        <v>8.859999999999999</v>
+        <v>10.24</v>
       </c>
       <c r="I81" t="n">
-        <v>8.859999999999999</v>
+        <v>11.58</v>
       </c>
       <c r="J81" t="inlineStr">
         <is>
@@ -26923,7 +26923,7 @@
         <v>57.61952442577206</v>
       </c>
       <c r="CV81" t="n">
-        <v>0.08857142857142856</v>
+        <v>0.110012586592348</v>
       </c>
       <c r="CW81" t="n">
         <v>5</v>
@@ -26947,19 +26947,19 @@
         </is>
       </c>
       <c r="E82" s="5" t="n">
-        <v>18</v>
+        <v>14.13</v>
       </c>
       <c r="F82" s="5" t="b">
         <v>0</v>
       </c>
       <c r="G82" s="5" t="n">
-        <v>18</v>
+        <v>16.14</v>
       </c>
       <c r="H82" s="5" t="n">
-        <v>18</v>
+        <v>10.5</v>
       </c>
       <c r="I82" s="5" t="n">
-        <v>18</v>
+        <v>11.62</v>
       </c>
       <c r="J82" s="5" t="inlineStr">
         <is>
@@ -27250,7 +27250,7 @@
         <v>53.96801563051854</v>
       </c>
       <c r="CV82" s="5" t="n">
-        <v>0.18</v>
+        <v>0.1413227815094745</v>
       </c>
       <c r="CW82" s="5" t="n">
         <v>1</v>
@@ -27274,19 +27274,19 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>11.14</v>
+        <v>10.67</v>
       </c>
       <c r="F83" t="b">
         <v>0</v>
       </c>
       <c r="G83" t="n">
-        <v>2</v>
+        <v>6.9</v>
       </c>
       <c r="H83" t="n">
-        <v>13.43</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="I83" t="n">
-        <v>15.71</v>
+        <v>11.58</v>
       </c>
       <c r="J83" t="inlineStr">
         <is>
@@ -27577,7 +27577,7 @@
         <v>50.07658093812963</v>
       </c>
       <c r="CV83" t="n">
-        <v>0.1114285714285714</v>
+        <v>0.1066546793715363</v>
       </c>
       <c r="CW83" t="n">
         <v>4</v>
@@ -27601,19 +27601,19 @@
         </is>
       </c>
       <c r="E84" s="1" t="n">
-        <v>15.71</v>
+        <v>11.81</v>
       </c>
       <c r="F84" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G84" s="1" t="n">
-        <v>15.71</v>
+        <v>10.56</v>
       </c>
       <c r="H84" s="1" t="n">
-        <v>11.14</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="I84" s="1" t="n">
-        <v>11.14</v>
+        <v>11.58</v>
       </c>
       <c r="J84" s="1" t="inlineStr">
         <is>
@@ -27902,7 +27902,7 @@
         <v>64.77720898919421</v>
       </c>
       <c r="CV84" s="1" t="n">
-        <v>0.1571428571428571</v>
+        <v>0.1181110315562744</v>
       </c>
       <c r="CW84" s="1" t="n">
         <v>2</v>
@@ -27926,19 +27926,19 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>2</v>
+        <v>8.76</v>
       </c>
       <c r="F85" t="b">
         <v>0</v>
       </c>
       <c r="G85" t="n">
-        <v>4.29</v>
+        <v>6.91</v>
       </c>
       <c r="H85" t="n">
-        <v>6.57</v>
+        <v>5.58</v>
       </c>
       <c r="I85" t="n">
-        <v>4.29</v>
+        <v>9.6</v>
       </c>
       <c r="J85" t="inlineStr">
         <is>
@@ -28229,7 +28229,7 @@
         <v>29.51395222324777</v>
       </c>
       <c r="CV85" t="n">
-        <v>0.01999999999999999</v>
+        <v>0.08761060563044189</v>
       </c>
       <c r="CW85" t="n">
         <v>8</v>
@@ -28253,19 +28253,19 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>4.29</v>
+        <v>8.82</v>
       </c>
       <c r="F86" t="b">
         <v>0</v>
       </c>
       <c r="G86" t="n">
-        <v>6.57</v>
+        <v>7.02</v>
       </c>
       <c r="H86" t="n">
-        <v>8.859999999999999</v>
+        <v>6.29</v>
       </c>
       <c r="I86" t="n">
-        <v>2</v>
+        <v>9.31</v>
       </c>
       <c r="J86" t="inlineStr">
         <is>
@@ -28554,7 +28554,7 @@
         <v>28.57141039010677</v>
       </c>
       <c r="CV86" t="n">
-        <v>0.04285714285714284</v>
+        <v>0.08821311567074383</v>
       </c>
       <c r="CW86" t="n">
         <v>7</v>
@@ -28578,19 +28578,19 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>6.57</v>
+        <v>9.74</v>
       </c>
       <c r="F87" t="b">
         <v>0</v>
       </c>
       <c r="G87" t="n">
-        <v>8.859999999999999</v>
+        <v>7.36</v>
       </c>
       <c r="H87" t="n">
-        <v>2</v>
+        <v>4.89</v>
       </c>
       <c r="I87" t="n">
-        <v>8.859999999999999</v>
+        <v>11.39</v>
       </c>
       <c r="J87" t="inlineStr">
         <is>
@@ -28881,7 +28881,7 @@
         <v>44.49737182697936</v>
       </c>
       <c r="CV87" t="n">
-        <v>0.0657142857142857</v>
+        <v>0.09741192330286901</v>
       </c>
       <c r="CW87" t="n">
         <v>6</v>
@@ -28905,19 +28905,19 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>8.859999999999999</v>
+        <v>9.94</v>
       </c>
       <c r="F88" t="b">
         <v>0</v>
       </c>
       <c r="G88" t="n">
-        <v>11.14</v>
+        <v>7.92</v>
       </c>
       <c r="H88" t="n">
-        <v>4.29</v>
+        <v>5.18</v>
       </c>
       <c r="I88" t="n">
-        <v>6.57</v>
+        <v>11.29</v>
       </c>
       <c r="J88" t="inlineStr">
         <is>
@@ -29206,7 +29206,7 @@
         <v>24.07066316723411</v>
       </c>
       <c r="CV88" t="n">
-        <v>0.08857142857142856</v>
+        <v>0.09943051305345639</v>
       </c>
       <c r="CW88" t="n">
         <v>5</v>
@@ -29230,19 +29230,19 @@
         </is>
       </c>
       <c r="E89" s="3" t="n">
-        <v>13.43</v>
+        <v>11.5</v>
       </c>
       <c r="F89" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G89" s="3" t="n">
-        <v>13.43</v>
+        <v>8.9</v>
       </c>
       <c r="H89" s="3" t="n">
-        <v>15.71</v>
+        <v>9.24</v>
       </c>
       <c r="I89" s="3" t="n">
-        <v>13.43</v>
+        <v>11.58</v>
       </c>
       <c r="J89" s="3" t="inlineStr">
         <is>
@@ -29531,7 +29531,7 @@
         <v>49.9400151730756</v>
       </c>
       <c r="CV89" s="3" t="n">
-        <v>0.1342857142857143</v>
+        <v>0.1149933309460629</v>
       </c>
       <c r="CW89" s="3" t="n">
         <v>3</v>
@@ -29555,19 +29555,19 @@
         </is>
       </c>
       <c r="E90" s="4" t="n">
-        <v>15.71</v>
+        <v>11.68</v>
       </c>
       <c r="F90" s="4" t="b">
         <v>0</v>
       </c>
       <c r="G90" s="4" t="n">
-        <v>15.71</v>
+        <v>9.16</v>
       </c>
       <c r="H90" s="4" t="n">
-        <v>18</v>
+        <v>10.24</v>
       </c>
       <c r="I90" s="4" t="n">
-        <v>11.14</v>
+        <v>11.29</v>
       </c>
       <c r="J90" s="4" t="inlineStr">
         <is>
@@ -29856,7 +29856,7 @@
         <v>28.3532464944545</v>
       </c>
       <c r="CV90" s="4" t="n">
-        <v>0.1571428571428571</v>
+        <v>0.1168354740954161</v>
       </c>
       <c r="CW90" s="4" t="n">
         <v>2</v>
@@ -29880,19 +29880,19 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>11.14</v>
+        <v>10.08</v>
       </c>
       <c r="F91" t="b">
         <v>0</v>
       </c>
       <c r="G91" t="n">
-        <v>8.859999999999999</v>
+        <v>5.61</v>
       </c>
       <c r="H91" t="n">
-        <v>11.14</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="I91" t="n">
-        <v>13.43</v>
+        <v>11.43</v>
       </c>
       <c r="J91" t="inlineStr">
         <is>
@@ -30181,7 +30181,7 @@
         <v>30.08154658232777</v>
       </c>
       <c r="CV91" t="n">
-        <v>0.1114285714285714</v>
+        <v>0.1008271316272244</v>
       </c>
       <c r="CW91" t="n">
         <v>4</v>
@@ -30205,19 +30205,19 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>8.859999999999999</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="F92" t="b">
         <v>0</v>
       </c>
       <c r="G92" t="n">
-        <v>11.14</v>
+        <v>6.35</v>
       </c>
       <c r="H92" t="n">
-        <v>8.859999999999999</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="I92" t="n">
-        <v>8.859999999999999</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="J92" t="inlineStr">
         <is>
@@ -30506,7 +30506,7 @@
         <v>18.85890646783279</v>
       </c>
       <c r="CV92" t="n">
-        <v>0.08857142857142856</v>
+        <v>0.09286910562217343</v>
       </c>
       <c r="CW92" t="n">
         <v>5</v>
@@ -30530,19 +30530,19 @@
         </is>
       </c>
       <c r="E93" s="3" t="n">
-        <v>13.43</v>
+        <v>11.44</v>
       </c>
       <c r="F93" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G93" s="3" t="n">
-        <v>13.43</v>
+        <v>7.78</v>
       </c>
       <c r="H93" s="3" t="n">
-        <v>15.71</v>
+        <v>10.24</v>
       </c>
       <c r="I93" s="3" t="n">
-        <v>18</v>
+        <v>11.62</v>
       </c>
       <c r="J93" s="3" t="inlineStr">
         <is>
@@ -30831,7 +30831,7 @@
         <v>27.18101321832401</v>
       </c>
       <c r="CV93" s="3" t="n">
-        <v>0.1342857142857143</v>
+        <v>0.1144087509620835</v>
       </c>
       <c r="CW93" s="3" t="n">
         <v>3</v>
@@ -30855,19 +30855,19 @@
         </is>
       </c>
       <c r="E94" s="2" t="n">
-        <v>18</v>
+        <v>13.77</v>
       </c>
       <c r="F94" s="2" t="b">
         <v>0</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>18</v>
+        <v>15.45</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>13.43</v>
+        <v>10.05</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>15.71</v>
+        <v>11.58</v>
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
@@ -31156,7 +31156,7 @@
         <v>64.93266365228394</v>
       </c>
       <c r="CV94" s="2" t="n">
-        <v>0.18</v>
+        <v>0.1376875317416117</v>
       </c>
       <c r="CW94" s="2" t="n">
         <v>1</v>
@@ -31180,7 +31180,7 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>6.57</v>
+        <v>7.6</v>
       </c>
       <c r="F95" t="b">
         <v>0</v>
@@ -31189,10 +31189,10 @@
         <v>2</v>
       </c>
       <c r="H95" t="n">
-        <v>4.29</v>
+        <v>7.6</v>
       </c>
       <c r="I95" t="n">
-        <v>6.57</v>
+        <v>9.31</v>
       </c>
       <c r="J95" t="inlineStr">
         <is>
@@ -31481,7 +31481,7 @@
         <v>22.67832686238685</v>
       </c>
       <c r="CV95" t="n">
-        <v>0.0657142857142857</v>
+        <v>0.07595555040667837</v>
       </c>
       <c r="CW95" t="n">
         <v>6</v>
@@ -31505,19 +31505,19 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>4.29</v>
+        <v>7.1</v>
       </c>
       <c r="F96" t="b">
         <v>0</v>
       </c>
       <c r="G96" t="n">
-        <v>6.57</v>
+        <v>4.45</v>
       </c>
       <c r="H96" t="n">
-        <v>2</v>
+        <v>6.29</v>
       </c>
       <c r="I96" t="n">
-        <v>4.29</v>
+        <v>7.72</v>
       </c>
       <c r="J96" t="inlineStr">
         <is>
@@ -31806,7 +31806,7 @@
         <v>16.04284401437255</v>
       </c>
       <c r="CV96" t="n">
-        <v>0.04285714285714284</v>
+        <v>0.07099413751803997</v>
       </c>
       <c r="CW96" t="n">
         <v>7</v>
@@ -31830,19 +31830,19 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>2</v>
+        <v>6.81</v>
       </c>
       <c r="F97" t="b">
         <v>0</v>
       </c>
       <c r="G97" t="n">
-        <v>4.29</v>
+        <v>3.67</v>
       </c>
       <c r="H97" t="n">
-        <v>6.57</v>
+        <v>7.69</v>
       </c>
       <c r="I97" t="n">
-        <v>2</v>
+        <v>6.98</v>
       </c>
       <c r="J97" t="inlineStr">
         <is>
@@ -32131,7 +32131,7 @@
         <v>30.34931018708762</v>
       </c>
       <c r="CV97" t="n">
-        <v>0.01999999999999999</v>
+        <v>0.06805660235555747</v>
       </c>
       <c r="CW97" t="n">
         <v>8</v>
@@ -32155,16 +32155,16 @@
         </is>
       </c>
       <c r="E98" s="4" t="n">
-        <v>15.71</v>
+        <v>17.8</v>
       </c>
       <c r="F98" s="4" t="b">
         <v>0</v>
       </c>
       <c r="G98" s="4" t="n">
-        <v>13.43</v>
+        <v>13.34</v>
       </c>
       <c r="H98" s="4" t="n">
-        <v>15.71</v>
+        <v>13.82</v>
       </c>
       <c r="I98" s="4" t="n">
         <v>18</v>
@@ -32456,7 +32456,7 @@
         <v>91.61958227166119</v>
       </c>
       <c r="CV98" s="4" t="n">
-        <v>0.1571428571428571</v>
+        <v>0.1779551445446888</v>
       </c>
       <c r="CW98" s="4" t="n">
         <v>2</v>
@@ -32480,19 +32480,19 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>6.57</v>
+        <v>9.51</v>
       </c>
       <c r="F99" t="b">
         <v>0</v>
       </c>
       <c r="G99" t="n">
-        <v>11.14</v>
+        <v>11.73</v>
       </c>
       <c r="H99" t="n">
-        <v>2</v>
+        <v>5.96</v>
       </c>
       <c r="I99" t="n">
-        <v>2</v>
+        <v>8.1</v>
       </c>
       <c r="J99" t="inlineStr">
         <is>
@@ -32781,7 +32781,7 @@
         <v>59.34107165923448</v>
       </c>
       <c r="CV99" t="n">
-        <v>0.0657142857142857</v>
+        <v>0.09510487901085468</v>
       </c>
       <c r="CW99" t="n">
         <v>6</v>
@@ -32805,19 +32805,19 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>8.859999999999999</v>
+        <v>11.22</v>
       </c>
       <c r="F100" t="b">
         <v>0</v>
       </c>
       <c r="G100" t="n">
-        <v>8.859999999999999</v>
+        <v>11.12</v>
       </c>
       <c r="H100" t="n">
-        <v>8.859999999999999</v>
+        <v>8.82</v>
       </c>
       <c r="I100" t="n">
-        <v>8.859999999999999</v>
+        <v>10.08</v>
       </c>
       <c r="J100" t="inlineStr">
         <is>
@@ -33106,7 +33106,7 @@
         <v>28.55079792458181</v>
       </c>
       <c r="CV100" t="n">
-        <v>0.08857142857142856</v>
+        <v>0.1122137824173133</v>
       </c>
       <c r="CW100" t="n">
         <v>5</v>
@@ -33130,19 +33130,19 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>11.14</v>
+        <v>13.89</v>
       </c>
       <c r="F101" t="b">
         <v>0</v>
       </c>
       <c r="G101" t="n">
-        <v>6.57</v>
+        <v>10.2</v>
       </c>
       <c r="H101" t="n">
-        <v>13.43</v>
+        <v>12.78</v>
       </c>
       <c r="I101" t="n">
-        <v>11.14</v>
+        <v>13.39</v>
       </c>
       <c r="J101" t="inlineStr">
         <is>
@@ -33431,7 +33431,7 @@
         <v>92.45537145739141</v>
       </c>
       <c r="CV101" t="n">
-        <v>0.1114285714285714</v>
+        <v>0.1389169596995703</v>
       </c>
       <c r="CW101" t="n">
         <v>4</v>
@@ -33455,19 +33455,19 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>2</v>
+        <v>7.79</v>
       </c>
       <c r="F102" t="b">
         <v>0</v>
       </c>
       <c r="G102" t="n">
-        <v>2</v>
+        <v>5.83</v>
       </c>
       <c r="H102" t="n">
-        <v>4.29</v>
+        <v>6.41</v>
       </c>
       <c r="I102" t="n">
-        <v>4.29</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="J102" t="inlineStr">
         <is>
@@ -33756,7 +33756,7 @@
         <v>43.29191348128838</v>
       </c>
       <c r="CV102" t="n">
-        <v>0.01999999999999999</v>
+        <v>0.07792872445607733</v>
       </c>
       <c r="CW102" t="n">
         <v>8</v>
@@ -33780,19 +33780,19 @@
         </is>
       </c>
       <c r="E103" s="3" t="n">
-        <v>13.43</v>
+        <v>14.99</v>
       </c>
       <c r="F103" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G103" s="3" t="n">
-        <v>15.71</v>
+        <v>14.18</v>
       </c>
       <c r="H103" s="3" t="n">
-        <v>11.14</v>
+        <v>11.99</v>
       </c>
       <c r="I103" s="3" t="n">
-        <v>13.43</v>
+        <v>13.5</v>
       </c>
       <c r="J103" s="3" t="inlineStr">
         <is>
@@ -34081,7 +34081,7 @@
         <v>30.15574520228456</v>
       </c>
       <c r="CV103" s="3" t="n">
-        <v>0.1342857142857143</v>
+        <v>0.1498924128068796</v>
       </c>
       <c r="CW103" s="3" t="n">
         <v>3</v>
@@ -34105,19 +34105,19 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>4.29</v>
+        <v>9.07</v>
       </c>
       <c r="F104" t="b">
         <v>0</v>
       </c>
       <c r="G104" t="n">
-        <v>4.29</v>
+        <v>6.8</v>
       </c>
       <c r="H104" t="n">
-        <v>6.57</v>
+        <v>8.5</v>
       </c>
       <c r="I104" t="n">
-        <v>6.57</v>
+        <v>8.84</v>
       </c>
       <c r="J104" t="inlineStr">
         <is>
@@ -34406,7 +34406,7 @@
         <v>44.51260000900377</v>
       </c>
       <c r="CV104" t="n">
-        <v>0.04285714285714284</v>
+        <v>0.09069924969842802</v>
       </c>
       <c r="CW104" t="n">
         <v>7</v>
@@ -34436,13 +34436,13 @@
         <v>0</v>
       </c>
       <c r="G105" s="2" t="n">
-        <v>18</v>
+        <v>16.63</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>18</v>
+        <v>17.09</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>15.71</v>
+        <v>15.03</v>
       </c>
       <c r="J105" s="2" t="inlineStr">
         <is>
@@ -34755,19 +34755,19 @@
         </is>
       </c>
       <c r="E106" s="6" t="n">
-        <v>6.57</v>
+        <v>11.48</v>
       </c>
       <c r="F106" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G106" s="6" t="n">
-        <v>8.859999999999999</v>
+        <v>11.05</v>
       </c>
       <c r="H106" s="6" t="n">
-        <v>6.57</v>
+        <v>7.26</v>
       </c>
       <c r="I106" s="6" t="n">
-        <v>6.57</v>
+        <v>11.29</v>
       </c>
       <c r="J106" s="6" t="inlineStr">
         <is>
@@ -35054,7 +35054,7 @@
         <v>30.37971239734789</v>
       </c>
       <c r="CV106" s="6" t="n">
-        <v>0.0657142857142857</v>
+        <v>0.1148037630057862</v>
       </c>
       <c r="CW106" s="6" t="n">
         <v>6</v>
@@ -35078,19 +35078,19 @@
         </is>
       </c>
       <c r="E107" s="2" t="n">
-        <v>18</v>
+        <v>14.82</v>
       </c>
       <c r="F107" s="2" t="b">
         <v>0</v>
       </c>
       <c r="G107" s="2" t="n">
-        <v>11.14</v>
+        <v>13.14</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>18</v>
+        <v>16.61</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>18</v>
+        <v>11.62</v>
       </c>
       <c r="J107" s="2" t="inlineStr">
         <is>
@@ -35379,7 +35379,7 @@
         <v>43.12778647289818</v>
       </c>
       <c r="CV107" s="2" t="n">
-        <v>0.18</v>
+        <v>0.1482450244317615</v>
       </c>
       <c r="CW107" s="2" t="n">
         <v>1</v>
@@ -35403,19 +35403,19 @@
         </is>
       </c>
       <c r="E108" s="3" t="n">
-        <v>13.43</v>
+        <v>14.63</v>
       </c>
       <c r="F108" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G108" s="3" t="n">
-        <v>15.71</v>
+        <v>14.62</v>
       </c>
       <c r="H108" s="3" t="n">
-        <v>15.71</v>
+        <v>14.14</v>
       </c>
       <c r="I108" s="3" t="n">
-        <v>15.71</v>
+        <v>11.62</v>
       </c>
       <c r="J108" s="3" t="inlineStr">
         <is>
@@ -35704,7 +35704,7 @@
         <v>24.21244959699635</v>
       </c>
       <c r="CV108" s="3" t="n">
-        <v>0.1342857142857143</v>
+        <v>0.1462933805433594</v>
       </c>
       <c r="CW108" s="3" t="n">
         <v>3</v>
@@ -35728,19 +35728,19 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>11.14</v>
+        <v>13.83</v>
       </c>
       <c r="F109" t="b">
         <v>0</v>
       </c>
       <c r="G109" t="n">
-        <v>13.43</v>
+        <v>14.07</v>
       </c>
       <c r="H109" t="n">
-        <v>13.43</v>
+        <v>11.81</v>
       </c>
       <c r="I109" t="n">
-        <v>13.43</v>
+        <v>11.62</v>
       </c>
       <c r="J109" t="inlineStr">
         <is>
@@ -36029,7 +36029,7 @@
         <v>42.20660116092578</v>
       </c>
       <c r="CV109" t="n">
-        <v>0.1114285714285714</v>
+        <v>0.1383368596873879</v>
       </c>
       <c r="CW109" t="n">
         <v>4</v>
@@ -36053,19 +36053,19 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>8.859999999999999</v>
+        <v>11.92</v>
       </c>
       <c r="F110" t="b">
         <v>0</v>
       </c>
       <c r="G110" t="n">
-        <v>6.57</v>
+        <v>10.86</v>
       </c>
       <c r="H110" t="n">
-        <v>8.859999999999999</v>
+        <v>8.529999999999999</v>
       </c>
       <c r="I110" t="n">
-        <v>11.14</v>
+        <v>11.58</v>
       </c>
       <c r="J110" t="inlineStr">
         <is>
@@ -36356,7 +36356,7 @@
         <v>47.34855344121042</v>
       </c>
       <c r="CV110" t="n">
-        <v>0.08857142857142856</v>
+        <v>0.1192485346300177</v>
       </c>
       <c r="CW110" t="n">
         <v>5</v>
@@ -36380,19 +36380,19 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>2</v>
+        <v>8.640000000000001</v>
       </c>
       <c r="F111" t="b">
         <v>0</v>
       </c>
       <c r="G111" t="n">
-        <v>2</v>
+        <v>4.52</v>
       </c>
       <c r="H111" t="n">
-        <v>2</v>
+        <v>4.72</v>
       </c>
       <c r="I111" t="n">
-        <v>4.29</v>
+        <v>11.1</v>
       </c>
       <c r="J111" t="inlineStr">
         <is>
@@ -36683,7 +36683,7 @@
         <v>27.07594089234863</v>
       </c>
       <c r="CV111" t="n">
-        <v>0.01999999999999999</v>
+        <v>0.08643995202848505</v>
       </c>
       <c r="CW111" t="n">
         <v>8</v>
@@ -36707,19 +36707,19 @@
         </is>
       </c>
       <c r="E112" s="1" t="n">
-        <v>15.71</v>
+        <v>14.65</v>
       </c>
       <c r="F112" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G112" s="1" t="n">
-        <v>18</v>
+        <v>17.48</v>
       </c>
       <c r="H112" s="1" t="n">
-        <v>11.14</v>
+        <v>10.95</v>
       </c>
       <c r="I112" s="1" t="n">
-        <v>8.859999999999999</v>
+        <v>11.58</v>
       </c>
       <c r="J112" s="1" t="inlineStr">
         <is>
@@ -37008,7 +37008,7 @@
         <v>60.30245636445544</v>
       </c>
       <c r="CV112" s="1" t="n">
-        <v>0.1571428571428571</v>
+        <v>0.1464767422145831</v>
       </c>
       <c r="CW112" s="1" t="n">
         <v>2</v>
@@ -37032,19 +37032,19 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>4.29</v>
+        <v>9.779999999999999</v>
       </c>
       <c r="F113" t="b">
         <v>0</v>
       </c>
       <c r="G113" t="n">
-        <v>4.29</v>
+        <v>7.59</v>
       </c>
       <c r="H113" t="n">
-        <v>4.29</v>
+        <v>6.27</v>
       </c>
       <c r="I113" t="n">
-        <v>2</v>
+        <v>10.69</v>
       </c>
       <c r="J113" t="inlineStr">
         <is>
@@ -37333,7 +37333,7 @@
         <v>32.49249494855098</v>
       </c>
       <c r="CV113" t="n">
-        <v>0.04285714285714284</v>
+        <v>0.09783443958946111</v>
       </c>
       <c r="CW113" t="n">
         <v>7</v>
@@ -37357,19 +37357,19 @@
         </is>
       </c>
       <c r="E114" s="6" t="n">
-        <v>4.67</v>
+        <v>10.56</v>
       </c>
       <c r="F114" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G114" s="6" t="n">
-        <v>7.33</v>
+        <v>5.73</v>
       </c>
       <c r="H114" s="6" t="n">
-        <v>7.33</v>
+        <v>10.05</v>
       </c>
       <c r="I114" s="6" t="n">
-        <v>4.67</v>
+        <v>11.29</v>
       </c>
       <c r="J114" s="6" t="inlineStr">
         <is>
@@ -37658,7 +37658,7 @@
         <v>26.3508581179673</v>
       </c>
       <c r="CV114" s="6" t="n">
-        <v>0.04666666666666666</v>
+        <v>0.1055844910087013</v>
       </c>
       <c r="CW114" s="6" t="n">
         <v>6</v>
@@ -37682,19 +37682,19 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>10</v>
+        <v>11.15</v>
       </c>
       <c r="F115" t="b">
         <v>0</v>
       </c>
       <c r="G115" t="n">
-        <v>10</v>
+        <v>6.93</v>
       </c>
       <c r="H115" t="n">
-        <v>18</v>
+        <v>10.24</v>
       </c>
       <c r="I115" t="n">
-        <v>15.33</v>
+        <v>11.58</v>
       </c>
       <c r="J115" t="inlineStr">
         <is>
@@ -37983,7 +37983,7 @@
         <v>40.54367880590419</v>
       </c>
       <c r="CV115" t="n">
-        <v>0.09999999999999999</v>
+        <v>0.1114705197104486</v>
       </c>
       <c r="CW115" t="n">
         <v>4</v>
@@ -38007,19 +38007,19 @@
         </is>
       </c>
       <c r="E116" s="2" t="n">
-        <v>18</v>
+        <v>12.15</v>
       </c>
       <c r="F116" s="2" t="b">
         <v>0</v>
       </c>
       <c r="G116" s="2" t="n">
-        <v>18</v>
+        <v>10.92</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>4.67</v>
+        <v>9.32</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>12.67</v>
+        <v>11.58</v>
       </c>
       <c r="J116" s="2" t="inlineStr">
         <is>
@@ -38308,7 +38308,7 @@
         <v>24.04664557708335</v>
       </c>
       <c r="CV116" s="2" t="n">
-        <v>0.18</v>
+        <v>0.1215364409829806</v>
       </c>
       <c r="CW116" s="2" t="n">
         <v>1</v>
@@ -38332,19 +38332,19 @@
         </is>
       </c>
       <c r="E117" s="3" t="n">
-        <v>12.67</v>
+        <v>11.84</v>
       </c>
       <c r="F117" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G117" s="3" t="n">
-        <v>12.67</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="H117" s="3" t="n">
-        <v>15.33</v>
+        <v>10.24</v>
       </c>
       <c r="I117" s="3" t="n">
-        <v>18</v>
+        <v>11.58</v>
       </c>
       <c r="J117" s="3" t="inlineStr">
         <is>
@@ -38633,7 +38633,7 @@
         <v>62.87238122348094</v>
       </c>
       <c r="CV117" s="3" t="n">
-        <v>0.1266666666666666</v>
+        <v>0.1183711655661594</v>
       </c>
       <c r="CW117" s="3" t="n">
         <v>3</v>
@@ -38657,19 +38657,19 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>7.33</v>
+        <v>10.67</v>
       </c>
       <c r="F118" t="b">
         <v>0</v>
       </c>
       <c r="G118" t="n">
-        <v>4.67</v>
+        <v>5.41</v>
       </c>
       <c r="H118" t="n">
-        <v>12.67</v>
+        <v>10.24</v>
       </c>
       <c r="I118" t="n">
-        <v>10</v>
+        <v>11.58</v>
       </c>
       <c r="J118" t="inlineStr">
         <is>
@@ -38956,7 +38956,7 @@
         <v>21.64574847573774</v>
       </c>
       <c r="CV118" t="n">
-        <v>0.07333333333333333</v>
+        <v>0.1067186287996932</v>
       </c>
       <c r="CW118" t="n">
         <v>5</v>
@@ -38980,19 +38980,19 @@
         </is>
       </c>
       <c r="E119" s="1" t="n">
-        <v>15.33</v>
+        <v>11.93</v>
       </c>
       <c r="F119" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G119" s="1" t="n">
-        <v>15.33</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="H119" s="1" t="n">
-        <v>10</v>
+        <v>10.24</v>
       </c>
       <c r="I119" s="1" t="n">
-        <v>7.33</v>
+        <v>11.39</v>
       </c>
       <c r="J119" s="1" t="inlineStr">
         <is>
@@ -39281,7 +39281,7 @@
         <v>11.5815264566629</v>
       </c>
       <c r="CV119" s="1" t="n">
-        <v>0.1533333333333333</v>
+        <v>0.1193437212732578</v>
       </c>
       <c r="CW119" s="1" t="n">
         <v>2</v>
@@ -39305,19 +39305,19 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>2</v>
+        <v>6.47</v>
       </c>
       <c r="F120" t="b">
         <v>0</v>
       </c>
       <c r="G120" t="n">
-        <v>2</v>
+        <v>3.24</v>
       </c>
       <c r="H120" t="n">
-        <v>2</v>
+        <v>6.11</v>
       </c>
       <c r="I120" t="n">
-        <v>2</v>
+        <v>7.36</v>
       </c>
       <c r="J120" t="inlineStr">
         <is>
@@ -39606,7 +39606,7 @@
         <v>23.92513236435896</v>
       </c>
       <c r="CV120" t="n">
-        <v>0.01999999999999999</v>
+        <v>0.06467712609156663</v>
       </c>
       <c r="CW120" t="n">
         <v>7</v>
@@ -39630,19 +39630,19 @@
         </is>
       </c>
       <c r="E121" s="7" t="n">
-        <v>14</v>
+        <v>11.34</v>
       </c>
       <c r="F121" s="7" t="b">
         <v>0</v>
       </c>
       <c r="G121" s="7" t="n">
-        <v>14</v>
+        <v>11.16</v>
       </c>
       <c r="H121" s="7" t="n">
-        <v>18</v>
+        <v>10.24</v>
       </c>
       <c r="I121" s="7" t="n">
-        <v>8</v>
+        <v>9.6</v>
       </c>
       <c r="J121" s="7" t="inlineStr">
         <is>
@@ -39931,7 +39931,7 @@
         <v>24.49721249836809</v>
       </c>
       <c r="CV121" s="7" t="n">
-        <v>0.14</v>
+        <v>0.1133803182161693</v>
       </c>
       <c r="CW121" s="7" t="n">
         <v>3</v>
@@ -39955,19 +39955,19 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>10</v>
+        <v>11.05</v>
       </c>
       <c r="F122" t="b">
         <v>0</v>
       </c>
       <c r="G122" t="n">
-        <v>8</v>
+        <v>10.25</v>
       </c>
       <c r="H122" t="n">
-        <v>16</v>
+        <v>10.24</v>
       </c>
       <c r="I122" t="n">
-        <v>12</v>
+        <v>9.6</v>
       </c>
       <c r="J122" t="inlineStr">
         <is>
@@ -40256,7 +40256,7 @@
         <v>21.50906655216243</v>
       </c>
       <c r="CV122" t="n">
-        <v>0.09999999999999999</v>
+        <v>0.1105247524605231</v>
       </c>
       <c r="CW122" t="n">
         <v>5</v>
@@ -40280,19 +40280,19 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>4</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="F123" t="b">
         <v>0</v>
       </c>
       <c r="G123" t="n">
-        <v>2</v>
+        <v>4.34</v>
       </c>
       <c r="H123" t="n">
-        <v>14</v>
+        <v>10.24</v>
       </c>
       <c r="I123" t="n">
-        <v>6</v>
+        <v>9.31</v>
       </c>
       <c r="J123" t="inlineStr">
         <is>
@@ -40581,7 +40581,7 @@
         <v>21.19791767548602</v>
       </c>
       <c r="CV123" t="n">
-        <v>0.03999999999999998</v>
+        <v>0.09034258685754863</v>
       </c>
       <c r="CW123" t="n">
         <v>8</v>
@@ -40605,19 +40605,19 @@
         </is>
       </c>
       <c r="E124" s="1" t="n">
-        <v>16</v>
+        <v>12.21</v>
       </c>
       <c r="F124" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G124" s="1" t="n">
-        <v>10</v>
+        <v>10.6</v>
       </c>
       <c r="H124" s="1" t="n">
-        <v>12</v>
+        <v>10.24</v>
       </c>
       <c r="I124" s="1" t="n">
-        <v>16</v>
+        <v>11.43</v>
       </c>
       <c r="J124" s="1" t="inlineStr">
         <is>
@@ -40906,7 +40906,7 @@
         <v>18.22201178917614</v>
       </c>
       <c r="CV124" s="1" t="n">
-        <v>0.16</v>
+        <v>0.122139879081418</v>
       </c>
       <c r="CW124" s="1" t="n">
         <v>2</v>
@@ -40930,19 +40930,19 @@
         </is>
       </c>
       <c r="E125" s="2" t="n">
-        <v>18</v>
+        <v>13.28</v>
       </c>
       <c r="F125" s="2" t="b">
         <v>0</v>
       </c>
       <c r="G125" s="2" t="n">
-        <v>18</v>
+        <v>13.66</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>10</v>
+        <v>10.24</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>18</v>
+        <v>11.62</v>
       </c>
       <c r="J125" s="2" t="inlineStr">
         <is>
@@ -41231,7 +41231,7 @@
         <v>18.72317700674582</v>
       </c>
       <c r="CV125" s="2" t="n">
-        <v>0.18</v>
+        <v>0.1328329378366367</v>
       </c>
       <c r="CW125" s="2" t="n">
         <v>1</v>
@@ -41255,19 +41255,19 @@
         </is>
       </c>
       <c r="E126" t="n">
-        <v>6</v>
+        <v>9.35</v>
       </c>
       <c r="F126" t="b">
         <v>0</v>
       </c>
       <c r="G126" t="n">
-        <v>16</v>
+        <v>11.65</v>
       </c>
       <c r="H126" t="n">
-        <v>2</v>
+        <v>6.26</v>
       </c>
       <c r="I126" t="n">
-        <v>4</v>
+        <v>7.72</v>
       </c>
       <c r="J126" t="inlineStr">
         <is>
@@ -41556,7 +41556,7 @@
         <v>12.98002757137192</v>
       </c>
       <c r="CV126" t="n">
-        <v>0.06</v>
+        <v>0.09350685320716766</v>
       </c>
       <c r="CW126" t="n">
         <v>7</v>
@@ -41580,19 +41580,19 @@
         </is>
       </c>
       <c r="E127" t="n">
-        <v>12</v>
+        <v>11.26</v>
       </c>
       <c r="F127" t="b">
         <v>0</v>
       </c>
       <c r="G127" t="n">
-        <v>12</v>
+        <v>10.82</v>
       </c>
       <c r="H127" t="n">
-        <v>8</v>
+        <v>10.24</v>
       </c>
       <c r="I127" t="n">
-        <v>14</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="J127" t="inlineStr">
         <is>
@@ -41881,7 +41881,7 @@
         <v>51.13650385067046</v>
       </c>
       <c r="CV127" t="n">
-        <v>0.12</v>
+        <v>0.1125828877180351</v>
       </c>
       <c r="CW127" t="n">
         <v>4</v>
@@ -41905,19 +41905,19 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>8</v>
+        <v>10.2</v>
       </c>
       <c r="F128" t="b">
         <v>0</v>
       </c>
       <c r="G128" t="n">
-        <v>6</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="H128" t="n">
-        <v>6</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="I128" t="n">
-        <v>10</v>
+        <v>9.6</v>
       </c>
       <c r="J128" t="inlineStr">
         <is>
@@ -42206,7 +42206,7 @@
         <v>27.64384684853832</v>
       </c>
       <c r="CV128" t="n">
-        <v>0.07999999999999999</v>
+        <v>0.1019636707485432</v>
       </c>
       <c r="CW128" t="n">
         <v>6</v>
@@ -42230,19 +42230,19 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>2</v>
+        <v>8.6</v>
       </c>
       <c r="F129" t="b">
         <v>0</v>
       </c>
       <c r="G129" t="n">
-        <v>4</v>
+        <v>8.56</v>
       </c>
       <c r="H129" t="n">
-        <v>4</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="I129" t="n">
-        <v>2</v>
+        <v>7.23</v>
       </c>
       <c r="J129" t="inlineStr">
         <is>
@@ -42531,7 +42531,7 @@
         <v>28.81866530568137</v>
       </c>
       <c r="CV129" t="n">
-        <v>0.01999999999999999</v>
+        <v>0.08599834028628116</v>
       </c>
       <c r="CW129" t="n">
         <v>9</v>

</xml_diff>

<commit_message>
Remove ALL artificial normalization — output raw ML probabilities from PDF data only
Co-authored-by: danieljohnconstantine-a11y <229551202+danieljohnconstantine-a11y@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/track_ensemble_predictions.xlsx
+++ b/outputs/track_ensemble_predictions.xlsx
@@ -971,19 +971,19 @@
         </is>
       </c>
       <c r="E2" s="1" t="n">
-        <v>13.61</v>
+        <v>17.7065</v>
       </c>
       <c r="F2" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>13.07</v>
+        <v>22.3744</v>
       </c>
       <c r="H2" s="1" t="n">
-        <v>12.92</v>
+        <v>16.2981</v>
       </c>
       <c r="I2" s="1" t="n">
-        <v>10.64</v>
+        <v>16.0768</v>
       </c>
       <c r="J2" s="1" t="inlineStr">
         <is>
@@ -1272,7 +1272,7 @@
         <v>34.72964079687296</v>
       </c>
       <c r="CV2" s="1" t="n">
-        <v>0.1361329569776661</v>
+        <v>0.1770650921913965</v>
       </c>
       <c r="CW2" s="1" t="n">
         <v>2</v>
@@ -1296,19 +1296,19 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>13.92</v>
+        <v>17.963</v>
       </c>
       <c r="F3" s="2" t="b">
         <v>0</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>14</v>
+        <v>23.4004</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>12.92</v>
+        <v>16.2981</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>10.64</v>
+        <v>16.0768</v>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
@@ -1595,7 +1595,7 @@
         <v>32.03800807223286</v>
       </c>
       <c r="CV3" s="2" t="n">
-        <v>0.1391732451813974</v>
+        <v>0.1796300987855446</v>
       </c>
       <c r="CW3" s="2" t="n">
         <v>1</v>
@@ -1619,19 +1619,19 @@
         </is>
       </c>
       <c r="E4" s="3" t="n">
-        <v>12.82</v>
+        <v>17.0371</v>
       </c>
       <c r="F4" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>10.64</v>
+        <v>19.6968</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>12.92</v>
+        <v>16.2981</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>10.64</v>
+        <v>16.0768</v>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
@@ -1920,7 +1920,7 @@
         <v>25.61890479836698</v>
       </c>
       <c r="CV4" s="3" t="n">
-        <v>0.1281986298224856</v>
+        <v>0.1703711210579394</v>
       </c>
       <c r="CW4" s="3" t="n">
         <v>3</v>
@@ -1944,19 +1944,19 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>12.41</v>
+        <v>16.6897</v>
       </c>
       <c r="F5" t="b">
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>10.28</v>
+        <v>19.2972</v>
       </c>
       <c r="H5" t="n">
-        <v>11.79</v>
+        <v>15.3081</v>
       </c>
       <c r="I5" t="n">
-        <v>10.64</v>
+        <v>16.0768</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -2243,7 +2243,7 @@
         <v>22.50741453971432</v>
       </c>
       <c r="CV5" t="n">
-        <v>0.1240807669875728</v>
+        <v>0.1668969947193948</v>
       </c>
       <c r="CW5" t="n">
         <v>4</v>
@@ -2267,19 +2267,19 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>10.15</v>
+        <v>14.7809</v>
       </c>
       <c r="F6" t="b">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>8.42</v>
+        <v>17.2508</v>
       </c>
       <c r="H6" t="n">
-        <v>9.199999999999999</v>
+        <v>13.0628</v>
       </c>
       <c r="I6" t="n">
-        <v>8.99</v>
+        <v>14.405</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
         <v>21.29686553522198</v>
       </c>
       <c r="CV6" t="n">
-        <v>0.1014557131860618</v>
+        <v>0.1478088661259903</v>
       </c>
       <c r="CW6" t="n">
         <v>5</v>
@@ -2592,19 +2592,19 @@
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>13.82</v>
+        <v>17.8799</v>
       </c>
       <c r="F7" s="4" t="b">
         <v>0</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>13.7</v>
+        <v>23.0679</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>12.92</v>
+        <v>16.2981</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>10.64</v>
+        <v>16.0768</v>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
@@ -2893,7 +2893,7 @@
         <v>69.41178693631963</v>
       </c>
       <c r="CV7" s="4" t="n">
-        <v>0.1381879754279961</v>
+        <v>0.1787988540991404</v>
       </c>
       <c r="CW7" s="4" t="n">
         <v>2</v>
@@ -2917,19 +2917,19 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>11.1</v>
+        <v>15.5847</v>
       </c>
       <c r="F8" t="b">
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>7.38</v>
+        <v>16.1033</v>
       </c>
       <c r="H8" t="n">
-        <v>11.65</v>
+        <v>15.1909</v>
       </c>
       <c r="I8" t="n">
-        <v>10.09</v>
+        <v>15.5224</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -3218,7 +3218,7 @@
         <v>39.65910723315122</v>
       </c>
       <c r="CV8" t="n">
-        <v>0.1109838248173262</v>
+        <v>0.1558474688919975</v>
       </c>
       <c r="CW8" t="n">
         <v>5</v>
@@ -3242,19 +3242,19 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>11.42</v>
+        <v>15.8541</v>
       </c>
       <c r="F9" t="b">
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>6.35</v>
+        <v>14.9648</v>
       </c>
       <c r="H9" t="n">
-        <v>12.92</v>
+        <v>16.2981</v>
       </c>
       <c r="I9" t="n">
-        <v>10.64</v>
+        <v>16.0768</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -3543,7 +3543,7 @@
         <v>68.98348778379983</v>
       </c>
       <c r="CV9" t="n">
-        <v>0.1141765297258671</v>
+        <v>0.1585410652206371</v>
       </c>
       <c r="CW9" t="n">
         <v>4</v>
@@ -3567,19 +3567,19 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>13.91</v>
+        <v>17.954</v>
       </c>
       <c r="F10" s="2" t="b">
         <v>0</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>13.97</v>
+        <v>23.3643</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>12.92</v>
+        <v>16.2981</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>10.64</v>
+        <v>16.0768</v>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
@@ -3868,7 +3868,7 @@
         <v>33.89278521174827</v>
       </c>
       <c r="CV10" s="2" t="n">
-        <v>0.1390661913302826</v>
+        <v>0.1795397804289818</v>
       </c>
       <c r="CW10" s="2" t="n">
         <v>1</v>
@@ -3892,19 +3892,19 @@
         </is>
       </c>
       <c r="E11" s="3" t="n">
-        <v>11.56</v>
+        <v>15.971</v>
       </c>
       <c r="F11" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>7.78</v>
+        <v>16.5411</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>12.92</v>
+        <v>16.2981</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>10.09</v>
+        <v>15.5224</v>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
@@ -4191,7 +4191,7 @@
         <v>40.68215311712356</v>
       </c>
       <c r="CV11" s="3" t="n">
-        <v>0.1155618596551397</v>
+        <v>0.1597098295500497</v>
       </c>
       <c r="CW11" s="3" t="n">
         <v>3</v>
@@ -4215,19 +4215,19 @@
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>12.54</v>
+        <v>16.804</v>
       </c>
       <c r="F12" s="5" t="b">
         <v>0</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>9.800000000000001</v>
+        <v>18.7646</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>12.92</v>
+        <v>16.2981</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>10.64</v>
+        <v>16.0768</v>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
@@ -4516,7 +4516,7 @@
         <v>38.13157336798139</v>
       </c>
       <c r="CV12" s="5" t="n">
-        <v>0.1254361572797913</v>
+        <v>0.1680404998097735</v>
       </c>
       <c r="CW12" s="5" t="n">
         <v>1</v>
@@ -4540,19 +4540,19 @@
         </is>
       </c>
       <c r="E13" s="1" t="n">
-        <v>12.5</v>
+        <v>16.7713</v>
       </c>
       <c r="F13" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G13" s="1" t="n">
-        <v>9.68</v>
+        <v>18.6336</v>
       </c>
       <c r="H13" s="1" t="n">
-        <v>12.92</v>
+        <v>16.2981</v>
       </c>
       <c r="I13" s="1" t="n">
-        <v>10.64</v>
+        <v>16.0768</v>
       </c>
       <c r="J13" s="1" t="inlineStr">
         <is>
@@ -4839,7 +4839,7 @@
         <v>30.45699061463905</v>
       </c>
       <c r="CV13" s="1" t="n">
-        <v>0.1250480299948628</v>
+        <v>0.1677130476149491</v>
       </c>
       <c r="CW13" s="1" t="n">
         <v>2</v>
@@ -4863,19 +4863,19 @@
         </is>
       </c>
       <c r="E14" s="3" t="n">
-        <v>10.71</v>
+        <v>15.2573</v>
       </c>
       <c r="F14" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>4.62</v>
+        <v>13.0596</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>12.37</v>
+        <v>15.8159</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>10.64</v>
+        <v>16.0768</v>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
@@ -5164,7 +5164,7 @@
         <v>35.49477212531589</v>
       </c>
       <c r="CV14" s="3" t="n">
-        <v>0.1071021012249545</v>
+        <v>0.1525725666643487</v>
       </c>
       <c r="CW14" s="3" t="n">
         <v>3</v>
@@ -5188,19 +5188,19 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>10.1</v>
+        <v>14.7454</v>
       </c>
       <c r="F15" t="b">
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>5.36</v>
+        <v>13.8734</v>
       </c>
       <c r="H15" t="n">
-        <v>12.92</v>
+        <v>16.2981</v>
       </c>
       <c r="I15" t="n">
-        <v>8.99</v>
+        <v>14.405</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -5489,7 +5489,7 @@
         <v>30.47009428669543</v>
       </c>
       <c r="CV15" t="n">
-        <v>0.1010347407347857</v>
+        <v>0.1474537033778822</v>
       </c>
       <c r="CW15" t="n">
         <v>4</v>
@@ -5513,19 +5513,19 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>8.960000000000001</v>
+        <v>13.781</v>
       </c>
       <c r="F16" t="b">
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>6.14</v>
+        <v>14.7329</v>
       </c>
       <c r="H16" t="n">
-        <v>9.09</v>
+        <v>12.9644</v>
       </c>
       <c r="I16" t="n">
-        <v>8.31</v>
+        <v>13.7134</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -5814,7 +5814,7 @@
         <v>16.45773528369265</v>
       </c>
       <c r="CV16" t="n">
-        <v>0.08960406842680481</v>
+        <v>0.1378099630872298</v>
       </c>
       <c r="CW16" t="n">
         <v>5</v>
@@ -5838,19 +5838,19 @@
         </is>
       </c>
       <c r="E17" s="6" t="n">
-        <v>8.140000000000001</v>
+        <v>13.092</v>
       </c>
       <c r="F17" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>7.29</v>
+        <v>15.9971</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>6.91</v>
+        <v>11.0653</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>7.26</v>
+        <v>12.65289974212646</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
@@ -6139,7 +6139,7 @@
         <v>46.31123877395689</v>
       </c>
       <c r="CV17" s="6" t="n">
-        <v>0.0814378297606214</v>
+        <v>0.1309203346623846</v>
       </c>
       <c r="CW17" s="6" t="n">
         <v>5</v>
@@ -6163,19 +6163,19 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>15.87</v>
+        <v>19.6082</v>
       </c>
       <c r="F18" s="2" t="b">
         <v>0</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>11.1</v>
+        <v>20.1985</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>14.13</v>
+        <v>17.3435</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>14.96</v>
+        <v>20.44540023803711</v>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
@@ -6464,7 +6464,7 @@
         <v>64.29480699112658</v>
       </c>
       <c r="CV18" s="2" t="n">
-        <v>0.1586738445185035</v>
+        <v>0.1960822120516922</v>
       </c>
       <c r="CW18" s="2" t="n">
         <v>1</v>
@@ -6488,19 +6488,19 @@
         </is>
       </c>
       <c r="E19" s="1" t="n">
-        <v>15.32</v>
+        <v>19.1502</v>
       </c>
       <c r="F19" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G19" s="1" t="n">
-        <v>16.12</v>
+        <v>25.7412</v>
       </c>
       <c r="H19" s="1" t="n">
-        <v>15.04</v>
+        <v>18.1362</v>
       </c>
       <c r="I19" s="1" t="n">
-        <v>10.92</v>
+        <v>16.3617992401123</v>
       </c>
       <c r="J19" s="1" t="inlineStr">
         <is>
@@ -6789,7 +6789,7 @@
         <v>87.27525463894267</v>
       </c>
       <c r="CV19" s="1" t="n">
-        <v>0.1532454146467241</v>
+        <v>0.1915023967565841</v>
       </c>
       <c r="CW19" s="1" t="n">
         <v>2</v>
@@ -6813,19 +6813,19 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4.79</v>
+        <v>10.2652</v>
       </c>
       <c r="F20" t="b">
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>7.28</v>
+        <v>15.9919</v>
       </c>
       <c r="H20" t="n">
-        <v>4.41</v>
+        <v>8.888299999999999</v>
       </c>
       <c r="I20" t="n">
-        <v>2.75</v>
+        <v>8.090299606323242</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -7114,7 +7114,7 @@
         <v>54.01328993905518</v>
       </c>
       <c r="CV20" t="n">
-        <v>0.04793159979826155</v>
+        <v>0.1026520603938392</v>
       </c>
       <c r="CW20" t="n">
         <v>6</v>
@@ -7138,19 +7138,19 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>8.619999999999999</v>
+        <v>13.4929</v>
       </c>
       <c r="F21" t="b">
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>3.48</v>
+        <v>11.8045</v>
       </c>
       <c r="H21" t="n">
-        <v>8.69</v>
+        <v>12.6155</v>
       </c>
       <c r="I21" t="n">
-        <v>9.359999999999999</v>
+        <v>14.77579975128174</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -7439,7 +7439,7 @@
         <v>26.46479136458998</v>
       </c>
       <c r="CV21" t="n">
-        <v>0.08618933392862109</v>
+        <v>0.1349290465693954</v>
       </c>
       <c r="CW21" t="n">
         <v>4</v>
@@ -7463,19 +7463,19 @@
         </is>
       </c>
       <c r="E22" s="3" t="n">
-        <v>13.36</v>
+        <v>17.4905</v>
       </c>
       <c r="F22" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>13.53</v>
+        <v>22.8835</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>13.44</v>
+        <v>16.7494</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>9.74</v>
+        <v>15.16450023651123</v>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
@@ -7764,7 +7764,7 @@
         <v>53.79607804334986</v>
       </c>
       <c r="CV22" s="3" t="n">
-        <v>0.1335725473012733</v>
+        <v>0.1749049457633018</v>
       </c>
       <c r="CW22" s="3" t="n">
         <v>3</v>
@@ -7788,19 +7788,19 @@
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>12.43</v>
+        <v>16.7046</v>
       </c>
       <c r="F23" s="7" t="b">
         <v>0</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>9.869999999999999</v>
+        <v>18.8451</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>12.37</v>
+        <v>15.8199</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>10.64</v>
+        <v>16.0768</v>
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
@@ -8091,7 +8091,7 @@
         <v>86.57372316731569</v>
       </c>
       <c r="CV23" s="7" t="n">
-        <v>0.1242577627519266</v>
+        <v>0.1670463211227755</v>
       </c>
       <c r="CW23" s="7" t="n">
         <v>3</v>
@@ -8115,19 +8115,19 @@
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>14.87</v>
+        <v>18.7678</v>
       </c>
       <c r="F24" s="2" t="b">
         <v>0</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>12.92</v>
+        <v>22.2038</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>18</v>
+        <v>20.714</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>10.64</v>
+        <v>16.0768</v>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
@@ -8416,7 +8416,7 @@
         <v>71.83467085044155</v>
       </c>
       <c r="CV24" s="2" t="n">
-        <v>0.1487126426164271</v>
+        <v>0.1876782230702825</v>
       </c>
       <c r="CW24" s="2" t="n">
         <v>1</v>
@@ -8440,19 +8440,19 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>9.33</v>
+        <v>14.0957</v>
       </c>
       <c r="F25" t="b">
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>6.07</v>
+        <v>14.6595</v>
       </c>
       <c r="H25" t="n">
-        <v>5.19</v>
+        <v>9.569599999999999</v>
       </c>
       <c r="I25" t="n">
-        <v>10.64</v>
+        <v>16.0768</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
@@ -8741,7 +8741,7 @@
         <v>25.95960081773428</v>
       </c>
       <c r="CV25" t="n">
-        <v>0.09333374851245842</v>
+        <v>0.1409565904372369</v>
       </c>
       <c r="CW25" t="n">
         <v>5</v>
@@ -8765,19 +8765,19 @@
         </is>
       </c>
       <c r="E26" s="1" t="n">
-        <v>12.96</v>
+        <v>17.1526</v>
       </c>
       <c r="F26" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G26" s="1" t="n">
-        <v>13.85</v>
+        <v>23.2356</v>
       </c>
       <c r="H26" s="1" t="n">
-        <v>9.390000000000001</v>
+        <v>13.2213</v>
       </c>
       <c r="I26" s="1" t="n">
-        <v>10.64</v>
+        <v>16.0768</v>
       </c>
       <c r="J26" s="1" t="inlineStr">
         <is>
@@ -9066,7 +9066,7 @@
         <v>34.36805861712836</v>
       </c>
       <c r="CV26" s="1" t="n">
-        <v>0.1295676381994014</v>
+        <v>0.1715261153476004</v>
       </c>
       <c r="CW26" s="1" t="n">
         <v>2</v>
@@ -9090,19 +9090,19 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>9.68</v>
+        <v>14.3873</v>
       </c>
       <c r="F27" t="b">
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>6.36</v>
+        <v>14.9791</v>
       </c>
       <c r="H27" t="n">
-        <v>8.73</v>
+        <v>12.6515</v>
       </c>
       <c r="I27" t="n">
-        <v>9.539999999999999</v>
+        <v>14.9593</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -9391,7 +9391,7 @@
         <v>35.31530196492779</v>
       </c>
       <c r="CV27" t="n">
-        <v>0.0967909051470203</v>
+        <v>0.1438732973315936</v>
       </c>
       <c r="CW27" t="n">
         <v>4</v>
@@ -9415,19 +9415,19 @@
         </is>
       </c>
       <c r="E28" s="4" t="n">
-        <v>13.52</v>
+        <v>17.6312</v>
       </c>
       <c r="F28" s="4" t="b">
         <v>0</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>12.8</v>
+        <v>22.073</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>12.92</v>
+        <v>16.2981</v>
       </c>
       <c r="I28" s="4" t="n">
-        <v>10.64</v>
+        <v>16.0768</v>
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
@@ -9716,7 +9716,7 @@
         <v>63.538250004872</v>
       </c>
       <c r="CV28" s="4" t="n">
-        <v>0.1352398210726929</v>
+        <v>0.176311578270277</v>
       </c>
       <c r="CW28" s="4" t="n">
         <v>2</v>
@@ -9740,19 +9740,19 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>10.1</v>
+        <v>14.7406</v>
       </c>
       <c r="F29" t="b">
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>12.66</v>
+        <v>21.9173</v>
       </c>
       <c r="H29" t="n">
-        <v>6.86</v>
+        <v>11.0242</v>
       </c>
       <c r="I29" t="n">
-        <v>7.61</v>
+        <v>13.0104</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -10041,7 +10041,7 @@
         <v>86.10919368570299</v>
       </c>
       <c r="CV29" t="n">
-        <v>0.100978002338154</v>
+        <v>0.14740583477078</v>
       </c>
       <c r="CW29" t="n">
         <v>5</v>
@@ -10065,19 +10065,19 @@
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>15.22</v>
+        <v>19.0651</v>
       </c>
       <c r="F30" s="2" t="b">
         <v>0</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>18</v>
+        <v>27.8088</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>12.92</v>
+        <v>16.2981</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>10.64</v>
+        <v>16.0768</v>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
@@ -10366,7 +10366,7 @@
         <v>45.21805941646117</v>
       </c>
       <c r="CV30" s="2" t="n">
-        <v>0.1522363831589941</v>
+        <v>0.1906511049558416</v>
       </c>
       <c r="CW30" s="2" t="n">
         <v>1</v>
@@ -10390,19 +10390,19 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>11.29</v>
+        <v>15.7459</v>
       </c>
       <c r="F31" t="b">
         <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>5.96</v>
+        <v>14.5321</v>
       </c>
       <c r="H31" t="n">
-        <v>12.92</v>
+        <v>16.2981</v>
       </c>
       <c r="I31" t="n">
-        <v>10.64</v>
+        <v>16.0768</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
@@ -10691,7 +10691,7 @@
         <v>62.56137227099106</v>
       </c>
       <c r="CV31" t="n">
-        <v>0.1128942503575277</v>
+        <v>0.1574592417832096</v>
       </c>
       <c r="CW31" t="n">
         <v>4</v>
@@ -10715,19 +10715,19 @@
         </is>
       </c>
       <c r="E32" s="3" t="n">
-        <v>11.58</v>
+        <v>15.9889</v>
       </c>
       <c r="F32" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>6.84</v>
+        <v>15.504</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>12.92</v>
+        <v>16.2981</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>10.64</v>
+        <v>16.0768</v>
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
@@ -11016,7 +11016,7 @@
         <v>65.68001746010384</v>
       </c>
       <c r="CV32" s="3" t="n">
-        <v>0.1157743554894085</v>
+        <v>0.1598891063750098</v>
       </c>
       <c r="CW32" s="3" t="n">
         <v>3</v>
@@ -11040,19 +11040,19 @@
         </is>
       </c>
       <c r="E33" s="6" t="n">
-        <v>9.210000000000001</v>
+        <v>13.9945</v>
       </c>
       <c r="F33" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G33" s="6" t="n">
-        <v>8.539999999999999</v>
+        <v>17.3746</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>11.65</v>
+        <v>15.1909</v>
       </c>
       <c r="I33" s="6" t="n">
-        <v>6.32</v>
+        <v>11.70619964599609</v>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
@@ -11343,7 +11343,7 @@
         <v>75.88267668374074</v>
       </c>
       <c r="CV33" s="6" t="n">
-        <v>0.09213420295376999</v>
+        <v>0.139944567213833</v>
       </c>
       <c r="CW33" s="6" t="n">
         <v>5</v>
@@ -11367,19 +11367,19 @@
         </is>
       </c>
       <c r="E34" s="3" t="n">
-        <v>16.21</v>
+        <v>19.8979</v>
       </c>
       <c r="F34" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>13.27</v>
+        <v>22.591</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>12.92</v>
+        <v>16.2981</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>14.87</v>
+        <v>20.35129928588867</v>
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
@@ -11668,7 +11668,7 @@
         <v>27.32606853835148</v>
       </c>
       <c r="CV34" s="3" t="n">
-        <v>0.1621073102994076</v>
+        <v>0.1989789316317613</v>
       </c>
       <c r="CW34" s="3" t="n">
         <v>3</v>
@@ -11692,19 +11692,19 @@
         </is>
       </c>
       <c r="E35" s="1" t="n">
-        <v>17.4</v>
+        <v>20.9046</v>
       </c>
       <c r="F35" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G35" s="1" t="n">
-        <v>13.27</v>
+        <v>22.5986</v>
       </c>
       <c r="H35" s="1" t="n">
-        <v>12.92</v>
+        <v>16.2981</v>
       </c>
       <c r="I35" s="1" t="n">
-        <v>16.86</v>
+        <v>22.36090087890625</v>
       </c>
       <c r="J35" s="1" t="inlineStr">
         <is>
@@ -11993,7 +11993,7 @@
         <v>50.37077242720862</v>
       </c>
       <c r="CV35" s="1" t="n">
-        <v>0.1740401909671463</v>
+        <v>0.2090463711469918</v>
       </c>
       <c r="CW35" s="1" t="n">
         <v>2</v>
@@ -12017,19 +12017,19 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>9.34</v>
+        <v>14.0979</v>
       </c>
       <c r="F36" t="b">
         <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>7.23</v>
+        <v>15.9394</v>
       </c>
       <c r="H36" t="n">
-        <v>12.92</v>
+        <v>16.2981</v>
       </c>
       <c r="I36" t="n">
-        <v>6.69</v>
+        <v>12.07699966430664</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
@@ -12318,7 +12318,7 @@
         <v>29.81788831280647</v>
       </c>
       <c r="CV36" t="n">
-        <v>0.09336010903885103</v>
+        <v>0.140978830080156</v>
       </c>
       <c r="CW36" t="n">
         <v>4</v>
@@ -12342,19 +12342,19 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>4</v>
+        <v>9.5938</v>
       </c>
       <c r="F37" t="b">
         <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>4.22</v>
+        <v>12.6165</v>
       </c>
       <c r="H37" t="n">
-        <v>6.86</v>
+        <v>11.0242</v>
       </c>
       <c r="I37" t="n">
-        <v>2.03</v>
+        <v>7.367300033569336</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
@@ -12643,7 +12643,7 @@
         <v>34.74305624093601</v>
       </c>
       <c r="CV37" t="n">
-        <v>0.03997400859598693</v>
+        <v>0.09593846203092088</v>
       </c>
       <c r="CW37" t="n">
         <v>6</v>
@@ -12667,19 +12667,19 @@
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>18</v>
+        <v>21.4074</v>
       </c>
       <c r="F38" s="2" t="b">
         <v>0</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>13</v>
+        <v>22.2938</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>12.92</v>
+        <v>16.2981</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>18</v>
+        <v>23.51889991760254</v>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
@@ -12968,7 +12968,7 @@
         <v>54.25516771030626</v>
       </c>
       <c r="CV38" s="2" t="n">
-        <v>0.18</v>
+        <v>0.2140744962603847</v>
       </c>
       <c r="CW38" s="2" t="n">
         <v>1</v>
@@ -12992,19 +12992,19 @@
         </is>
       </c>
       <c r="E39" s="5" t="n">
-        <v>14.26</v>
+        <v>18.2533</v>
       </c>
       <c r="F39" s="5" t="b">
         <v>0</v>
       </c>
       <c r="G39" s="5" t="n">
-        <v>10.1</v>
+        <v>19.103</v>
       </c>
       <c r="H39" s="5" t="n">
-        <v>12.95</v>
+        <v>16.3174</v>
       </c>
       <c r="I39" s="5" t="n">
-        <v>13.33</v>
+        <v>18.79640007019043</v>
       </c>
       <c r="J39" s="5" t="inlineStr">
         <is>
@@ -13293,7 +13293,7 @@
         <v>80.3037485203028</v>
       </c>
       <c r="CV39" s="5" t="n">
-        <v>0.1426139155211921</v>
+        <v>0.1825328966515603</v>
       </c>
       <c r="CW39" s="5" t="n">
         <v>1</v>
@@ -13317,19 +13317,19 @@
         </is>
       </c>
       <c r="E40" s="3" t="n">
-        <v>12.14</v>
+        <v>16.46</v>
       </c>
       <c r="F40" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>8.51</v>
+        <v>17.3511</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>13.79</v>
+        <v>17.0503</v>
       </c>
       <c r="I40" s="3" t="n">
-        <v>10.29</v>
+        <v>15.71940040588379</v>
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
@@ -13618,7 +13618,7 @@
         <v>56.9581760286313</v>
       </c>
       <c r="CV40" s="3" t="n">
-        <v>0.121358727757675</v>
+        <v>0.1646004859326131</v>
       </c>
       <c r="CW40" s="3" t="n">
         <v>3</v>
@@ -13642,19 +13642,19 @@
         </is>
       </c>
       <c r="E41" s="1" t="n">
-        <v>12.64</v>
+        <v>16.8813</v>
       </c>
       <c r="F41" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G41" s="1" t="n">
-        <v>8.81</v>
+        <v>17.6734</v>
       </c>
       <c r="H41" s="1" t="n">
-        <v>15.78</v>
+        <v>18.781</v>
       </c>
       <c r="I41" s="1" t="n">
-        <v>10.11</v>
+        <v>15.53530025482178</v>
       </c>
       <c r="J41" s="1" t="inlineStr">
         <is>
@@ -13943,7 +13943,7 @@
         <v>23.26155299711137</v>
       </c>
       <c r="CV41" s="1" t="n">
-        <v>0.1263513647643288</v>
+        <v>0.1688126349086669</v>
       </c>
       <c r="CW41" s="1" t="n">
         <v>2</v>
@@ -13967,19 +13967,19 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>7.13</v>
+        <v>12.2357</v>
       </c>
       <c r="F42" t="b">
         <v>0</v>
       </c>
       <c r="G42" t="n">
-        <v>6.21</v>
+        <v>14.8091</v>
       </c>
       <c r="H42" t="n">
-        <v>8.720000000000001</v>
+        <v>12.6408</v>
       </c>
       <c r="I42" t="n">
-        <v>5.37</v>
+        <v>10.74650001525879</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
@@ -14268,7 +14268,7 @@
         <v>38.12510585823195</v>
       </c>
       <c r="CV42" t="n">
-        <v>0.07128783173964839</v>
+        <v>0.1223570636466845</v>
       </c>
       <c r="CW42" t="n">
         <v>6</v>
@@ -14292,19 +14292,19 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>10.88</v>
+        <v>15.3997</v>
       </c>
       <c r="F43" t="b">
         <v>0</v>
       </c>
       <c r="G43" t="n">
-        <v>9.220000000000001</v>
+        <v>18.1319</v>
       </c>
       <c r="H43" t="n">
-        <v>11.82</v>
+        <v>15.3386</v>
       </c>
       <c r="I43" t="n">
-        <v>8.65</v>
+        <v>14.06420040130615</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
@@ -14593,7 +14593,7 @@
         <v>82.18611361379365</v>
       </c>
       <c r="CV43" t="n">
-        <v>0.1087905199298234</v>
+        <v>0.1539970385635446</v>
       </c>
       <c r="CW43" t="n">
         <v>5</v>
@@ -14617,19 +14617,19 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>11.42</v>
+        <v>15.8523</v>
       </c>
       <c r="F44" t="b">
         <v>0</v>
       </c>
       <c r="G44" t="n">
-        <v>6.21</v>
+        <v>14.8107</v>
       </c>
       <c r="H44" t="n">
-        <v>12.68</v>
+        <v>16.087</v>
       </c>
       <c r="I44" t="n">
-        <v>10.82</v>
+        <v>16.25580024719238</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
@@ -14918,7 +14918,7 @@
         <v>22.48239439190696</v>
       </c>
       <c r="CV44" t="n">
-        <v>0.1141555604731149</v>
+        <v>0.1585233740453341</v>
       </c>
       <c r="CW44" t="n">
         <v>4</v>
@@ -14942,19 +14942,19 @@
         </is>
       </c>
       <c r="E45" s="5" t="n">
-        <v>8.98</v>
+        <v>13.7957</v>
       </c>
       <c r="F45" s="5" t="b">
         <v>0</v>
       </c>
       <c r="G45" s="5" t="n">
-        <v>8.77</v>
+        <v>17.6304</v>
       </c>
       <c r="H45" s="5" t="n">
-        <v>8.130000000000001</v>
+        <v>12.131</v>
       </c>
       <c r="I45" s="5" t="n">
-        <v>7.31</v>
+        <v>12.71070003509521</v>
       </c>
       <c r="J45" s="5" t="inlineStr">
         <is>
@@ -15243,7 +15243,7 @@
         <v>30.07851398853546</v>
       </c>
       <c r="CV45" s="5" t="n">
-        <v>0.08977856872212464</v>
+        <v>0.1379571841327961</v>
       </c>
       <c r="CW45" s="5" t="n">
         <v>1</v>
@@ -15267,19 +15267,19 @@
         </is>
       </c>
       <c r="E46" s="1" t="n">
-        <v>5.53</v>
+        <v>10.8839</v>
       </c>
       <c r="F46" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G46" s="1" t="n">
-        <v>3.89</v>
+        <v>12.2505</v>
       </c>
       <c r="H46" s="1" t="n">
-        <v>5.55</v>
+        <v>9.881500000000001</v>
       </c>
       <c r="I46" s="1" t="n">
-        <v>5.33</v>
+        <v>10.70170021057129</v>
       </c>
       <c r="J46" s="1" t="inlineStr">
         <is>
@@ -15568,7 +15568,7 @@
         <v>45.6350105748115</v>
       </c>
       <c r="CV46" s="1" t="n">
-        <v>0.05526448237032087</v>
+        <v>0.1088386094612476</v>
       </c>
       <c r="CW46" s="1" t="n">
         <v>2</v>
@@ -15592,19 +15592,19 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>3.95</v>
+        <v>9.555300000000001</v>
       </c>
       <c r="F47" t="b">
         <v>0</v>
       </c>
       <c r="G47" t="n">
-        <v>3.06</v>
+        <v>11.3395</v>
       </c>
       <c r="H47" t="n">
-        <v>5.92</v>
+        <v>10.2011</v>
       </c>
       <c r="I47" t="n">
-        <v>2.99</v>
+        <v>8.340399742126465</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
@@ -15893,7 +15893,7 @@
         <v>36.82384198012345</v>
       </c>
       <c r="CV47" t="n">
-        <v>0.03951758648531395</v>
+        <v>0.09555339139118534</v>
       </c>
       <c r="CW47" t="n">
         <v>5</v>
@@ -15917,19 +15917,19 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>2</v>
+        <v>7.9087</v>
       </c>
       <c r="F48" t="b">
         <v>0</v>
       </c>
       <c r="G48" t="n">
-        <v>2</v>
+        <v>10.1699</v>
       </c>
       <c r="H48" t="n">
-        <v>2</v>
+        <v>6.7951</v>
       </c>
       <c r="I48" t="n">
-        <v>2</v>
+        <v>7.33489990234375</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
@@ -16218,7 +16218,7 @@
         <v>20.29090792882856</v>
       </c>
       <c r="CV48" t="n">
-        <v>0.02</v>
+        <v>0.07908694654057963</v>
       </c>
       <c r="CW48" t="n">
         <v>6</v>
@@ -16242,19 +16242,19 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>5.01</v>
+        <v>10.4455</v>
       </c>
       <c r="F49" t="b">
         <v>0</v>
       </c>
       <c r="G49" t="n">
-        <v>3.06</v>
+        <v>11.339</v>
       </c>
       <c r="H49" t="n">
-        <v>7.65</v>
+        <v>11.7145</v>
       </c>
       <c r="I49" t="n">
-        <v>4.01</v>
+        <v>9.364399909973145</v>
       </c>
       <c r="J49" t="inlineStr">
         <is>
@@ -16543,7 +16543,7 @@
         <v>22.87258425791754</v>
       </c>
       <c r="CV49" t="n">
-        <v>0.05006908360414854</v>
+        <v>0.1044553960283545</v>
       </c>
       <c r="CW49" t="n">
         <v>4</v>
@@ -16567,19 +16567,19 @@
         </is>
       </c>
       <c r="E50" s="3" t="n">
-        <v>5.27</v>
+        <v>10.6709</v>
       </c>
       <c r="F50" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G50" s="3" t="n">
-        <v>6.88</v>
+        <v>15.5511</v>
       </c>
       <c r="H50" s="3" t="n">
-        <v>6.56</v>
+        <v>10.7612</v>
       </c>
       <c r="I50" s="3" t="n">
-        <v>2.84</v>
+        <v>8.185700416564941</v>
       </c>
       <c r="J50" s="3" t="inlineStr">
         <is>
@@ -16868,7 +16868,7 @@
         <v>43.52254753168122</v>
       </c>
       <c r="CV50" s="3" t="n">
-        <v>0.05274071192659846</v>
+        <v>0.1067093745346642</v>
       </c>
       <c r="CW50" s="3" t="n">
         <v>3</v>
@@ -16892,19 +16892,19 @@
         </is>
       </c>
       <c r="E51" s="5" t="n">
-        <v>16.07</v>
+        <v>20.299</v>
       </c>
       <c r="F51" s="5" t="b">
         <v>0</v>
       </c>
       <c r="G51" s="5" t="n">
-        <v>15.92</v>
+        <v>25.3999</v>
       </c>
       <c r="H51" s="5" t="n">
-        <v>18</v>
+        <v>25.3266</v>
       </c>
       <c r="I51" s="5" t="n">
-        <v>11.62</v>
+        <v>15.2348</v>
       </c>
       <c r="J51" s="5" t="inlineStr">
         <is>
@@ -17191,7 +17191,7 @@
         <v>35.53697669699019</v>
       </c>
       <c r="CV51" s="5" t="n">
-        <v>0.1606895627533124</v>
+        <v>0.2029901795139889</v>
       </c>
       <c r="CW51" s="5" t="n">
         <v>1</v>
@@ -17215,19 +17215,19 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>11.19</v>
+        <v>14.2171</v>
       </c>
       <c r="F52" t="b">
         <v>0</v>
       </c>
       <c r="G52" t="n">
-        <v>9.18</v>
+        <v>14.867</v>
       </c>
       <c r="H52" t="n">
-        <v>8.359999999999999</v>
+        <v>12.4751</v>
       </c>
       <c r="I52" t="n">
-        <v>11.29</v>
+        <v>14.7631</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
@@ -17514,7 +17514,7 @@
         <v>20.37634261311368</v>
       </c>
       <c r="CV52" t="n">
-        <v>0.111875130074499</v>
+        <v>0.1421708191432573</v>
       </c>
       <c r="CW52" t="n">
         <v>4</v>
@@ -17538,19 +17538,19 @@
         </is>
       </c>
       <c r="E53" s="1" t="n">
-        <v>12.49</v>
+        <v>15.8458</v>
       </c>
       <c r="F53" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G53" s="1" t="n">
-        <v>10.28</v>
+        <v>16.5805</v>
       </c>
       <c r="H53" s="1" t="n">
-        <v>11.25</v>
+        <v>16.3333</v>
       </c>
       <c r="I53" s="1" t="n">
-        <v>11.62</v>
+        <v>15.2348</v>
       </c>
       <c r="J53" s="1" t="inlineStr">
         <is>
@@ -17837,7 +17837,7 @@
         <v>26.95190587771532</v>
       </c>
       <c r="CV53" s="1" t="n">
-        <v>0.1249477469668958</v>
+        <v>0.1584583831716778</v>
       </c>
       <c r="CW53" s="1" t="n">
         <v>2</v>
@@ -17861,19 +17861,19 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>9.51</v>
+        <v>12.1307</v>
       </c>
       <c r="F54" t="b">
         <v>0</v>
       </c>
       <c r="G54" t="n">
-        <v>8.539999999999999</v>
+        <v>13.8598</v>
       </c>
       <c r="H54" t="n">
-        <v>7.04</v>
+        <v>10.7153</v>
       </c>
       <c r="I54" t="n">
-        <v>9.34</v>
+        <v>11.9738</v>
       </c>
       <c r="J54" t="inlineStr">
         <is>
@@ -18160,7 +18160,7 @@
         <v>20.19450366483454</v>
       </c>
       <c r="CV54" t="n">
-        <v>0.09512944135130319</v>
+        <v>0.121306865160357</v>
       </c>
       <c r="CW54" t="n">
         <v>5</v>
@@ -18184,19 +18184,19 @@
         </is>
       </c>
       <c r="E55" s="3" t="n">
-        <v>11.39</v>
+        <v>14.4682</v>
       </c>
       <c r="F55" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G55" s="3" t="n">
-        <v>10.75</v>
+        <v>17.3126</v>
       </c>
       <c r="H55" s="3" t="n">
-        <v>6.98</v>
+        <v>10.6359</v>
       </c>
       <c r="I55" s="3" t="n">
-        <v>11.43</v>
+        <v>14.9622</v>
       </c>
       <c r="J55" s="3" t="inlineStr"/>
       <c r="K55" s="3" t="inlineStr">
@@ -18479,7 +18479,7 @@
         <v>13.2500871363948</v>
       </c>
       <c r="CV55" s="3" t="n">
-        <v>0.1138909381637958</v>
+        <v>0.1446823746790525</v>
       </c>
       <c r="CW55" s="3" t="n">
         <v>3</v>
@@ -18503,19 +18503,19 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>9.369999999999999</v>
+        <v>11.9478</v>
       </c>
       <c r="F56" t="b">
         <v>0</v>
       </c>
       <c r="G56" t="n">
-        <v>7.46</v>
+        <v>12.1674</v>
       </c>
       <c r="H56" t="n">
-        <v>3.98</v>
+        <v>6.6428</v>
       </c>
       <c r="I56" t="n">
-        <v>11.1</v>
+        <v>14.4905</v>
       </c>
       <c r="J56" t="inlineStr">
         <is>
@@ -18802,7 +18802,7 @@
         <v>13.85840582616767</v>
       </c>
       <c r="CV56" t="n">
-        <v>0.09366166091721105</v>
+        <v>0.1194781136566055</v>
       </c>
       <c r="CW56" t="n">
         <v>6</v>
@@ -18826,19 +18826,19 @@
         </is>
       </c>
       <c r="E57" s="6" t="n">
-        <v>6.57</v>
+        <v>8.4681</v>
       </c>
       <c r="F57" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G57" s="6" t="n">
-        <v>4.56</v>
+        <v>7.6409</v>
       </c>
       <c r="H57" s="6" t="n">
-        <v>4.96</v>
+        <v>7.945</v>
       </c>
       <c r="I57" s="6" t="n">
-        <v>7.36</v>
+        <v>9.1432</v>
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
@@ -19127,7 +19127,7 @@
         <v>26.92168578402094</v>
       </c>
       <c r="CV57" s="6" t="n">
-        <v>0.0657328280659851</v>
+        <v>0.08468074622453703</v>
       </c>
       <c r="CW57" s="6" t="n">
         <v>8</v>
@@ -19151,19 +19151,19 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>11.31</v>
+        <v>14.3637</v>
       </c>
       <c r="F58" t="b">
         <v>0</v>
       </c>
       <c r="G58" t="n">
-        <v>8.94</v>
+        <v>14.4872</v>
       </c>
       <c r="H58" t="n">
-        <v>9.08</v>
+        <v>13.4412</v>
       </c>
       <c r="I58" t="n">
-        <v>11.29</v>
+        <v>14.7631</v>
       </c>
       <c r="J58" t="inlineStr">
         <is>
@@ -19452,7 +19452,7 @@
         <v>22.20750461827885</v>
       </c>
       <c r="CV58" t="n">
-        <v>0.1130515633081382</v>
+        <v>0.1436365724637883</v>
       </c>
       <c r="CW58" t="n">
         <v>4</v>
@@ -19476,19 +19476,19 @@
         </is>
       </c>
       <c r="E59" s="1" t="n">
-        <v>13.09</v>
+        <v>16.5819</v>
       </c>
       <c r="F59" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G59" s="1" t="n">
-        <v>13.03</v>
+        <v>20.8763</v>
       </c>
       <c r="H59" s="1" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I59" s="1" t="n">
-        <v>11.62</v>
+        <v>15.2348</v>
       </c>
       <c r="J59" s="1" t="inlineStr">
         <is>
@@ -19777,7 +19777,7 @@
         <v>40.76865561318051</v>
       </c>
       <c r="CV59" s="1" t="n">
-        <v>0.130855498145536</v>
+        <v>0.1658190269033887</v>
       </c>
       <c r="CW59" s="1" t="n">
         <v>2</v>
@@ -19801,19 +19801,19 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>10.76</v>
+        <v>13.689</v>
       </c>
       <c r="F60" t="b">
         <v>0</v>
       </c>
       <c r="G60" t="n">
-        <v>5.7</v>
+        <v>9.430099999999999</v>
       </c>
       <c r="H60" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I60" t="n">
-        <v>11.58</v>
+        <v>15.1721</v>
       </c>
       <c r="J60" t="inlineStr">
         <is>
@@ -20102,7 +20102,7 @@
         <v>28.48222792320604</v>
       </c>
       <c r="CV60" t="n">
-        <v>0.1076366007302374</v>
+        <v>0.136889908775483</v>
       </c>
       <c r="CW60" t="n">
         <v>6</v>
@@ -20126,19 +20126,19 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>10.45</v>
+        <v>13.2966</v>
       </c>
       <c r="F61" t="b">
         <v>0</v>
       </c>
       <c r="G61" t="n">
-        <v>5.22</v>
+        <v>8.6783</v>
       </c>
       <c r="H61" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I61" t="n">
-        <v>11.29</v>
+        <v>14.7631</v>
       </c>
       <c r="J61" t="inlineStr">
         <is>
@@ -20427,7 +20427,7 @@
         <v>59.33229979952294</v>
       </c>
       <c r="CV61" t="n">
-        <v>0.104486963036356</v>
+        <v>0.1329656810536979</v>
       </c>
       <c r="CW61" t="n">
         <v>7</v>
@@ -20451,19 +20451,19 @@
         </is>
       </c>
       <c r="E62" s="3" t="n">
-        <v>12.4</v>
+        <v>15.7271</v>
       </c>
       <c r="F62" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G62" s="3" t="n">
-        <v>10.84</v>
+        <v>17.4572</v>
       </c>
       <c r="H62" s="3" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I62" s="3" t="n">
-        <v>11.62</v>
+        <v>15.2348</v>
       </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
@@ -20752,7 +20752,7 @@
         <v>28.33671922732409</v>
       </c>
       <c r="CV62" s="3" t="n">
-        <v>0.1239950530017397</v>
+        <v>0.1572713932916335</v>
       </c>
       <c r="CW62" s="3" t="n">
         <v>3</v>
@@ -20776,19 +20776,19 @@
         </is>
       </c>
       <c r="E63" s="2" t="n">
-        <v>14.64</v>
+        <v>18.5243</v>
       </c>
       <c r="F63" s="2" t="b">
         <v>0</v>
       </c>
       <c r="G63" s="2" t="n">
-        <v>18</v>
+        <v>28.6457</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>11.62</v>
+        <v>15.2348</v>
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
@@ -21077,7 +21077,7 @@
         <v>51.77891737471481</v>
       </c>
       <c r="CV63" s="2" t="n">
-        <v>0.1464450538998176</v>
+        <v>0.185242520272201</v>
       </c>
       <c r="CW63" s="2" t="n">
         <v>1</v>
@@ -21101,19 +21101,19 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>11.07</v>
+        <v>14.0736</v>
       </c>
       <c r="F64" t="b">
         <v>0</v>
       </c>
       <c r="G64" t="n">
-        <v>6.69</v>
+        <v>10.9687</v>
       </c>
       <c r="H64" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I64" t="n">
-        <v>11.58</v>
+        <v>15.1721</v>
       </c>
       <c r="J64" t="inlineStr">
         <is>
@@ -21402,7 +21402,7 @@
         <v>27.90654415353914</v>
       </c>
       <c r="CV64" t="n">
-        <v>0.110723842664261</v>
+        <v>0.1407363957555214</v>
       </c>
       <c r="CW64" t="n">
         <v>5</v>
@@ -21426,19 +21426,19 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>2</v>
+        <v>2.7701</v>
       </c>
       <c r="F65" t="b">
         <v>0</v>
       </c>
       <c r="G65" t="n">
-        <v>2.3</v>
+        <v>4.1089</v>
       </c>
       <c r="H65" t="n">
-        <v>2</v>
+        <v>4.0059</v>
       </c>
       <c r="I65" t="n">
-        <v>2</v>
+        <v>1.4828</v>
       </c>
       <c r="J65" t="inlineStr">
         <is>
@@ -21727,7 +21727,7 @@
         <v>34.47356959119575</v>
       </c>
       <c r="CV65" t="n">
-        <v>0.02</v>
+        <v>0.0277008491269094</v>
       </c>
       <c r="CW65" t="n">
         <v>9</v>
@@ -21751,19 +21751,19 @@
         </is>
       </c>
       <c r="E66" s="6" t="n">
-        <v>8.369999999999999</v>
+        <v>10.7066</v>
       </c>
       <c r="F66" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G66" s="6" t="n">
-        <v>11.16</v>
+        <v>17.9561</v>
       </c>
       <c r="H66" s="6" t="n">
-        <v>5.57</v>
+        <v>8.764699999999999</v>
       </c>
       <c r="I66" s="6" t="n">
-        <v>6.6</v>
+        <v>8.0528</v>
       </c>
       <c r="J66" s="6" t="inlineStr">
         <is>
@@ -22052,7 +22052,7 @@
         <v>44.15057677199813</v>
       </c>
       <c r="CV66" s="6" t="n">
-        <v>0.08369938500866404</v>
+        <v>0.1070658164046587</v>
       </c>
       <c r="CW66" s="6" t="n">
         <v>8</v>
@@ -22076,19 +22076,19 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>11.72</v>
+        <v>14.8831</v>
       </c>
       <c r="F67" t="b">
         <v>0</v>
       </c>
       <c r="G67" t="n">
-        <v>8.68</v>
+        <v>14.0812</v>
       </c>
       <c r="H67" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I67" t="n">
-        <v>11.62</v>
+        <v>15.2348</v>
       </c>
       <c r="J67" t="inlineStr">
         <is>
@@ -22377,7 +22377,7 @@
         <v>32.98110470944309</v>
       </c>
       <c r="CV67" t="n">
-        <v>0.1172208394992819</v>
+        <v>0.1488311982586372</v>
       </c>
       <c r="CW67" t="n">
         <v>5</v>
@@ -22401,19 +22401,19 @@
         </is>
       </c>
       <c r="E68" s="3" t="n">
-        <v>12.32</v>
+        <v>15.6246</v>
       </c>
       <c r="F68" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G68" s="3" t="n">
-        <v>10.58</v>
+        <v>17.0469</v>
       </c>
       <c r="H68" s="3" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I68" s="3" t="n">
-        <v>11.62</v>
+        <v>15.2348</v>
       </c>
       <c r="J68" s="3" t="inlineStr">
         <is>
@@ -22702,7 +22702,7 @@
         <v>21.18032588064538</v>
       </c>
       <c r="CV68" s="3" t="n">
-        <v>0.1231718024636708</v>
+        <v>0.1562456808454876</v>
       </c>
       <c r="CW68" s="3" t="n">
         <v>3</v>
@@ -22726,19 +22726,19 @@
         </is>
       </c>
       <c r="E69" s="1" t="n">
-        <v>12.42</v>
+        <v>15.758</v>
       </c>
       <c r="F69" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G69" s="1" t="n">
-        <v>10.92</v>
+        <v>17.5808</v>
       </c>
       <c r="H69" s="1" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I69" s="1" t="n">
-        <v>11.62</v>
+        <v>15.2348</v>
       </c>
       <c r="J69" s="1" t="inlineStr">
         <is>
@@ -23027,7 +23027,7 @@
         <v>63.12166763346953</v>
       </c>
       <c r="CV69" s="1" t="n">
-        <v>0.1242430460983302</v>
+        <v>0.1575803753013238</v>
       </c>
       <c r="CW69" s="1" t="n">
         <v>2</v>
@@ -23051,19 +23051,19 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>12.21</v>
+        <v>15.4916</v>
       </c>
       <c r="F70" t="b">
         <v>0</v>
       </c>
       <c r="G70" t="n">
-        <v>10.32</v>
+        <v>16.6406</v>
       </c>
       <c r="H70" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I70" t="n">
-        <v>11.58</v>
+        <v>15.1721</v>
       </c>
       <c r="J70" t="inlineStr">
         <is>
@@ -23352,7 +23352,7 @@
         <v>38.80055686046524</v>
       </c>
       <c r="CV70" t="n">
-        <v>0.1221047926044134</v>
+        <v>0.1549162613769405</v>
       </c>
       <c r="CW70" t="n">
         <v>4</v>
@@ -23376,19 +23376,19 @@
         </is>
       </c>
       <c r="E71" s="2" t="n">
-        <v>12.43</v>
+        <v>15.7602</v>
       </c>
       <c r="F71" s="2" t="b">
         <v>0</v>
       </c>
       <c r="G71" s="2" t="n">
-        <v>12.52</v>
+        <v>20.0825</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>8.460000000000001</v>
+        <v>12.614</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>11.58</v>
+        <v>15.1721</v>
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
@@ -23677,7 +23677,7 @@
         <v>31.60264059661428</v>
       </c>
       <c r="CV71" s="2" t="n">
-        <v>0.1242600734309794</v>
+        <v>0.1576015901638904</v>
       </c>
       <c r="CW71" s="2" t="n">
         <v>1</v>
@@ -23701,19 +23701,19 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>11.1</v>
+        <v>14.108</v>
       </c>
       <c r="F72" t="b">
         <v>0</v>
       </c>
       <c r="G72" t="n">
-        <v>6.78</v>
+        <v>11.1062</v>
       </c>
       <c r="H72" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I72" t="n">
-        <v>11.58</v>
+        <v>15.1721</v>
       </c>
       <c r="J72" t="inlineStr">
         <is>
@@ -24002,7 +24002,7 @@
         <v>53.70946451048647</v>
       </c>
       <c r="CV72" t="n">
-        <v>0.1109997146973182</v>
+        <v>0.1410801129652471</v>
       </c>
       <c r="CW72" t="n">
         <v>6</v>
@@ -24026,19 +24026,19 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>9.01</v>
+        <v>11.5027</v>
       </c>
       <c r="F73" t="b">
         <v>0</v>
       </c>
       <c r="G73" t="n">
-        <v>4.46</v>
+        <v>7.4819</v>
       </c>
       <c r="H73" t="n">
-        <v>9.390000000000001</v>
+        <v>13.8497</v>
       </c>
       <c r="I73" t="n">
-        <v>9.6</v>
+        <v>12.3395</v>
       </c>
       <c r="J73" t="inlineStr">
         <is>
@@ -24327,7 +24327,7 @@
         <v>29.06154264337536</v>
       </c>
       <c r="CV73" t="n">
-        <v>0.09008876386284712</v>
+        <v>0.1150265344495568</v>
       </c>
       <c r="CW73" t="n">
         <v>7</v>
@@ -24351,19 +24351,19 @@
         </is>
       </c>
       <c r="E74" s="5" t="n">
-        <v>14.62</v>
+        <v>18.4883</v>
       </c>
       <c r="F74" s="5" t="b">
         <v>0</v>
       </c>
       <c r="G74" s="5" t="n">
-        <v>17.91</v>
+        <v>28.5018</v>
       </c>
       <c r="H74" s="5" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I74" s="5" t="n">
-        <v>11.62</v>
+        <v>15.2348</v>
       </c>
       <c r="J74" s="5" t="inlineStr">
         <is>
@@ -24652,7 +24652,7 @@
         <v>85.8015852009059</v>
       </c>
       <c r="CV74" s="5" t="n">
-        <v>0.1461562568166435</v>
+        <v>0.184882699356302</v>
       </c>
       <c r="CW74" s="5" t="n">
         <v>1</v>
@@ -24676,19 +24676,19 @@
         </is>
       </c>
       <c r="E75" s="3" t="n">
-        <v>12.6</v>
+        <v>15.9733</v>
       </c>
       <c r="F75" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G75" s="3" t="n">
-        <v>11.55</v>
+        <v>18.5712</v>
       </c>
       <c r="H75" s="3" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I75" s="3" t="n">
-        <v>11.58</v>
+        <v>15.1701</v>
       </c>
       <c r="J75" s="3" t="inlineStr">
         <is>
@@ -24975,7 +24975,7 @@
         <v>25.47754324226814</v>
       </c>
       <c r="CV75" s="3" t="n">
-        <v>0.12597087874892</v>
+        <v>0.1597331336326144</v>
       </c>
       <c r="CW75" s="3" t="n">
         <v>3</v>
@@ -24999,19 +24999,19 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>7.23</v>
+        <v>9.286300000000001</v>
       </c>
       <c r="F76" t="b">
         <v>0</v>
       </c>
       <c r="G76" t="n">
-        <v>5.37</v>
+        <v>8.9147</v>
       </c>
       <c r="H76" t="n">
-        <v>6.46</v>
+        <v>9.9442</v>
       </c>
       <c r="I76" t="n">
-        <v>7.36</v>
+        <v>9.1432</v>
       </c>
       <c r="J76" t="inlineStr">
         <is>
@@ -25300,7 +25300,7 @@
         <v>38.43614274873409</v>
       </c>
       <c r="CV76" t="n">
-        <v>0.07230010924647921</v>
+        <v>0.09286311809394834</v>
       </c>
       <c r="CW76" t="n">
         <v>6</v>
@@ -25324,19 +25324,19 @@
         </is>
       </c>
       <c r="E77" s="1" t="n">
-        <v>13.38</v>
+        <v>16.9549</v>
       </c>
       <c r="F77" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G77" s="1" t="n">
-        <v>14.07</v>
+        <v>22.4975</v>
       </c>
       <c r="H77" s="1" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I77" s="1" t="n">
-        <v>11.58</v>
+        <v>15.1701</v>
       </c>
       <c r="J77" s="1" t="inlineStr">
         <is>
@@ -25623,7 +25623,7 @@
         <v>36.03382967907977</v>
       </c>
       <c r="CV77" s="1" t="n">
-        <v>0.1338490735697367</v>
+        <v>0.1695488119798514</v>
       </c>
       <c r="CW77" s="1" t="n">
         <v>2</v>
@@ -25647,19 +25647,19 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>4.28</v>
+        <v>5.6079</v>
       </c>
       <c r="F78" t="b">
         <v>0</v>
       </c>
       <c r="G78" t="n">
-        <v>2.7</v>
+        <v>4.7332</v>
       </c>
       <c r="H78" t="n">
-        <v>3.63</v>
+        <v>6.1745</v>
       </c>
       <c r="I78" t="n">
-        <v>4.99</v>
+        <v>5.762</v>
       </c>
       <c r="J78" t="inlineStr">
         <is>
@@ -25948,7 +25948,7 @@
         <v>24.81903031572897</v>
       </c>
       <c r="CV78" t="n">
-        <v>0.04277681384407453</v>
+        <v>0.0560791621228746</v>
       </c>
       <c r="CW78" t="n">
         <v>8</v>
@@ -25972,19 +25972,19 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>6.65</v>
+        <v>8.5688</v>
       </c>
       <c r="F79" t="b">
         <v>0</v>
       </c>
       <c r="G79" t="n">
-        <v>2.28</v>
+        <v>4.0803</v>
       </c>
       <c r="H79" t="n">
-        <v>7.34</v>
+        <v>11.1267</v>
       </c>
       <c r="I79" t="n">
-        <v>7.64</v>
+        <v>9.5341</v>
       </c>
       <c r="J79" t="inlineStr">
         <is>
@@ -26273,7 +26273,7 @@
         <v>22.87088606731296</v>
       </c>
       <c r="CV79" t="n">
-        <v>0.06654146272515976</v>
+        <v>0.08568824831040994</v>
       </c>
       <c r="CW79" t="n">
         <v>7</v>
@@ -26297,19 +26297,19 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>12.1</v>
+        <v>15.3484</v>
       </c>
       <c r="F80" t="b">
         <v>0</v>
       </c>
       <c r="G80" t="n">
-        <v>9.869999999999999</v>
+        <v>15.9425</v>
       </c>
       <c r="H80" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I80" t="n">
-        <v>11.62</v>
+        <v>15.2348</v>
       </c>
       <c r="J80" t="inlineStr">
         <is>
@@ -26598,7 +26598,7 @@
         <v>22.22177619022168</v>
       </c>
       <c r="CV80" t="n">
-        <v>0.1209556339874651</v>
+        <v>0.1534844903163778</v>
       </c>
       <c r="CW80" t="n">
         <v>4</v>
@@ -26622,19 +26622,19 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>11</v>
+        <v>13.985</v>
       </c>
       <c r="F81" t="b">
         <v>0</v>
       </c>
       <c r="G81" t="n">
-        <v>6.46</v>
+        <v>10.6181</v>
       </c>
       <c r="H81" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I81" t="n">
-        <v>11.58</v>
+        <v>15.1701</v>
       </c>
       <c r="J81" t="inlineStr">
         <is>
@@ -26923,7 +26923,7 @@
         <v>57.61952442577206</v>
       </c>
       <c r="CV81" t="n">
-        <v>0.110012586592348</v>
+        <v>0.1398502205614312</v>
       </c>
       <c r="CW81" t="n">
         <v>5</v>
@@ -26947,19 +26947,19 @@
         </is>
       </c>
       <c r="E82" s="5" t="n">
-        <v>14.13</v>
+        <v>17.8861</v>
       </c>
       <c r="F82" s="5" t="b">
         <v>0</v>
       </c>
       <c r="G82" s="5" t="n">
-        <v>16.14</v>
+        <v>25.7394</v>
       </c>
       <c r="H82" s="5" t="n">
-        <v>10.5</v>
+        <v>15.3353</v>
       </c>
       <c r="I82" s="5" t="n">
-        <v>11.62</v>
+        <v>15.2348</v>
       </c>
       <c r="J82" s="5" t="inlineStr">
         <is>
@@ -27250,7 +27250,7 @@
         <v>53.96801563051854</v>
       </c>
       <c r="CV82" s="5" t="n">
-        <v>0.1413227815094745</v>
+        <v>0.1788605280348818</v>
       </c>
       <c r="CW82" s="5" t="n">
         <v>1</v>
@@ -27274,19 +27274,19 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>10.67</v>
+        <v>13.5667</v>
       </c>
       <c r="F83" t="b">
         <v>0</v>
       </c>
       <c r="G83" t="n">
-        <v>6.9</v>
+        <v>11.2928</v>
       </c>
       <c r="H83" t="n">
-        <v>8.470000000000001</v>
+        <v>12.6297</v>
       </c>
       <c r="I83" t="n">
-        <v>11.58</v>
+        <v>15.1721</v>
       </c>
       <c r="J83" t="inlineStr">
         <is>
@@ -27577,7 +27577,7 @@
         <v>50.07658093812963</v>
       </c>
       <c r="CV83" t="n">
-        <v>0.1066546793715363</v>
+        <v>0.1356665036124341</v>
       </c>
       <c r="CW83" t="n">
         <v>4</v>
@@ -27601,19 +27601,19 @@
         </is>
       </c>
       <c r="E84" s="1" t="n">
-        <v>11.81</v>
+        <v>14.994</v>
       </c>
       <c r="F84" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G84" s="1" t="n">
-        <v>10.56</v>
+        <v>17.0131</v>
       </c>
       <c r="H84" s="1" t="n">
-        <v>8.470000000000001</v>
+        <v>12.6227</v>
       </c>
       <c r="I84" s="1" t="n">
-        <v>11.58</v>
+        <v>15.1701</v>
       </c>
       <c r="J84" s="1" t="inlineStr">
         <is>
@@ -27902,7 +27902,7 @@
         <v>64.77720898919421</v>
       </c>
       <c r="CV84" s="1" t="n">
-        <v>0.1181110315562744</v>
+        <v>0.1499403151435885</v>
       </c>
       <c r="CW84" s="1" t="n">
         <v>2</v>
@@ -27926,19 +27926,19 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>8.76</v>
+        <v>11.1939</v>
       </c>
       <c r="F85" t="b">
         <v>0</v>
       </c>
       <c r="G85" t="n">
-        <v>6.91</v>
+        <v>11.3202</v>
       </c>
       <c r="H85" t="n">
-        <v>5.58</v>
+        <v>8.772600000000001</v>
       </c>
       <c r="I85" t="n">
-        <v>9.6</v>
+        <v>12.3414</v>
       </c>
       <c r="J85" t="inlineStr">
         <is>
@@ -28229,7 +28229,7 @@
         <v>29.51395222324777</v>
       </c>
       <c r="CV85" t="n">
-        <v>0.08761060563044189</v>
+        <v>0.1119389230542949</v>
       </c>
       <c r="CW85" t="n">
         <v>8</v>
@@ -28253,19 +28253,19 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>8.82</v>
+        <v>11.269</v>
       </c>
       <c r="F86" t="b">
         <v>0</v>
       </c>
       <c r="G86" t="n">
-        <v>7.02</v>
+        <v>11.4895</v>
       </c>
       <c r="H86" t="n">
-        <v>6.29</v>
+        <v>9.721500000000001</v>
       </c>
       <c r="I86" t="n">
-        <v>9.31</v>
+        <v>11.9324</v>
       </c>
       <c r="J86" t="inlineStr">
         <is>
@@ -28554,7 +28554,7 @@
         <v>28.57141039010677</v>
       </c>
       <c r="CV86" t="n">
-        <v>0.08821311567074383</v>
+        <v>0.1126896083179999</v>
       </c>
       <c r="CW86" t="n">
         <v>7</v>
@@ -28578,19 +28578,19 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>9.74</v>
+        <v>12.4151</v>
       </c>
       <c r="F87" t="b">
         <v>0</v>
       </c>
       <c r="G87" t="n">
-        <v>7.36</v>
+        <v>12.0107</v>
       </c>
       <c r="H87" t="n">
-        <v>4.89</v>
+        <v>7.8545</v>
       </c>
       <c r="I87" t="n">
-        <v>11.39</v>
+        <v>14.8976</v>
       </c>
       <c r="J87" t="inlineStr">
         <is>
@@ -28881,7 +28881,7 @@
         <v>44.49737182697936</v>
       </c>
       <c r="CV87" t="n">
-        <v>0.09741192330286901</v>
+        <v>0.124150677630029</v>
       </c>
       <c r="CW87" t="n">
         <v>6</v>
@@ -28905,19 +28905,19 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>9.94</v>
+        <v>12.6666</v>
       </c>
       <c r="F88" t="b">
         <v>0</v>
       </c>
       <c r="G88" t="n">
-        <v>7.92</v>
+        <v>12.8943</v>
       </c>
       <c r="H88" t="n">
-        <v>5.18</v>
+        <v>8.245799999999999</v>
       </c>
       <c r="I88" t="n">
-        <v>11.29</v>
+        <v>14.7631</v>
       </c>
       <c r="J88" t="inlineStr">
         <is>
@@ -29206,7 +29206,7 @@
         <v>24.07066316723411</v>
       </c>
       <c r="CV88" t="n">
-        <v>0.09943051305345639</v>
+        <v>0.1266656989207491</v>
       </c>
       <c r="CW88" t="n">
         <v>5</v>
@@ -29230,19 +29230,19 @@
         </is>
       </c>
       <c r="E89" s="3" t="n">
-        <v>11.5</v>
+        <v>14.6056</v>
       </c>
       <c r="F89" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G89" s="3" t="n">
-        <v>8.9</v>
+        <v>14.4295</v>
       </c>
       <c r="H89" s="3" t="n">
-        <v>9.24</v>
+        <v>13.6487</v>
       </c>
       <c r="I89" s="3" t="n">
-        <v>11.58</v>
+        <v>15.1721</v>
       </c>
       <c r="J89" s="3" t="inlineStr">
         <is>
@@ -29531,7 +29531,7 @@
         <v>49.9400151730756</v>
       </c>
       <c r="CV89" s="3" t="n">
-        <v>0.1149933309460629</v>
+        <v>0.1460558787887068</v>
       </c>
       <c r="CW89" s="3" t="n">
         <v>3</v>
@@ -29555,19 +29555,19 @@
         </is>
       </c>
       <c r="E90" s="4" t="n">
-        <v>11.68</v>
+        <v>14.8351</v>
       </c>
       <c r="F90" s="4" t="b">
         <v>0</v>
       </c>
       <c r="G90" s="4" t="n">
-        <v>9.16</v>
+        <v>14.8325</v>
       </c>
       <c r="H90" s="4" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I90" s="4" t="n">
-        <v>11.29</v>
+        <v>14.7631</v>
       </c>
       <c r="J90" s="4" t="inlineStr">
         <is>
@@ -29856,7 +29856,7 @@
         <v>28.3532464944545</v>
       </c>
       <c r="CV90" s="4" t="n">
-        <v>0.1168354740954161</v>
+        <v>0.1483510599862877</v>
       </c>
       <c r="CW90" s="4" t="n">
         <v>2</v>
@@ -29880,19 +29880,19 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>10.08</v>
+        <v>12.8406</v>
       </c>
       <c r="F91" t="b">
         <v>0</v>
       </c>
       <c r="G91" t="n">
-        <v>5.61</v>
+        <v>9.282999999999999</v>
       </c>
       <c r="H91" t="n">
-        <v>8.119999999999999</v>
+        <v>12.1549</v>
       </c>
       <c r="I91" t="n">
-        <v>11.43</v>
+        <v>14.9622</v>
       </c>
       <c r="J91" t="inlineStr">
         <is>
@@ -30181,7 +30181,7 @@
         <v>30.08154658232777</v>
       </c>
       <c r="CV91" t="n">
-        <v>0.1008271316272244</v>
+        <v>0.1284057877362302</v>
       </c>
       <c r="CW91" t="n">
         <v>4</v>
@@ -30205,19 +30205,19 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>9.289999999999999</v>
+        <v>11.8491</v>
       </c>
       <c r="F92" t="b">
         <v>0</v>
       </c>
       <c r="G92" t="n">
-        <v>6.35</v>
+        <v>10.4331</v>
       </c>
       <c r="H92" t="n">
-        <v>8.119999999999999</v>
+        <v>12.1549</v>
       </c>
       <c r="I92" t="n">
-        <v>9.640000000000001</v>
+        <v>12.4041</v>
       </c>
       <c r="J92" t="inlineStr">
         <is>
@@ -30506,7 +30506,7 @@
         <v>18.85890646783279</v>
       </c>
       <c r="CV92" t="n">
-        <v>0.09286910562217343</v>
+        <v>0.1184906453310022</v>
       </c>
       <c r="CW92" t="n">
         <v>5</v>
@@ -30530,19 +30530,19 @@
         </is>
       </c>
       <c r="E93" s="3" t="n">
-        <v>11.44</v>
+        <v>14.5328</v>
       </c>
       <c r="F93" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G93" s="3" t="n">
-        <v>7.78</v>
+        <v>12.6797</v>
       </c>
       <c r="H93" s="3" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I93" s="3" t="n">
-        <v>11.62</v>
+        <v>15.2348</v>
       </c>
       <c r="J93" s="3" t="inlineStr">
         <is>
@@ -30831,7 +30831,7 @@
         <v>27.18101321832401</v>
       </c>
       <c r="CV93" s="3" t="n">
-        <v>0.1144087509620835</v>
+        <v>0.1453275331179686</v>
       </c>
       <c r="CW93" s="3" t="n">
         <v>3</v>
@@ -30855,19 +30855,19 @@
         </is>
       </c>
       <c r="E94" s="2" t="n">
-        <v>13.77</v>
+        <v>17.4331</v>
       </c>
       <c r="F94" s="2" t="b">
         <v>0</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>15.45</v>
+        <v>24.6559</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>10.05</v>
+        <v>14.7325</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>11.58</v>
+        <v>15.1721</v>
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
@@ -31156,7 +31156,7 @@
         <v>64.93266365228394</v>
       </c>
       <c r="CV94" s="2" t="n">
-        <v>0.1376875317416117</v>
+        <v>0.1743312617188313</v>
       </c>
       <c r="CW94" s="2" t="n">
         <v>1</v>
@@ -31180,19 +31180,19 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>7.6</v>
+        <v>9.7418</v>
       </c>
       <c r="F95" t="b">
         <v>0</v>
       </c>
       <c r="G95" t="n">
-        <v>2</v>
+        <v>3.6402</v>
       </c>
       <c r="H95" t="n">
-        <v>7.6</v>
+        <v>11.4619</v>
       </c>
       <c r="I95" t="n">
-        <v>9.31</v>
+        <v>11.9324</v>
       </c>
       <c r="J95" t="inlineStr">
         <is>
@@ -31481,7 +31481,7 @@
         <v>22.67832686238685</v>
       </c>
       <c r="CV95" t="n">
-        <v>0.07595555040667837</v>
+        <v>0.09741754146907958</v>
       </c>
       <c r="CW95" t="n">
         <v>6</v>
@@ -31505,19 +31505,19 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>7.1</v>
+        <v>9.1236</v>
       </c>
       <c r="F96" t="b">
         <v>0</v>
       </c>
       <c r="G96" t="n">
-        <v>4.45</v>
+        <v>7.4632</v>
       </c>
       <c r="H96" t="n">
-        <v>6.29</v>
+        <v>9.7248</v>
       </c>
       <c r="I96" t="n">
-        <v>7.72</v>
+        <v>9.6532</v>
       </c>
       <c r="J96" t="inlineStr">
         <is>
@@ -31806,7 +31806,7 @@
         <v>16.04284401437255</v>
       </c>
       <c r="CV96" t="n">
-        <v>0.07099413751803997</v>
+        <v>0.09123596889181479</v>
       </c>
       <c r="CW96" t="n">
         <v>7</v>
@@ -31830,19 +31830,19 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>6.81</v>
+        <v>8.7576</v>
       </c>
       <c r="F97" t="b">
         <v>0</v>
       </c>
       <c r="G97" t="n">
-        <v>3.67</v>
+        <v>6.2555</v>
       </c>
       <c r="H97" t="n">
-        <v>7.69</v>
+        <v>11.5915</v>
       </c>
       <c r="I97" t="n">
-        <v>6.98</v>
+        <v>8.591699999999999</v>
       </c>
       <c r="J97" t="inlineStr">
         <is>
@@ -32131,7 +32131,7 @@
         <v>30.34931018708762</v>
       </c>
       <c r="CV97" t="n">
-        <v>0.06805660235555747</v>
+        <v>0.08757600605204872</v>
       </c>
       <c r="CW97" t="n">
         <v>8</v>
@@ -32155,19 +32155,19 @@
         </is>
       </c>
       <c r="E98" s="4" t="n">
-        <v>17.8</v>
+        <v>22.4502</v>
       </c>
       <c r="F98" s="4" t="b">
         <v>0</v>
       </c>
       <c r="G98" s="4" t="n">
-        <v>13.34</v>
+        <v>21.3613</v>
       </c>
       <c r="H98" s="4" t="n">
-        <v>13.82</v>
+        <v>19.7527</v>
       </c>
       <c r="I98" s="4" t="n">
-        <v>18</v>
+        <v>24.34339904785156</v>
       </c>
       <c r="J98" s="4" t="inlineStr">
         <is>
@@ -32456,7 +32456,7 @@
         <v>91.61958227166119</v>
       </c>
       <c r="CV98" s="4" t="n">
-        <v>0.1779551445446888</v>
+        <v>0.2245018838062284</v>
       </c>
       <c r="CW98" s="4" t="n">
         <v>2</v>
@@ -32480,19 +32480,19 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>9.51</v>
+        <v>12.1276</v>
       </c>
       <c r="F99" t="b">
         <v>0</v>
       </c>
       <c r="G99" t="n">
-        <v>11.73</v>
+        <v>18.8464</v>
       </c>
       <c r="H99" t="n">
-        <v>5.96</v>
+        <v>9.2807</v>
       </c>
       <c r="I99" t="n">
-        <v>8.1</v>
+        <v>10.19169998168945</v>
       </c>
       <c r="J99" t="inlineStr">
         <is>
@@ -32781,7 +32781,7 @@
         <v>59.34107165923448</v>
       </c>
       <c r="CV99" t="n">
-        <v>0.09510487901085468</v>
+        <v>0.1212762622064086</v>
       </c>
       <c r="CW99" t="n">
         <v>6</v>
@@ -32805,19 +32805,19 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>11.22</v>
+        <v>14.2593</v>
       </c>
       <c r="F100" t="b">
         <v>0</v>
       </c>
       <c r="G100" t="n">
-        <v>11.12</v>
+        <v>17.8923</v>
       </c>
       <c r="H100" t="n">
-        <v>8.82</v>
+        <v>13.0876</v>
       </c>
       <c r="I100" t="n">
-        <v>10.08</v>
+        <v>13.02859973907471</v>
       </c>
       <c r="J100" t="inlineStr">
         <is>
@@ -33106,7 +33106,7 @@
         <v>28.55079792458181</v>
       </c>
       <c r="CV100" t="n">
-        <v>0.1122137824173133</v>
+        <v>0.1425927562169407</v>
       </c>
       <c r="CW100" t="n">
         <v>5</v>
@@ -33130,19 +33130,19 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>13.89</v>
+        <v>17.5863</v>
       </c>
       <c r="F101" t="b">
         <v>0</v>
       </c>
       <c r="G101" t="n">
-        <v>10.2</v>
+        <v>16.4518</v>
       </c>
       <c r="H101" t="n">
-        <v>12.78</v>
+        <v>18.3711</v>
       </c>
       <c r="I101" t="n">
-        <v>13.39</v>
+        <v>17.76110076904297</v>
       </c>
       <c r="J101" t="inlineStr">
         <is>
@@ -33431,7 +33431,7 @@
         <v>92.45537145739141</v>
       </c>
       <c r="CV101" t="n">
-        <v>0.1389169596995703</v>
+        <v>0.1758630427500055</v>
       </c>
       <c r="CW101" t="n">
         <v>4</v>
@@ -33455,19 +33455,19 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>7.79</v>
+        <v>9.9876</v>
       </c>
       <c r="F102" t="b">
         <v>0</v>
       </c>
       <c r="G102" t="n">
-        <v>5.83</v>
+        <v>9.627000000000001</v>
       </c>
       <c r="H102" t="n">
-        <v>6.41</v>
+        <v>9.885300000000001</v>
       </c>
       <c r="I102" t="n">
-        <v>8.109999999999999</v>
+        <v>10.21909999847412</v>
       </c>
       <c r="J102" t="inlineStr">
         <is>
@@ -33756,7 +33756,7 @@
         <v>43.29191348128838</v>
       </c>
       <c r="CV102" t="n">
-        <v>0.07792872445607733</v>
+        <v>0.09987597798055536</v>
       </c>
       <c r="CW102" t="n">
         <v>8</v>
@@ -33780,19 +33780,19 @@
         </is>
       </c>
       <c r="E103" s="3" t="n">
-        <v>14.99</v>
+        <v>18.9538</v>
       </c>
       <c r="F103" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G103" s="3" t="n">
-        <v>14.18</v>
+        <v>22.6785</v>
       </c>
       <c r="H103" s="3" t="n">
-        <v>11.99</v>
+        <v>17.3129</v>
       </c>
       <c r="I103" s="3" t="n">
-        <v>13.5</v>
+        <v>17.91180038452148</v>
       </c>
       <c r="J103" s="3" t="inlineStr">
         <is>
@@ -34081,7 +34081,7 @@
         <v>30.15574520228456</v>
       </c>
       <c r="CV103" s="3" t="n">
-        <v>0.1498924128068796</v>
+        <v>0.1895376877501354</v>
       </c>
       <c r="CW103" s="3" t="n">
         <v>3</v>
@@ -34105,19 +34105,19 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>9.07</v>
+        <v>11.5787</v>
       </c>
       <c r="F104" t="b">
         <v>0</v>
       </c>
       <c r="G104" t="n">
-        <v>6.8</v>
+        <v>11.1473</v>
       </c>
       <c r="H104" t="n">
-        <v>8.5</v>
+        <v>12.6616</v>
       </c>
       <c r="I104" t="n">
-        <v>8.84</v>
+        <v>11.25300025939941</v>
       </c>
       <c r="J104" t="inlineStr">
         <is>
@@ -34406,7 +34406,7 @@
         <v>44.51260000900377</v>
       </c>
       <c r="CV104" t="n">
-        <v>0.09069924969842802</v>
+        <v>0.1157871569949364</v>
       </c>
       <c r="CW104" t="n">
         <v>7</v>
@@ -34430,19 +34430,19 @@
         </is>
       </c>
       <c r="E105" s="2" t="n">
-        <v>18</v>
+        <v>22.705</v>
       </c>
       <c r="F105" s="2" t="b">
         <v>0</v>
       </c>
       <c r="G105" s="2" t="n">
-        <v>16.63</v>
+        <v>26.5046</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>17.09</v>
+        <v>24.1136</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>15.03</v>
+        <v>20.10079956054688</v>
       </c>
       <c r="J105" s="2" t="inlineStr">
         <is>
@@ -34731,7 +34731,7 @@
         <v>112.3742202828741</v>
       </c>
       <c r="CV105" s="2" t="n">
-        <v>0.18</v>
+        <v>0.2270496303233482</v>
       </c>
       <c r="CW105" s="2" t="n">
         <v>1</v>
@@ -34755,19 +34755,19 @@
         </is>
       </c>
       <c r="E106" s="6" t="n">
-        <v>11.48</v>
+        <v>14.582</v>
       </c>
       <c r="F106" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G106" s="6" t="n">
-        <v>11.05</v>
+        <v>17.7814</v>
       </c>
       <c r="H106" s="6" t="n">
-        <v>7.26</v>
+        <v>11.0203</v>
       </c>
       <c r="I106" s="6" t="n">
-        <v>11.29</v>
+        <v>14.7631</v>
       </c>
       <c r="J106" s="6" t="inlineStr">
         <is>
@@ -35054,7 +35054,7 @@
         <v>30.37971239734789</v>
       </c>
       <c r="CV106" s="6" t="n">
-        <v>0.1148037630057862</v>
+        <v>0.1458196904271563</v>
       </c>
       <c r="CW106" s="6" t="n">
         <v>6</v>
@@ -35078,19 +35078,19 @@
         </is>
       </c>
       <c r="E107" s="2" t="n">
-        <v>14.82</v>
+        <v>18.7485</v>
       </c>
       <c r="F107" s="2" t="b">
         <v>0</v>
       </c>
       <c r="G107" s="2" t="n">
-        <v>13.14</v>
+        <v>21.0532</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>16.61</v>
+        <v>23.4713</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>11.62</v>
+        <v>15.2348</v>
       </c>
       <c r="J107" s="2" t="inlineStr">
         <is>
@@ -35379,7 +35379,7 @@
         <v>43.12778647289818</v>
       </c>
       <c r="CV107" s="2" t="n">
-        <v>0.1482450244317615</v>
+        <v>0.1874851573455293</v>
       </c>
       <c r="CW107" s="2" t="n">
         <v>1</v>
@@ -35403,19 +35403,19 @@
         </is>
       </c>
       <c r="E108" s="3" t="n">
-        <v>14.63</v>
+        <v>18.5054</v>
       </c>
       <c r="F108" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G108" s="3" t="n">
-        <v>14.62</v>
+        <v>23.3664</v>
       </c>
       <c r="H108" s="3" t="n">
-        <v>14.14</v>
+        <v>20.1855</v>
       </c>
       <c r="I108" s="3" t="n">
-        <v>11.62</v>
+        <v>15.2348</v>
       </c>
       <c r="J108" s="3" t="inlineStr">
         <is>
@@ -35704,7 +35704,7 @@
         <v>24.21244959699635</v>
       </c>
       <c r="CV108" s="3" t="n">
-        <v>0.1462933805433594</v>
+        <v>0.185053545905014</v>
       </c>
       <c r="CW108" s="3" t="n">
         <v>3</v>
@@ -35728,19 +35728,19 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>13.83</v>
+        <v>17.514</v>
       </c>
       <c r="F109" t="b">
         <v>0</v>
       </c>
       <c r="G109" t="n">
-        <v>14.07</v>
+        <v>22.5102</v>
       </c>
       <c r="H109" t="n">
-        <v>11.81</v>
+        <v>17.0764</v>
       </c>
       <c r="I109" t="n">
-        <v>11.62</v>
+        <v>15.2348</v>
       </c>
       <c r="J109" t="inlineStr">
         <is>
@@ -36029,7 +36029,7 @@
         <v>42.20660116092578</v>
       </c>
       <c r="CV109" t="n">
-        <v>0.1383368596873879</v>
+        <v>0.1751402788100017</v>
       </c>
       <c r="CW109" t="n">
         <v>4</v>
@@ -36053,19 +36053,19 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>11.92</v>
+        <v>15.1358</v>
       </c>
       <c r="F110" t="b">
         <v>0</v>
       </c>
       <c r="G110" t="n">
-        <v>10.86</v>
+        <v>17.4886</v>
       </c>
       <c r="H110" t="n">
-        <v>8.529999999999999</v>
+        <v>12.7103</v>
       </c>
       <c r="I110" t="n">
-        <v>11.58</v>
+        <v>15.1721</v>
       </c>
       <c r="J110" t="inlineStr">
         <is>
@@ -36356,7 +36356,7 @@
         <v>47.34855344121042</v>
       </c>
       <c r="CV110" t="n">
-        <v>0.1192485346300177</v>
+        <v>0.1513575642145756</v>
       </c>
       <c r="CW110" t="n">
         <v>5</v>
@@ -36380,19 +36380,19 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>8.640000000000001</v>
+        <v>11.048</v>
       </c>
       <c r="F111" t="b">
         <v>0</v>
       </c>
       <c r="G111" t="n">
-        <v>4.52</v>
+        <v>7.5807</v>
       </c>
       <c r="H111" t="n">
-        <v>4.72</v>
+        <v>7.6304</v>
       </c>
       <c r="I111" t="n">
-        <v>11.1</v>
+        <v>14.4905</v>
       </c>
       <c r="J111" t="inlineStr">
         <is>
@@ -36683,7 +36683,7 @@
         <v>27.07594089234863</v>
       </c>
       <c r="CV111" t="n">
-        <v>0.08643995202848505</v>
+        <v>0.1104803707495866</v>
       </c>
       <c r="CW111" t="n">
         <v>8</v>
@@ -36707,19 +36707,19 @@
         </is>
       </c>
       <c r="E112" s="1" t="n">
-        <v>14.65</v>
+        <v>18.5282</v>
       </c>
       <c r="F112" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G112" s="1" t="n">
-        <v>17.48</v>
+        <v>27.8385</v>
       </c>
       <c r="H112" s="1" t="n">
-        <v>10.95</v>
+        <v>15.9302</v>
       </c>
       <c r="I112" s="1" t="n">
-        <v>11.58</v>
+        <v>15.1721</v>
       </c>
       <c r="J112" s="1" t="inlineStr">
         <is>
@@ -37008,7 +37008,7 @@
         <v>60.30245636445544</v>
       </c>
       <c r="CV112" s="1" t="n">
-        <v>0.1464767422145831</v>
+        <v>0.1852820016904926</v>
       </c>
       <c r="CW112" s="1" t="n">
         <v>2</v>
@@ -37032,19 +37032,19 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>9.779999999999999</v>
+        <v>12.4677</v>
       </c>
       <c r="F113" t="b">
         <v>0</v>
       </c>
       <c r="G113" t="n">
-        <v>7.59</v>
+        <v>12.3819</v>
       </c>
       <c r="H113" t="n">
-        <v>6.27</v>
+        <v>9.6982</v>
       </c>
       <c r="I113" t="n">
-        <v>10.69</v>
+        <v>13.8954</v>
       </c>
       <c r="J113" t="inlineStr">
         <is>
@@ -37333,7 +37333,7 @@
         <v>32.49249494855098</v>
       </c>
       <c r="CV113" t="n">
-        <v>0.09783443958946111</v>
+        <v>0.1246771032973276</v>
       </c>
       <c r="CW113" t="n">
         <v>7</v>
@@ -37357,19 +37357,19 @@
         </is>
       </c>
       <c r="E114" s="6" t="n">
-        <v>10.56</v>
+        <v>13.4333</v>
       </c>
       <c r="F114" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G114" s="6" t="n">
-        <v>5.73</v>
+        <v>9.474600000000001</v>
       </c>
       <c r="H114" s="6" t="n">
-        <v>10.05</v>
+        <v>14.7325</v>
       </c>
       <c r="I114" s="6" t="n">
-        <v>11.29</v>
+        <v>14.7631</v>
       </c>
       <c r="J114" s="6" t="inlineStr">
         <is>
@@ -37658,7 +37658,7 @@
         <v>26.3508581179673</v>
       </c>
       <c r="CV114" s="6" t="n">
-        <v>0.1055844910087013</v>
+        <v>0.134333123951298</v>
       </c>
       <c r="CW114" s="6" t="n">
         <v>6</v>
@@ -37682,19 +37682,19 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>11.15</v>
+        <v>14.1667</v>
       </c>
       <c r="F115" t="b">
         <v>0</v>
       </c>
       <c r="G115" t="n">
-        <v>6.93</v>
+        <v>11.3447</v>
       </c>
       <c r="H115" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I115" t="n">
-        <v>11.58</v>
+        <v>15.1701</v>
       </c>
       <c r="J115" t="inlineStr">
         <is>
@@ -37983,7 +37983,7 @@
         <v>40.54367880590419</v>
       </c>
       <c r="CV115" t="n">
-        <v>0.1114705197104486</v>
+        <v>0.1416667029999266</v>
       </c>
       <c r="CW115" t="n">
         <v>4</v>
@@ -38007,19 +38007,19 @@
         </is>
       </c>
       <c r="E116" s="2" t="n">
-        <v>12.15</v>
+        <v>15.4208</v>
       </c>
       <c r="F116" s="2" t="b">
         <v>0</v>
       </c>
       <c r="G116" s="2" t="n">
-        <v>10.92</v>
+        <v>17.585</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>9.32</v>
+        <v>13.758</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>11.58</v>
+        <v>15.1701</v>
       </c>
       <c r="J116" s="2" t="inlineStr">
         <is>
@@ -38308,7 +38308,7 @@
         <v>24.04664557708335</v>
       </c>
       <c r="CV116" s="2" t="n">
-        <v>0.1215364409829806</v>
+        <v>0.1542081351080426</v>
       </c>
       <c r="CW116" s="2" t="n">
         <v>1</v>
@@ -38332,19 +38332,19 @@
         </is>
       </c>
       <c r="E117" s="3" t="n">
-        <v>11.84</v>
+        <v>15.0264</v>
       </c>
       <c r="F117" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G117" s="3" t="n">
-        <v>9.130000000000001</v>
+        <v>14.7799</v>
       </c>
       <c r="H117" s="3" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I117" s="3" t="n">
-        <v>11.58</v>
+        <v>15.1721</v>
       </c>
       <c r="J117" s="3" t="inlineStr">
         <is>
@@ -38633,7 +38633,7 @@
         <v>62.87238122348094</v>
       </c>
       <c r="CV117" s="3" t="n">
-        <v>0.1183711655661594</v>
+        <v>0.1502644238799529</v>
       </c>
       <c r="CW117" s="3" t="n">
         <v>3</v>
@@ -38657,19 +38657,19 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>10.67</v>
+        <v>13.5746</v>
       </c>
       <c r="F118" t="b">
         <v>0</v>
       </c>
       <c r="G118" t="n">
-        <v>5.41</v>
+        <v>8.9765</v>
       </c>
       <c r="H118" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I118" t="n">
-        <v>11.58</v>
+        <v>15.1701</v>
       </c>
       <c r="J118" t="inlineStr">
         <is>
@@ -38956,7 +38956,7 @@
         <v>21.64574847573774</v>
       </c>
       <c r="CV118" t="n">
-        <v>0.1067186287996932</v>
+        <v>0.1357461801159422</v>
       </c>
       <c r="CW118" t="n">
         <v>5</v>
@@ -38980,19 +38980,19 @@
         </is>
       </c>
       <c r="E119" s="1" t="n">
-        <v>11.93</v>
+        <v>15.1476</v>
       </c>
       <c r="F119" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G119" s="1" t="n">
-        <v>9.789999999999999</v>
+        <v>15.8136</v>
       </c>
       <c r="H119" s="1" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I119" s="1" t="n">
-        <v>11.39</v>
+        <v>14.8976</v>
       </c>
       <c r="J119" s="1" t="inlineStr">
         <is>
@@ -39281,7 +39281,7 @@
         <v>11.5815264566629</v>
       </c>
       <c r="CV119" s="1" t="n">
-        <v>0.1193437212732578</v>
+        <v>0.1514761600978011</v>
       </c>
       <c r="CW119" s="1" t="n">
         <v>2</v>
@@ -39305,19 +39305,19 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>6.47</v>
+        <v>8.336499999999999</v>
       </c>
       <c r="F120" t="b">
         <v>0</v>
       </c>
       <c r="G120" t="n">
-        <v>3.24</v>
+        <v>5.5813</v>
       </c>
       <c r="H120" t="n">
-        <v>6.11</v>
+        <v>9.4785</v>
       </c>
       <c r="I120" t="n">
-        <v>7.36</v>
+        <v>9.1432</v>
       </c>
       <c r="J120" t="inlineStr">
         <is>
@@ -39606,7 +39606,7 @@
         <v>23.92513236435896</v>
       </c>
       <c r="CV120" t="n">
-        <v>0.06467712609156663</v>
+        <v>0.08336541558761831</v>
       </c>
       <c r="CW120" t="n">
         <v>7</v>
@@ -39630,19 +39630,19 @@
         </is>
       </c>
       <c r="E121" s="7" t="n">
-        <v>11.34</v>
+        <v>14.4046</v>
       </c>
       <c r="F121" s="7" t="b">
         <v>0</v>
       </c>
       <c r="G121" s="7" t="n">
-        <v>11.16</v>
+        <v>17.9578</v>
       </c>
       <c r="H121" s="7" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I121" s="7" t="n">
-        <v>9.6</v>
+        <v>12.3395</v>
       </c>
       <c r="J121" s="7" t="inlineStr">
         <is>
@@ -39931,7 +39931,7 @@
         <v>24.49721249836809</v>
       </c>
       <c r="CV121" s="7" t="n">
-        <v>0.1133803182161693</v>
+        <v>0.1440461780277155</v>
       </c>
       <c r="CW121" s="7" t="n">
         <v>3</v>
@@ -39955,19 +39955,19 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>11.05</v>
+        <v>14.0488</v>
       </c>
       <c r="F122" t="b">
         <v>0</v>
       </c>
       <c r="G122" t="n">
-        <v>10.25</v>
+        <v>16.5308</v>
       </c>
       <c r="H122" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I122" t="n">
-        <v>9.6</v>
+        <v>12.3414</v>
       </c>
       <c r="J122" t="inlineStr">
         <is>
@@ -40256,7 +40256,7 @@
         <v>21.50906655216243</v>
       </c>
       <c r="CV122" t="n">
-        <v>0.1105247524605231</v>
+        <v>0.1404883433213757</v>
       </c>
       <c r="CW122" t="n">
         <v>5</v>
@@ -40280,19 +40280,19 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>9.029999999999999</v>
+        <v>11.5343</v>
       </c>
       <c r="F123" t="b">
         <v>0</v>
       </c>
       <c r="G123" t="n">
-        <v>4.34</v>
+        <v>7.2905</v>
       </c>
       <c r="H123" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I123" t="n">
-        <v>9.31</v>
+        <v>11.9324</v>
       </c>
       <c r="J123" t="inlineStr">
         <is>
@@ -40581,7 +40581,7 @@
         <v>21.19791767548602</v>
       </c>
       <c r="CV123" t="n">
-        <v>0.09034258685754863</v>
+        <v>0.1153427801035154</v>
       </c>
       <c r="CW123" t="n">
         <v>8</v>
@@ -40605,19 +40605,19 @@
         </is>
       </c>
       <c r="E124" s="1" t="n">
-        <v>12.21</v>
+        <v>15.496</v>
       </c>
       <c r="F124" s="1" t="b">
         <v>0</v>
       </c>
       <c r="G124" s="1" t="n">
-        <v>10.6</v>
+        <v>17.0778</v>
       </c>
       <c r="H124" s="1" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I124" s="1" t="n">
-        <v>11.43</v>
+        <v>14.9622</v>
       </c>
       <c r="J124" s="1" t="inlineStr">
         <is>
@@ -40906,7 +40906,7 @@
         <v>18.22201178917614</v>
       </c>
       <c r="CV124" s="1" t="n">
-        <v>0.122139879081418</v>
+        <v>0.1549599766671114</v>
       </c>
       <c r="CW124" s="1" t="n">
         <v>2</v>
@@ -40930,19 +40930,19 @@
         </is>
       </c>
       <c r="E125" s="2" t="n">
-        <v>13.28</v>
+        <v>16.8283</v>
       </c>
       <c r="F125" s="2" t="b">
         <v>0</v>
       </c>
       <c r="G125" s="2" t="n">
-        <v>13.66</v>
+        <v>21.8618</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>11.62</v>
+        <v>15.2348</v>
       </c>
       <c r="J125" s="2" t="inlineStr">
         <is>
@@ -41231,7 +41231,7 @@
         <v>18.72317700674582</v>
       </c>
       <c r="CV125" s="2" t="n">
-        <v>0.1328329378366367</v>
+        <v>0.1682827781053286</v>
       </c>
       <c r="CW125" s="2" t="n">
         <v>1</v>
@@ -41255,19 +41255,19 @@
         </is>
       </c>
       <c r="E126" t="n">
-        <v>9.35</v>
+        <v>11.9285</v>
       </c>
       <c r="F126" t="b">
         <v>0</v>
       </c>
       <c r="G126" t="n">
-        <v>11.65</v>
+        <v>18.7287</v>
       </c>
       <c r="H126" t="n">
-        <v>6.26</v>
+        <v>9.678900000000001</v>
       </c>
       <c r="I126" t="n">
-        <v>7.72</v>
+        <v>9.6532</v>
       </c>
       <c r="J126" t="inlineStr">
         <is>
@@ -41556,7 +41556,7 @@
         <v>12.98002757137192</v>
       </c>
       <c r="CV126" t="n">
-        <v>0.09350685320716766</v>
+        <v>0.1192852341046245</v>
       </c>
       <c r="CW126" t="n">
         <v>7</v>
@@ -41580,19 +41580,19 @@
         </is>
       </c>
       <c r="E127" t="n">
-        <v>11.26</v>
+        <v>14.3053</v>
       </c>
       <c r="F127" t="b">
         <v>0</v>
       </c>
       <c r="G127" t="n">
-        <v>10.82</v>
+        <v>17.431</v>
       </c>
       <c r="H127" t="n">
-        <v>10.24</v>
+        <v>14.9818</v>
       </c>
       <c r="I127" t="n">
-        <v>9.640000000000001</v>
+        <v>12.4041</v>
       </c>
       <c r="J127" t="inlineStr">
         <is>
@@ -41881,7 +41881,7 @@
         <v>51.13650385067046</v>
       </c>
       <c r="CV127" t="n">
-        <v>0.1125828877180351</v>
+        <v>0.143052635540891</v>
       </c>
       <c r="CW127" t="n">
         <v>4</v>
@@ -41905,19 +41905,19 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>10.2</v>
+        <v>12.9822</v>
       </c>
       <c r="F128" t="b">
         <v>0</v>
       </c>
       <c r="G128" t="n">
-        <v>8.890000000000001</v>
+        <v>14.4011</v>
       </c>
       <c r="H128" t="n">
-        <v>8.630000000000001</v>
+        <v>12.8448</v>
       </c>
       <c r="I128" t="n">
-        <v>9.6</v>
+        <v>12.3414</v>
       </c>
       <c r="J128" t="inlineStr">
         <is>
@@ -42206,7 +42206,7 @@
         <v>27.64384684853832</v>
       </c>
       <c r="CV128" t="n">
-        <v>0.1019636707485432</v>
+        <v>0.1298218357900862</v>
       </c>
       <c r="CW128" t="n">
         <v>6</v>
@@ -42230,19 +42230,19 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>8.6</v>
+        <v>10.993</v>
       </c>
       <c r="F129" t="b">
         <v>0</v>
       </c>
       <c r="G129" t="n">
-        <v>8.56</v>
+        <v>13.8924</v>
       </c>
       <c r="H129" t="n">
-        <v>8.119999999999999</v>
+        <v>12.1631</v>
       </c>
       <c r="I129" t="n">
-        <v>7.23</v>
+        <v>8.958299999999999</v>
       </c>
       <c r="J129" t="inlineStr">
         <is>
@@ -42531,7 +42531,7 @@
         <v>28.81866530568137</v>
       </c>
       <c r="CV129" t="n">
-        <v>0.08599834028628116</v>
+        <v>0.1099301534835218</v>
       </c>
       <c r="CW129" t="n">
         <v>9</v>

</xml_diff>